<commit_message>
New feeds process, updating salmon feeds
</commit_message>
<xml_diff>
--- a/data/raw_data/all_ingredients.xlsx
+++ b/data/raw_data/all_ingredients.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\FAO_CC_Risks_to_Fed_Mariculture\data\raw_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F9D82B-8FE7-4C29-8332-ECF3C66F6023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC45CDDA-4947-4CF3-ACD1-5B3569575FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13488" yWindow="0" windowWidth="24144" windowHeight="16656" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="all_ingredients" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="trash fish table" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sources!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="116">
   <si>
     <t>ingredient</t>
   </si>
@@ -381,6 +381,12 @@
   </si>
   <si>
     <t>trash-fish</t>
+  </si>
+  <si>
+    <t>lupin-seed</t>
+  </si>
+  <si>
+    <t>blood-meal</t>
   </si>
 </sst>
 </file>
@@ -983,17 +989,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1344,7 +1340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.21875" bestFit="1" customWidth="1"/>
@@ -1445,7 +1441,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="9">
-        <f t="shared" ref="J2:J47" si="0">SUM(F2:I2)</f>
+        <f t="shared" ref="J2:J49" si="0">SUM(F2:I2)</f>
         <v>1</v>
       </c>
       <c r="K2" s="5">
@@ -1474,11 +1470,11 @@
         <v>0</v>
       </c>
       <c r="R2" s="7">
-        <f t="shared" ref="R2:R11" si="1">Q2*0.95</f>
+        <f t="shared" ref="R2:R12" si="1">Q2*0.95</f>
         <v>0</v>
       </c>
       <c r="S2" s="7">
-        <f t="shared" ref="S2:S11" si="2">R2*1.05</f>
+        <f t="shared" ref="S2:S12" si="2">R2*1.05</f>
         <v>0</v>
       </c>
     </row>
@@ -1716,7 +1712,7 @@
         <v>0.95176181599999998</v>
       </c>
       <c r="O6" s="5">
-        <f>N6*0.95</f>
+        <f t="shared" ref="O6:O11" si="3">N6*0.95</f>
         <v>0.90417372519999994</v>
       </c>
       <c r="P6" s="5">
@@ -1782,7 +1778,7 @@
         <v>0.93</v>
       </c>
       <c r="O7" s="5">
-        <f>N7*0.95</f>
+        <f t="shared" si="3"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P7" s="5">
@@ -1824,7 +1820,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="H8" s="7">
-        <f t="shared" ref="H8:H13" si="3">1-SUM(F8:G8,I8)</f>
+        <f>1-SUM(F8:G8,I8)</f>
         <v>0.22999999999999998</v>
       </c>
       <c r="I8" s="5">
@@ -1849,7 +1845,7 @@
         <v>0.93</v>
       </c>
       <c r="O8" s="5">
-        <f>N8*0.95</f>
+        <f t="shared" si="3"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P8" s="5">
@@ -1891,7 +1887,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="H9" s="7">
-        <f t="shared" si="3"/>
+        <f>1-SUM(F9:G9,I9)</f>
         <v>0.22999999999999998</v>
       </c>
       <c r="I9" s="5">
@@ -1916,7 +1912,7 @@
         <v>0.93</v>
       </c>
       <c r="O9" s="5">
-        <f>N9*0.95</f>
+        <f t="shared" si="3"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P9" s="5">
@@ -1937,13 +1933,13 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
         <v>73</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D10" t="s">
         <v>69</v>
@@ -1951,128 +1947,129 @@
       <c r="E10" t="s">
         <v>69</v>
       </c>
-      <c r="F10">
-        <v>0.3</v>
-      </c>
-      <c r="G10">
-        <v>0.02</v>
-      </c>
-      <c r="H10" s="7">
-        <f t="shared" si="3"/>
-        <v>0.64</v>
-      </c>
-      <c r="I10">
+      <c r="F10" s="11">
+        <v>0.84</v>
+      </c>
+      <c r="G10" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="H10" s="11">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I10" s="11">
         <v>0.04</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="12">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K10">
-        <v>0.86</v>
-      </c>
-      <c r="L10" s="4">
-        <f>K10*0.95</f>
-        <v>0.81699999999999995</v>
-      </c>
-      <c r="M10" s="4">
-        <f>L10*1.05</f>
-        <v>0.85785</v>
-      </c>
-      <c r="N10">
-        <v>0.93</v>
-      </c>
-      <c r="O10">
-        <f>N10*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P10">
-        <f>MIN(N10*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q10">
-        <v>0.6</v>
-      </c>
-      <c r="R10" s="4">
+      <c r="K10" s="11">
+        <v>0.88</v>
+      </c>
+      <c r="L10" s="11">
+        <f>K10*0.94</f>
+        <v>0.82719999999999994</v>
+      </c>
+      <c r="M10" s="11">
+        <f>L10*1.06</f>
+        <v>0.87683199999999994</v>
+      </c>
+      <c r="N10" s="11">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O10" s="11">
+        <f t="shared" si="3"/>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P10" s="11">
+        <f>N10*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q10" s="11">
+        <v>0.77</v>
+      </c>
+      <c r="R10" s="11">
         <f t="shared" si="1"/>
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="S10" s="4">
+        <v>0.73149999999999993</v>
+      </c>
+      <c r="S10" s="11">
         <f t="shared" si="2"/>
-        <v>0.59849999999999992</v>
+        <v>0.76807499999999995</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0.86849038461538397</v>
-      </c>
-      <c r="G11" s="6">
-        <f>6.7799419/100</f>
-        <v>6.7799419E-2</v>
+        <v>69</v>
+      </c>
+      <c r="F11">
+        <v>0.3</v>
+      </c>
+      <c r="G11">
+        <v>0.02</v>
       </c>
       <c r="H11" s="7">
-        <f t="shared" si="3"/>
-        <v>1.3710196384616014E-2</v>
-      </c>
-      <c r="I11" s="5">
-        <f>5/100</f>
-        <v>0.05</v>
+        <f>1-SUM(F11:G11,I11)</f>
+        <v>0.64</v>
+      </c>
+      <c r="I11">
+        <v>0.04</v>
       </c>
       <c r="J11" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K11" s="6">
-        <v>0.86599999999999999</v>
-      </c>
-      <c r="L11" s="6">
-        <v>0.75829999999999997</v>
-      </c>
-      <c r="M11" s="6">
-        <v>0.94739999999999991</v>
-      </c>
-      <c r="N11" s="6">
-        <v>0.93709999999999993</v>
-      </c>
-      <c r="O11" s="6">
-        <v>0.87280000000000002</v>
-      </c>
-      <c r="P11" s="6">
-        <v>0.97950000000000004</v>
-      </c>
-      <c r="Q11" s="5">
-        <v>0.78</v>
-      </c>
-      <c r="R11" s="7">
+      <c r="K11">
+        <v>0.86</v>
+      </c>
+      <c r="L11" s="4">
+        <f>K11*0.95</f>
+        <v>0.81699999999999995</v>
+      </c>
+      <c r="M11" s="4">
+        <f>L11*1.05</f>
+        <v>0.85785</v>
+      </c>
+      <c r="N11">
+        <v>0.93</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="3"/>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P11">
+        <f>MIN(N11*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q11">
+        <v>0.6</v>
+      </c>
+      <c r="R11" s="4">
         <f t="shared" si="1"/>
-        <v>0.74099999999999999</v>
-      </c>
-      <c r="S11" s="7">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="S11" s="4">
         <f t="shared" si="2"/>
-        <v>0.77805000000000002</v>
+        <v>0.59849999999999992</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
         <v>68</v>
@@ -2084,57 +2081,57 @@
         <v>68</v>
       </c>
       <c r="F12" s="6">
-        <v>0.73424999999999996</v>
+        <v>0.86849038461538397</v>
       </c>
       <c r="G12" s="6">
-        <v>8.3000000000000004E-2</v>
+        <f>6.7799419/100</f>
+        <v>6.7799419E-2</v>
       </c>
       <c r="H12" s="7">
-        <f t="shared" si="3"/>
-        <v>4.3750000000000067E-2</v>
+        <f>1-SUM(F12:G12,I12)</f>
+        <v>1.3710196384616014E-2</v>
       </c>
       <c r="I12" s="5">
-        <f>13.9/100</f>
-        <v>0.13900000000000001</v>
+        <f>5/100</f>
+        <v>0.05</v>
       </c>
       <c r="J12" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K12" s="6">
-        <v>0.87980000000000003</v>
+        <v>0.86599999999999999</v>
       </c>
       <c r="L12" s="6">
-        <v>0.82969999999999999</v>
+        <v>0.75829999999999997</v>
       </c>
       <c r="M12" s="6">
-        <v>0.92209999999999992</v>
+        <v>0.94739999999999991</v>
       </c>
       <c r="N12" s="6">
-        <v>0.95669999999999999</v>
+        <v>0.93709999999999993</v>
       </c>
       <c r="O12" s="6">
-        <v>0.8993000000000001</v>
+        <v>0.87280000000000002</v>
       </c>
       <c r="P12" s="6">
-        <v>0.99199999999999999</v>
+        <v>0.97950000000000004</v>
       </c>
       <c r="Q12" s="5">
-        <f>83.3/100</f>
-        <v>0.83299999999999996</v>
-      </c>
-      <c r="R12" s="5">
-        <f>74.5/100</f>
-        <v>0.745</v>
-      </c>
-      <c r="S12" s="5">
-        <f>92.6/100</f>
-        <v>0.92599999999999993</v>
+        <v>0.78</v>
+      </c>
+      <c r="R12" s="7">
+        <f t="shared" si="1"/>
+        <v>0.74099999999999999</v>
+      </c>
+      <c r="S12" s="7">
+        <f t="shared" si="2"/>
+        <v>0.77805000000000002</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
         <v>74</v>
@@ -2155,7 +2152,7 @@
         <v>8.3000000000000004E-2</v>
       </c>
       <c r="H13" s="7">
-        <f t="shared" si="3"/>
+        <f>1-SUM(F13:G13,I13)</f>
         <v>4.3750000000000067E-2</v>
       </c>
       <c r="I13" s="5">
@@ -2185,21 +2182,21 @@
         <v>0.99199999999999999</v>
       </c>
       <c r="Q13" s="5">
-        <f>81.7/100</f>
-        <v>0.81700000000000006</v>
+        <f>83.3/100</f>
+        <v>0.83299999999999996</v>
       </c>
       <c r="R13" s="5">
-        <f>71.8/100</f>
-        <v>0.71799999999999997</v>
+        <f>74.5/100</f>
+        <v>0.745</v>
       </c>
       <c r="S13" s="5">
-        <f>91.6/100</f>
-        <v>0.91599999999999993</v>
+        <f>92.6/100</f>
+        <v>0.92599999999999993</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
         <v>74</v>
@@ -2211,34 +2208,34 @@
         <v>68</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="5">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>1</v>
-      </c>
-      <c r="H14" s="5">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0.73424999999999996</v>
+      </c>
+      <c r="G14" s="6">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="H14" s="7">
+        <f>1-SUM(F14:G14,I14)</f>
+        <v>4.3750000000000067E-2</v>
       </c>
       <c r="I14" s="5">
-        <v>0</v>
+        <f>13.9/100</f>
+        <v>0.13900000000000001</v>
       </c>
       <c r="J14" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K14" s="5">
-        <v>0</v>
-      </c>
-      <c r="L14" s="5">
-        <f>K14*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="5">
-        <f>L14*1.05</f>
-        <v>0</v>
+      <c r="K14" s="6">
+        <v>0.87980000000000003</v>
+      </c>
+      <c r="L14" s="6">
+        <v>0.82969999999999999</v>
+      </c>
+      <c r="M14" s="6">
+        <v>0.92209999999999992</v>
       </c>
       <c r="N14" s="6">
         <v>0.95669999999999999</v>
@@ -2250,20 +2247,21 @@
         <v>0.99199999999999999</v>
       </c>
       <c r="Q14" s="5">
-        <v>0</v>
-      </c>
-      <c r="R14" s="7">
-        <f>Q14*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="S14" s="7">
-        <f>R14*1.05</f>
-        <v>0</v>
+        <f>81.7/100</f>
+        <v>0.81700000000000006</v>
+      </c>
+      <c r="R14" s="5">
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="S14" s="5">
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
@@ -2327,16 +2325,16 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
         <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
         <v>69</v>
@@ -2345,13 +2343,13 @@
         <v>0</v>
       </c>
       <c r="G16" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="5">
         <v>0</v>
       </c>
       <c r="I16" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" s="9">
         <f t="shared" si="0"/>
@@ -2361,33 +2359,37 @@
         <v>0</v>
       </c>
       <c r="L16" s="5">
+        <f>K16*0.95</f>
         <v>0</v>
       </c>
       <c r="M16" s="5">
+        <f>L16*1.05</f>
         <v>0</v>
       </c>
-      <c r="N16" s="5">
-        <v>0</v>
-      </c>
-      <c r="O16" s="5">
-        <v>0</v>
-      </c>
-      <c r="P16" s="5">
-        <v>0</v>
+      <c r="N16" s="6">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O16" s="6">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P16" s="6">
+        <v>0.99199999999999999</v>
       </c>
       <c r="Q16" s="5">
         <v>0</v>
       </c>
-      <c r="R16" s="5">
+      <c r="R16" s="7">
+        <f>Q16*0.95</f>
         <v>0</v>
       </c>
-      <c r="S16" s="5">
+      <c r="S16" s="7">
+        <f>R16*1.05</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
         <v>73</v>
@@ -2396,263 +2398,260 @@
         <v>68</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E17" t="s">
         <v>69</v>
       </c>
       <c r="F17" s="5">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="G17" s="5">
-        <v>5.2999999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="H17" s="5">
-        <v>0.46899999999999997</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5">
-        <v>5.8000000000000003E-2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K17" s="5">
-        <v>0.63000000000000012</v>
-      </c>
-      <c r="L17" s="10">
-        <f>K17*0.95</f>
-        <v>0.59850000000000003</v>
-      </c>
-      <c r="M17" s="10">
-        <f>L17*1.05</f>
-        <v>0.62842500000000001</v>
+        <v>0</v>
+      </c>
+      <c r="L17" s="5">
+        <v>0</v>
+      </c>
+      <c r="M17" s="5">
+        <v>0</v>
       </c>
       <c r="N17" s="5">
-        <v>0.95176181599999998</v>
+        <v>0</v>
       </c>
       <c r="O17" s="5">
-        <f>N17*0.95</f>
-        <v>0.90417372519999994</v>
+        <v>0</v>
       </c>
       <c r="P17" s="5">
-        <f>N17*1.05</f>
-        <v>0.99934990680000002</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="5">
-        <v>0.71</v>
-      </c>
-      <c r="R17" s="7">
-        <f>Q17*0.95</f>
-        <v>0.67449999999999999</v>
-      </c>
-      <c r="S17" s="7">
-        <f>R17*1.05</f>
-        <v>0.70822499999999999</v>
+        <v>0</v>
+      </c>
+      <c r="R17" s="5">
+        <v>0</v>
+      </c>
+      <c r="S17" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
         <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
         <v>69</v>
       </c>
-      <c r="F18">
-        <v>0.55800000000000005</v>
-      </c>
-      <c r="G18">
-        <v>4.7E-2</v>
-      </c>
-      <c r="H18">
-        <v>0.34100000000000003</v>
-      </c>
-      <c r="I18">
-        <v>5.3999999999999999E-2</v>
+      <c r="F18" s="5">
+        <v>0.42</v>
+      </c>
+      <c r="G18" s="5">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="H18" s="5">
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="I18" s="5">
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="J18" s="9">
         <f t="shared" si="0"/>
-        <v>1.0000000000000002</v>
-      </c>
-      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="K18" s="5">
         <v>0.63000000000000012</v>
       </c>
-      <c r="L18" s="4">
+      <c r="L18" s="10">
         <f>K18*0.95</f>
         <v>0.59850000000000003</v>
       </c>
-      <c r="M18" s="4">
+      <c r="M18" s="10">
         <f>L18*1.05</f>
         <v>0.62842500000000001</v>
       </c>
-      <c r="N18">
-        <v>0.93</v>
-      </c>
-      <c r="O18">
+      <c r="N18" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O18" s="5">
         <f>N18*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P18">
-        <f>MIN(N18*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q18">
-        <v>0.65000000000000013</v>
-      </c>
-      <c r="R18" s="4">
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P18" s="5">
+        <f>N18*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q18" s="5">
+        <v>0.71</v>
+      </c>
+      <c r="R18" s="7">
         <f>Q18*0.95</f>
-        <v>0.61750000000000005</v>
-      </c>
-      <c r="S18" s="4">
+        <v>0.67449999999999999</v>
+      </c>
+      <c r="S18" s="7">
         <f>R18*1.05</f>
-        <v>0.64837500000000003</v>
+        <v>0.70822499999999999</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E19" t="s">
         <v>69</v>
       </c>
-      <c r="F19" s="5">
-        <v>0.93</v>
-      </c>
-      <c r="G19" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H19" s="7">
-        <f>1-SUM(F19:G19,I19)</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="5">
-        <v>0</v>
+      <c r="F19">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="G19">
+        <v>4.7E-2</v>
+      </c>
+      <c r="H19">
+        <v>0.34100000000000003</v>
+      </c>
+      <c r="I19">
+        <v>5.3999999999999999E-2</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="K19" s="5">
-        <v>0.622</v>
-      </c>
-      <c r="L19" s="10">
-        <f>K19*0.94</f>
-        <v>0.58467999999999998</v>
-      </c>
-      <c r="M19" s="10">
-        <f>L19*1.06</f>
-        <v>0.6197608</v>
-      </c>
-      <c r="N19" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O19" s="5">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="K19">
+        <v>0.63000000000000012</v>
+      </c>
+      <c r="L19" s="4">
+        <f>K19*0.95</f>
+        <v>0.59850000000000003</v>
+      </c>
+      <c r="M19" s="4">
+        <f>L19*1.05</f>
+        <v>0.62842500000000001</v>
+      </c>
+      <c r="N19">
+        <v>0.93</v>
+      </c>
+      <c r="O19">
         <f>N19*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P19" s="5">
-        <f>N19*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q19" s="5">
-        <v>0.60399999999999998</v>
-      </c>
-      <c r="R19" s="7">
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P19">
+        <f>MIN(N19*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q19">
+        <v>0.65000000000000013</v>
+      </c>
+      <c r="R19" s="4">
         <f>Q19*0.95</f>
-        <v>0.57379999999999998</v>
-      </c>
-      <c r="S19" s="7">
+        <v>0.61750000000000005</v>
+      </c>
+      <c r="S19" s="4">
         <f>R19*1.05</f>
-        <v>0.60248999999999997</v>
+        <v>0.64837500000000003</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" t="s">
         <v>69</v>
       </c>
-      <c r="D20" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" t="s">
-        <v>68</v>
-      </c>
-      <c r="F20" s="6">
-        <v>0.58399999999999996</v>
-      </c>
-      <c r="G20" s="6">
-        <v>0.17899999999999999</v>
+      <c r="F20" s="5">
+        <v>0.93</v>
+      </c>
+      <c r="G20" s="5">
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H20" s="7">
         <f>1-SUM(F20:G20,I20)</f>
-        <v>0.1070000000000001</v>
+        <v>0</v>
       </c>
       <c r="I20" s="5">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="J20" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J20" si="4">SUM(F20:I20)</f>
         <v>1</v>
       </c>
-      <c r="K20" s="6">
-        <v>0.88470000000000004</v>
-      </c>
-      <c r="L20" s="6">
-        <v>0.84920000000000007</v>
-      </c>
-      <c r="M20" s="6">
-        <v>0.93629999999999991</v>
-      </c>
-      <c r="N20" s="6">
-        <v>0.9466</v>
-      </c>
-      <c r="O20" s="6">
-        <v>0.91510000000000002</v>
-      </c>
-      <c r="P20" s="6">
-        <v>0.97360000000000002</v>
+      <c r="K20" s="5">
+        <v>0.622</v>
+      </c>
+      <c r="L20" s="10">
+        <f>K20*0.94</f>
+        <v>0.58467999999999998</v>
+      </c>
+      <c r="M20" s="10">
+        <f>L20*1.06</f>
+        <v>0.6197608</v>
+      </c>
+      <c r="N20" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O20" s="5">
+        <f>N20*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P20" s="5">
+        <f>N20*1.05</f>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q20" s="5">
-        <v>0.41000000000000003</v>
+        <v>0.60399999999999998</v>
       </c>
       <c r="R20" s="7">
         <f>Q20*0.95</f>
-        <v>0.38950000000000001</v>
+        <v>0.57379999999999998</v>
       </c>
       <c r="S20" s="7">
         <f>R20*1.05</f>
-        <v>0.40897500000000003</v>
+        <v>0.60248999999999997</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
         <v>68</v>
@@ -2661,63 +2660,65 @@
         <v>68</v>
       </c>
       <c r="E21" t="s">
-        <v>68</v>
-      </c>
-      <c r="F21" s="6">
-        <v>0.55099999999999993</v>
-      </c>
-      <c r="G21" s="6">
-        <f>26.92252/100</f>
-        <v>0.2692252</v>
+        <v>69</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0.93</v>
+      </c>
+      <c r="G21" s="5">
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H21" s="7">
         <f>1-SUM(F21:G21,I21)</f>
-        <v>4.08748000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="I21" s="5">
-        <f>13.89/100</f>
-        <v>0.1389</v>
+        <v>0</v>
       </c>
       <c r="J21" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K21" s="6">
-        <v>0.87769999999999992</v>
-      </c>
-      <c r="L21" s="6">
-        <v>0.86930000000000007</v>
-      </c>
-      <c r="M21" s="6">
-        <v>0.88549999999999995</v>
-      </c>
-      <c r="N21" s="6">
-        <v>0.95109999999999995</v>
-      </c>
-      <c r="O21" s="6">
-        <v>0.93889999999999996</v>
-      </c>
-      <c r="P21" s="6">
-        <v>0.95739999999999992</v>
+      <c r="K21" s="5">
+        <v>0.622</v>
+      </c>
+      <c r="L21" s="10">
+        <f>K21*0.94</f>
+        <v>0.58467999999999998</v>
+      </c>
+      <c r="M21" s="10">
+        <f>L21*1.06</f>
+        <v>0.6197608</v>
+      </c>
+      <c r="N21" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O21" s="5">
+        <f>N21*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P21" s="5">
+        <f>N21*1.05</f>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q21" s="5">
-        <v>0.59399999999999997</v>
-      </c>
-      <c r="R21" s="5">
-        <f>Q21-3*(2.16/100)</f>
-        <v>0.5292</v>
-      </c>
-      <c r="S21" s="5">
-        <f>Q21+3*(2.16/100)</f>
-        <v>0.65879999999999994</v>
+        <v>0.60399999999999998</v>
+      </c>
+      <c r="R21" s="7">
+        <f>Q21*0.95</f>
+        <v>0.57379999999999998</v>
+      </c>
+      <c r="S21" s="7">
+        <f>R21*1.05</f>
+        <v>0.60248999999999997</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C22" t="s">
         <v>69</v>
@@ -2726,64 +2727,61 @@
         <v>69</v>
       </c>
       <c r="E22" t="s">
-        <v>69</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22">
-        <v>1</v>
-      </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
-      <c r="I22">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F22" s="6">
+        <v>0.58399999999999996</v>
+      </c>
+      <c r="G22" s="6">
+        <v>0.17899999999999999</v>
+      </c>
+      <c r="H22" s="7">
+        <f>1-SUM(F22:G22,I22)</f>
+        <v>0.1070000000000001</v>
+      </c>
+      <c r="I22" s="5">
+        <v>0.13</v>
       </c>
       <c r="J22" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K22" s="4">
-        <v>0.84588505065844988</v>
-      </c>
-      <c r="L22" s="4">
-        <f>K22*0.95</f>
-        <v>0.80359079812552736</v>
-      </c>
-      <c r="M22" s="4">
-        <f>L22*1.05</f>
-        <v>0.84377033803180379</v>
-      </c>
-      <c r="N22">
-        <v>0.93</v>
-      </c>
-      <c r="O22">
-        <f>N22*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P22">
-        <f>MIN(N22*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q22" s="4">
-        <v>0.71148214285714262</v>
-      </c>
-      <c r="R22" s="4">
+      <c r="K22" s="6">
+        <v>0.88470000000000004</v>
+      </c>
+      <c r="L22" s="6">
+        <v>0.84920000000000007</v>
+      </c>
+      <c r="M22" s="6">
+        <v>0.93629999999999991</v>
+      </c>
+      <c r="N22" s="6">
+        <v>0.9466</v>
+      </c>
+      <c r="O22" s="6">
+        <v>0.91510000000000002</v>
+      </c>
+      <c r="P22" s="6">
+        <v>0.97360000000000002</v>
+      </c>
+      <c r="Q22" s="5">
+        <v>0.41000000000000003</v>
+      </c>
+      <c r="R22" s="7">
         <f>Q22*0.95</f>
-        <v>0.67590803571428548</v>
-      </c>
-      <c r="S22" s="4">
+        <v>0.38950000000000001</v>
+      </c>
+      <c r="S22" s="7">
         <f>R22*1.05</f>
-        <v>0.70970343749999976</v>
+        <v>0.40897500000000003</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C23" t="s">
         <v>68</v>
@@ -2792,194 +2790,201 @@
         <v>68</v>
       </c>
       <c r="E23" t="s">
-        <v>69</v>
-      </c>
-      <c r="F23" s="5">
-        <f>AVERAGE(420.2,405.3,420.2,403.8,390.7,468.4)/1000</f>
-        <v>0.41809999999999997</v>
-      </c>
-      <c r="G23" s="5">
-        <f>AVERAGE(175.4,153.9,171.8,132.3,106.7,100.1)/1000</f>
-        <v>0.14003333333333337</v>
+        <v>68</v>
+      </c>
+      <c r="F23" s="6">
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="G23" s="6">
+        <f>26.92252/100</f>
+        <v>0.2692252</v>
       </c>
       <c r="H23" s="7">
         <f>1-SUM(F23:G23,I23)</f>
-        <v>0.41068333333333329</v>
+        <v>4.08748000000001E-2</v>
       </c>
       <c r="I23" s="5">
-        <f>AVERAGE(28.6,37.6,28,37.3,25.9,29.7)/1000</f>
-        <v>3.1183333333333334E-2</v>
+        <f>13.89/100</f>
+        <v>0.1389</v>
       </c>
       <c r="J23" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K23" s="5">
-        <f>AVERAGE(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
-        <v>0.89050000000000007</v>
-      </c>
-      <c r="L23" s="5">
-        <f>MIN(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
-        <v>0.879</v>
-      </c>
-      <c r="M23" s="5">
-        <f>MAX(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
-        <v>0.90099999999999991</v>
-      </c>
-      <c r="N23" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O23" s="5">
-        <f>N23*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P23" s="5">
-        <f>N23*1.05</f>
-        <v>0.99934990680000002</v>
+      <c r="K23" s="6">
+        <v>0.87769999999999992</v>
+      </c>
+      <c r="L23" s="6">
+        <v>0.86930000000000007</v>
+      </c>
+      <c r="M23" s="6">
+        <v>0.88549999999999995</v>
+      </c>
+      <c r="N23" s="6">
+        <v>0.95109999999999995</v>
+      </c>
+      <c r="O23" s="6">
+        <v>0.93889999999999996</v>
+      </c>
+      <c r="P23" s="6">
+        <v>0.95739999999999992</v>
       </c>
       <c r="Q23" s="5">
-        <f>AVERAGE(79.7,80.2,80,80,81.2,77.4)/100</f>
-        <v>0.79749999999999999</v>
+        <v>0.59399999999999997</v>
       </c>
       <c r="R23" s="5">
-        <f>MIN(79.7,80.2,80,80,81.2,77.4)/100</f>
-        <v>0.77400000000000002</v>
+        <f>Q23-3*(2.16/100)</f>
+        <v>0.5292</v>
       </c>
       <c r="S23" s="5">
-        <f>MAX(79.7,80.2,80,80,81.2,77.4)/100</f>
-        <v>0.81200000000000006</v>
+        <f>Q23+3*(2.16/100)</f>
+        <v>0.65879999999999994</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
-      </c>
-      <c r="F24" s="6">
-        <v>0.53783333333333327</v>
-      </c>
-      <c r="G24" s="6">
-        <f>13.249433/100</f>
-        <v>0.13249432999999999</v>
-      </c>
-      <c r="H24" s="7">
-        <f>1-SUM(F24:G24,I24)</f>
-        <v>2.4672336666666794E-2</v>
-      </c>
-      <c r="I24" s="5">
-        <v>0.30499999999999999</v>
+        <v>69</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
       </c>
       <c r="J24" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K24" s="6">
-        <v>0.83030000000000004</v>
-      </c>
-      <c r="L24" s="6">
-        <v>0.72499999999999998</v>
-      </c>
-      <c r="M24" s="6">
-        <v>0.9194</v>
-      </c>
-      <c r="N24" s="6">
-        <v>0.93189999999999995</v>
-      </c>
-      <c r="O24" s="6">
-        <v>0.86629999999999996</v>
-      </c>
-      <c r="P24" s="6">
-        <v>0.96779999999999999</v>
-      </c>
-      <c r="Q24" s="5">
-        <v>0.68700000000000006</v>
-      </c>
-      <c r="R24" s="10">
-        <f t="shared" ref="R24:R36" si="4">Q24*0.95</f>
-        <v>0.65265000000000006</v>
-      </c>
-      <c r="S24" s="10">
-        <f t="shared" ref="S24:S45" si="5">R24*1.05</f>
-        <v>0.68528250000000013</v>
+      <c r="K24" s="4">
+        <v>0.84588505065844988</v>
+      </c>
+      <c r="L24" s="4">
+        <f>K24*0.95</f>
+        <v>0.80359079812552736</v>
+      </c>
+      <c r="M24" s="4">
+        <f>L24*1.05</f>
+        <v>0.84377033803180379</v>
+      </c>
+      <c r="N24">
+        <v>0.93</v>
+      </c>
+      <c r="O24">
+        <f>N24*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P24">
+        <f>MIN(N24*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q24" s="4">
+        <v>0.71148214285714262</v>
+      </c>
+      <c r="R24" s="4">
+        <f>Q24*0.95</f>
+        <v>0.67590803571428548</v>
+      </c>
+      <c r="S24" s="4">
+        <f>R24*1.05</f>
+        <v>0.70970343749999976</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D25" t="s">
         <v>68</v>
       </c>
       <c r="E25" t="s">
-        <v>68</v>
-      </c>
-      <c r="F25" s="6">
-        <v>0.56188888888888899</v>
-      </c>
-      <c r="G25" s="6">
-        <v>8.6999999999999994E-2</v>
+        <v>69</v>
+      </c>
+      <c r="F25" s="5">
+        <f>AVERAGE(420.2,405.3,420.2,403.8,390.7,468.4)/1000</f>
+        <v>0.41809999999999997</v>
+      </c>
+      <c r="G25" s="5">
+        <f>AVERAGE(175.4,153.9,171.8,132.3,106.7,100.1)/1000</f>
+        <v>0.14003333333333337</v>
       </c>
       <c r="H25" s="7">
         <f>1-SUM(F25:G25,I25)</f>
-        <v>0.23711111111111105</v>
-      </c>
-      <c r="I25" s="8">
-        <v>0.114</v>
+        <v>0.41068333333333329</v>
+      </c>
+      <c r="I25" s="5">
+        <f>AVERAGE(28.6,37.6,28,37.3,25.9,29.7)/1000</f>
+        <v>3.1183333333333334E-2</v>
       </c>
       <c r="J25" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J25" si="5">SUM(F25:I25)</f>
         <v>1</v>
       </c>
-      <c r="K25" s="6">
-        <v>0.81159999999999999</v>
-      </c>
-      <c r="L25" s="6">
-        <v>0.70010000000000006</v>
-      </c>
-      <c r="M25" s="6">
-        <v>0.93319999999999992</v>
-      </c>
-      <c r="N25" s="6">
-        <v>0.95489999999999997</v>
-      </c>
-      <c r="O25" s="6">
-        <v>0.90229999999999999</v>
-      </c>
-      <c r="P25" s="6">
-        <v>0.98790000000000011</v>
+      <c r="K25" s="5">
+        <f>AVERAGE(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.89050000000000007</v>
+      </c>
+      <c r="L25" s="5">
+        <f>MIN(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.879</v>
+      </c>
+      <c r="M25" s="5">
+        <f>MAX(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.90099999999999991</v>
+      </c>
+      <c r="N25" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O25" s="5">
+        <f>N25*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P25" s="5">
+        <f>N25*1.05</f>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q25" s="5">
-        <v>0.68700000000000006</v>
-      </c>
-      <c r="R25" s="10">
-        <f t="shared" si="4"/>
-        <v>0.65265000000000006</v>
-      </c>
-      <c r="S25" s="10">
-        <f t="shared" si="5"/>
-        <v>0.68528250000000013</v>
+        <f>AVERAGE(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.79749999999999999</v>
+      </c>
+      <c r="R25" s="5">
+        <f>MIN(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="S25" s="5">
+        <f>MAX(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.81200000000000006</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>88</v>
+      </c>
+      <c r="B26" t="s">
+        <v>73</v>
       </c>
       <c r="C26" t="s">
         <v>68</v>
@@ -2991,62 +2996,70 @@
         <v>69</v>
       </c>
       <c r="F26" s="5">
-        <v>0</v>
+        <f>AVERAGE(420.2,405.3,420.2,403.8,390.7,468.4)/1000</f>
+        <v>0.41809999999999997</v>
       </c>
       <c r="G26" s="5">
-        <v>0</v>
-      </c>
-      <c r="H26" s="5">
-        <v>0</v>
+        <f>AVERAGE(175.4,153.9,171.8,132.3,106.7,100.1)/1000</f>
+        <v>0.14003333333333337</v>
+      </c>
+      <c r="H26" s="7">
+        <f>1-SUM(F26:G26,I26)</f>
+        <v>0.41068333333333329</v>
       </c>
       <c r="I26" s="5">
-        <v>1</v>
+        <f>AVERAGE(28.6,37.6,28,37.3,25.9,29.7)/1000</f>
+        <v>3.1183333333333334E-2</v>
       </c>
       <c r="J26" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K26" s="5">
-        <v>0</v>
+        <f>AVERAGE(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.89050000000000007</v>
       </c>
       <c r="L26" s="5">
-        <v>0</v>
+        <f>MIN(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.879</v>
       </c>
       <c r="M26" s="5">
-        <v>0</v>
+        <f>MAX(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.90099999999999991</v>
       </c>
       <c r="N26" s="5">
-        <v>0</v>
+        <v>0.95176181599999998</v>
       </c>
       <c r="O26" s="5">
         <f>N26*0.95</f>
-        <v>0</v>
+        <v>0.90417372519999994</v>
       </c>
       <c r="P26" s="5">
         <f>N26*1.05</f>
-        <v>0</v>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q26" s="5">
-        <v>0</v>
-      </c>
-      <c r="R26" s="10">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S26" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>AVERAGE(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.79749999999999999</v>
+      </c>
+      <c r="R26" s="5">
+        <f>MIN(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="S26" s="5">
+        <f>MAX(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.81200000000000006</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B27" t="s">
         <v>75</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D27" t="s">
         <v>68</v>
@@ -3055,322 +3068,312 @@
         <v>68</v>
       </c>
       <c r="F27" s="6">
-        <v>0.62166666666666659</v>
+        <v>0.53783333333333327</v>
       </c>
       <c r="G27" s="6">
-        <v>0.122</v>
+        <f>13.249433/100</f>
+        <v>0.13249432999999999</v>
       </c>
       <c r="H27" s="7">
         <f>1-SUM(F27:G27,I27)</f>
-        <v>0.14233333333333342</v>
-      </c>
-      <c r="I27" s="8">
-        <v>0.114</v>
+        <v>2.4672336666666794E-2</v>
+      </c>
+      <c r="I27" s="5">
+        <v>0.30499999999999999</v>
       </c>
       <c r="J27" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K27" s="6">
-        <v>0.78639999999999999</v>
+        <v>0.83030000000000004</v>
       </c>
       <c r="L27" s="6">
-        <v>0.71209999999999996</v>
+        <v>0.72499999999999998</v>
       </c>
       <c r="M27" s="6">
-        <v>0.84200000000000008</v>
+        <v>0.9194</v>
       </c>
       <c r="N27" s="6">
-        <v>0.9325</v>
+        <v>0.93189999999999995</v>
       </c>
       <c r="O27" s="6">
-        <v>0.91139999999999999</v>
+        <v>0.86629999999999996</v>
       </c>
       <c r="P27" s="6">
-        <v>0.94950000000000001</v>
+        <v>0.96779999999999999</v>
       </c>
       <c r="Q27" s="5">
-        <v>0.68900000000000006</v>
+        <v>0.68700000000000006</v>
       </c>
       <c r="R27" s="10">
-        <f t="shared" si="4"/>
-        <v>0.65455000000000008</v>
+        <f t="shared" ref="R27:R39" si="6">Q27*0.95</f>
+        <v>0.65265000000000006</v>
       </c>
       <c r="S27" s="10">
-        <f t="shared" si="5"/>
-        <v>0.6872775000000001</v>
+        <f t="shared" ref="S27:S45" si="7">R27*1.05</f>
+        <v>0.68528250000000013</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C28" t="s">
         <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E28" t="s">
-        <v>69</v>
-      </c>
-      <c r="F28">
-        <v>0.23</v>
-      </c>
-      <c r="G28">
-        <v>0.01</v>
-      </c>
-      <c r="H28">
-        <v>0.45</v>
-      </c>
-      <c r="I28">
-        <v>0.31</v>
+        <v>68</v>
+      </c>
+      <c r="F28" s="6">
+        <v>0.56188888888888899</v>
+      </c>
+      <c r="G28" s="6">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="H28" s="7">
+        <f>1-SUM(F28:G28,I28)</f>
+        <v>0.23711111111111105</v>
+      </c>
+      <c r="I28" s="8">
+        <v>0.114</v>
       </c>
       <c r="J28" s="9">
-        <f t="shared" ref="J28:J29" si="6">SUM(F28:I28)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K28">
-        <v>0.8</v>
-      </c>
-      <c r="L28" s="4">
-        <f>K28*0.95</f>
-        <v>0.76</v>
-      </c>
-      <c r="M28" s="4">
-        <f>L28*1.05</f>
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="N28">
-        <v>0.93</v>
-      </c>
-      <c r="O28">
-        <f>N28*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P28">
-        <f>MIN(N28*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q28">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="R28" s="4">
-        <f t="shared" si="4"/>
-        <v>0.55099999999999993</v>
-      </c>
-      <c r="S28" s="4">
-        <f t="shared" si="5"/>
-        <v>0.57855000000000001</v>
+      <c r="K28" s="6">
+        <v>0.81159999999999999</v>
+      </c>
+      <c r="L28" s="6">
+        <v>0.70010000000000006</v>
+      </c>
+      <c r="M28" s="6">
+        <v>0.93319999999999992</v>
+      </c>
+      <c r="N28" s="6">
+        <v>0.95489999999999997</v>
+      </c>
+      <c r="O28" s="6">
+        <v>0.90229999999999999</v>
+      </c>
+      <c r="P28" s="6">
+        <v>0.98790000000000011</v>
+      </c>
+      <c r="Q28" s="5">
+        <v>0.68700000000000006</v>
+      </c>
+      <c r="R28" s="10">
+        <f t="shared" si="6"/>
+        <v>0.65265000000000006</v>
+      </c>
+      <c r="S28" s="10">
+        <f t="shared" si="7"/>
+        <v>0.68528250000000013</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>96</v>
-      </c>
-      <c r="B29" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E29" t="s">
         <v>69</v>
       </c>
-      <c r="F29">
-        <v>0.23</v>
-      </c>
-      <c r="G29">
-        <v>0.01</v>
-      </c>
-      <c r="H29">
-        <v>0.45</v>
-      </c>
-      <c r="I29">
-        <v>0.31</v>
+      <c r="F29" s="5">
+        <v>0</v>
+      </c>
+      <c r="G29" s="5">
+        <v>0</v>
+      </c>
+      <c r="H29" s="5">
+        <v>0</v>
+      </c>
+      <c r="I29" s="5">
+        <v>1</v>
       </c>
       <c r="J29" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K29" s="5">
+        <v>0</v>
+      </c>
+      <c r="L29" s="5">
+        <v>0</v>
+      </c>
+      <c r="M29" s="5">
+        <v>0</v>
+      </c>
+      <c r="N29" s="5">
+        <v>0</v>
+      </c>
+      <c r="O29" s="5">
+        <f>N29*0.95</f>
+        <v>0</v>
+      </c>
+      <c r="P29" s="5">
+        <f>N29*1.05</f>
+        <v>0</v>
+      </c>
+      <c r="Q29" s="5">
+        <v>0</v>
+      </c>
+      <c r="R29" s="10">
         <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="K29">
-        <v>0.8</v>
-      </c>
-      <c r="L29" s="4">
-        <f>K29*0.95</f>
-        <v>0.76</v>
-      </c>
-      <c r="M29" s="4">
-        <f>L29*1.05</f>
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="N29">
-        <v>0.93</v>
-      </c>
-      <c r="O29">
-        <f>N29*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P29">
-        <f>MIN(N29*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q29">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="R29" s="4">
-        <f t="shared" si="4"/>
-        <v>0.55099999999999993</v>
-      </c>
-      <c r="S29" s="4">
-        <f t="shared" si="5"/>
-        <v>0.57855000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="S29" s="10">
+        <f t="shared" si="7"/>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
         <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E30" t="s">
-        <v>69</v>
-      </c>
-      <c r="F30">
-        <v>0.23</v>
-      </c>
-      <c r="G30">
-        <v>0.01</v>
-      </c>
-      <c r="H30">
-        <v>0.45</v>
-      </c>
-      <c r="I30">
-        <v>0.31</v>
+        <v>68</v>
+      </c>
+      <c r="F30" s="6">
+        <v>0.62166666666666659</v>
+      </c>
+      <c r="G30" s="6">
+        <v>0.122</v>
+      </c>
+      <c r="H30" s="7">
+        <f>1-SUM(F30:G30,I30)</f>
+        <v>0.14233333333333342</v>
+      </c>
+      <c r="I30" s="8">
+        <v>0.114</v>
       </c>
       <c r="J30" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K30">
-        <v>0.8</v>
-      </c>
-      <c r="L30" s="4">
-        <f>K30*0.95</f>
-        <v>0.76</v>
-      </c>
-      <c r="M30" s="4">
-        <f>L30*1.05</f>
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="N30">
-        <v>0.93</v>
-      </c>
-      <c r="O30">
-        <f>N30*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P30">
-        <f>MIN(N30*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q30">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="R30" s="4">
-        <f t="shared" si="4"/>
-        <v>0.55099999999999993</v>
-      </c>
-      <c r="S30" s="4">
-        <f t="shared" si="5"/>
-        <v>0.57855000000000001</v>
+      <c r="K30" s="6">
+        <v>0.78639999999999999</v>
+      </c>
+      <c r="L30" s="6">
+        <v>0.71209999999999996</v>
+      </c>
+      <c r="M30" s="6">
+        <v>0.84200000000000008</v>
+      </c>
+      <c r="N30" s="6">
+        <v>0.9325</v>
+      </c>
+      <c r="O30" s="6">
+        <v>0.91139999999999999</v>
+      </c>
+      <c r="P30" s="6">
+        <v>0.94950000000000001</v>
+      </c>
+      <c r="Q30" s="5">
+        <v>0.68900000000000006</v>
+      </c>
+      <c r="R30" s="10">
+        <f t="shared" si="6"/>
+        <v>0.65455000000000008</v>
+      </c>
+      <c r="S30" s="10">
+        <f t="shared" si="7"/>
+        <v>0.6872775000000001</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B31" t="s">
         <v>73</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E31" t="s">
         <v>69</v>
       </c>
-      <c r="F31" s="5">
-        <v>0.84</v>
-      </c>
-      <c r="G31" s="5">
-        <v>0.05</v>
-      </c>
-      <c r="H31" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="I31" s="5">
-        <v>0.04</v>
+      <c r="F31">
+        <v>0.23</v>
+      </c>
+      <c r="G31">
+        <v>0.01</v>
+      </c>
+      <c r="H31">
+        <v>0.45</v>
+      </c>
+      <c r="I31">
+        <v>0.31</v>
       </c>
       <c r="J31" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K31" s="5">
-        <v>0.88</v>
-      </c>
-      <c r="L31" s="10">
-        <f>K31*0.94</f>
-        <v>0.82719999999999994</v>
-      </c>
-      <c r="M31" s="10">
-        <f>L31*1.06</f>
-        <v>0.87683199999999994</v>
-      </c>
-      <c r="N31" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O31" s="5">
+      <c r="K31">
+        <v>0.8</v>
+      </c>
+      <c r="L31" s="4">
+        <f>K31*0.95</f>
+        <v>0.76</v>
+      </c>
+      <c r="M31" s="4">
+        <f>L31*1.05</f>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="N31">
+        <v>0.93</v>
+      </c>
+      <c r="O31">
         <f>N31*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P31" s="5">
-        <f>N31*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q31" s="5">
-        <v>0.77</v>
-      </c>
-      <c r="R31" s="10">
-        <f t="shared" si="4"/>
-        <v>0.73149999999999993</v>
-      </c>
-      <c r="S31" s="10">
-        <f t="shared" si="5"/>
-        <v>0.76807499999999995</v>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P31">
+        <f>MIN(N31*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q31">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="R31" s="4">
+        <f t="shared" si="6"/>
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="S31" s="4">
+        <f t="shared" si="7"/>
+        <v>0.57855000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C32" t="s">
         <v>68</v>
@@ -3379,194 +3382,199 @@
         <v>68</v>
       </c>
       <c r="E32" t="s">
-        <v>68</v>
-      </c>
-      <c r="F32" s="6">
-        <v>0.72292857142857125</v>
-      </c>
-      <c r="G32" s="6">
-        <f>11.68969/100</f>
-        <v>0.11689690000000001</v>
-      </c>
-      <c r="H32" s="7">
-        <f>1-SUM(F32:G32,I32)</f>
-        <v>5.4174528571428793E-2</v>
+        <v>69</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0.84</v>
+      </c>
+      <c r="G32" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="H32" s="5">
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="I32" s="5">
-        <v>0.106</v>
+        <v>0.04</v>
       </c>
       <c r="J32" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K32" s="6">
-        <v>0.86609999999999998</v>
-      </c>
-      <c r="L32" s="6">
-        <v>0.79749999999999999</v>
-      </c>
-      <c r="M32" s="6">
-        <v>0.93370000000000009</v>
-      </c>
-      <c r="N32" s="6">
-        <v>0.94900000000000007</v>
-      </c>
-      <c r="O32" s="6">
-        <v>0.90069999999999995</v>
-      </c>
-      <c r="P32" s="6">
-        <v>0.98250000000000004</v>
+      <c r="K32" s="5">
+        <v>0.88</v>
+      </c>
+      <c r="L32" s="10">
+        <f>K32*0.94</f>
+        <v>0.82719999999999994</v>
+      </c>
+      <c r="M32" s="10">
+        <f>L32*1.06</f>
+        <v>0.87683199999999994</v>
+      </c>
+      <c r="N32" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O32" s="5">
+        <f>N32*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P32" s="5">
+        <f>N32*1.05</f>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q32" s="5">
-        <v>0.68899999999999995</v>
+        <v>0.77</v>
       </c>
       <c r="R32" s="10">
-        <f t="shared" si="4"/>
-        <v>0.65454999999999997</v>
+        <f t="shared" si="6"/>
+        <v>0.73149999999999993</v>
       </c>
       <c r="S32" s="10">
-        <f t="shared" si="5"/>
-        <v>0.68727749999999999</v>
+        <f t="shared" si="7"/>
+        <v>0.76807499999999995</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E33" t="s">
         <v>69</v>
       </c>
-      <c r="F33" s="5">
-        <v>0</v>
-      </c>
-      <c r="G33" s="5">
-        <v>1</v>
-      </c>
-      <c r="H33" s="5">
-        <v>0</v>
-      </c>
-      <c r="I33" s="5">
-        <v>0</v>
+      <c r="F33">
+        <v>0.23</v>
+      </c>
+      <c r="G33">
+        <v>0.01</v>
+      </c>
+      <c r="H33">
+        <v>0.45</v>
+      </c>
+      <c r="I33">
+        <v>0.31</v>
       </c>
       <c r="J33" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K33" s="5">
-        <v>0</v>
-      </c>
-      <c r="L33" s="5">
+      <c r="K33">
+        <v>0.8</v>
+      </c>
+      <c r="L33" s="4">
         <f>K33*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="M33" s="5">
+        <v>0.76</v>
+      </c>
+      <c r="M33" s="4">
         <f>L33*1.05</f>
-        <v>0</v>
-      </c>
-      <c r="N33" s="6">
-        <v>0.94900000000000007</v>
-      </c>
-      <c r="O33" s="6">
-        <v>0.90069999999999995</v>
-      </c>
-      <c r="P33" s="6">
-        <v>0.98250000000000004</v>
-      </c>
-      <c r="Q33" s="5">
-        <v>0</v>
-      </c>
-      <c r="R33" s="10">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S33" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="N33">
+        <v>0.93</v>
+      </c>
+      <c r="O33">
+        <f>N33*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P33">
+        <f>MIN(N33*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q33">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="R33" s="4">
+        <f t="shared" si="6"/>
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="S33" s="4">
+        <f t="shared" si="7"/>
+        <v>0.57855000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>52</v>
+        <v>95</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C34" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E34" t="s">
-        <v>68</v>
-      </c>
-      <c r="F34" s="6">
-        <f>81.85/100</f>
-        <v>0.81849999999999989</v>
-      </c>
-      <c r="G34" s="6">
-        <f>0.1448625</f>
-        <v>0.14486250000000001</v>
-      </c>
-      <c r="H34" s="7">
-        <f>1-SUM(F34:G34,I34)</f>
-        <v>6.6375000000000739E-3</v>
-      </c>
-      <c r="I34" s="5">
-        <v>0.03</v>
+        <v>69</v>
+      </c>
+      <c r="F34">
+        <v>0.23</v>
+      </c>
+      <c r="G34">
+        <v>0.01</v>
+      </c>
+      <c r="H34">
+        <v>0.45</v>
+      </c>
+      <c r="I34">
+        <v>0.31</v>
       </c>
       <c r="J34" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K34" s="6">
-        <v>0.88379999999999992</v>
-      </c>
-      <c r="L34" s="6">
-        <v>0.87650000000000006</v>
-      </c>
-      <c r="M34" s="6">
-        <v>0.88790000000000002</v>
-      </c>
-      <c r="N34" s="6">
-        <v>0.96579999999999999</v>
-      </c>
-      <c r="O34" s="6">
-        <v>0.94930000000000003</v>
-      </c>
-      <c r="P34" s="6">
-        <v>0.98499999999999999</v>
-      </c>
-      <c r="Q34" s="5">
-        <v>0.88000000000000012</v>
-      </c>
-      <c r="R34" s="10">
-        <f t="shared" si="4"/>
-        <v>0.83600000000000008</v>
-      </c>
-      <c r="S34" s="10">
-        <f t="shared" si="5"/>
-        <v>0.87780000000000014</v>
+      <c r="K34">
+        <v>0.8</v>
+      </c>
+      <c r="L34" s="4">
+        <f>K34*0.95</f>
+        <v>0.76</v>
+      </c>
+      <c r="M34" s="4">
+        <f>L34*1.05</f>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="N34">
+        <v>0.93</v>
+      </c>
+      <c r="O34">
+        <f>N34*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P34">
+        <f>MIN(N34*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q34">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="R34" s="4">
+        <f t="shared" si="6"/>
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="S34" s="4">
+        <f t="shared" si="7"/>
+        <v>0.57855000000000001</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
         <v>68</v>
@@ -3575,187 +3583,191 @@
         <v>68</v>
       </c>
       <c r="F35" s="6">
-        <v>0.75900000000000001</v>
+        <v>0.72292857142857125</v>
       </c>
       <c r="G35" s="6">
-        <v>0.10100000000000001</v>
+        <f>11.68969/100</f>
+        <v>0.11689690000000001</v>
       </c>
       <c r="H35" s="7">
         <f>1-SUM(F35:G35,I35)</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="8">
-        <v>0.14000000000000001</v>
+        <v>5.4174528571428793E-2</v>
+      </c>
+      <c r="I35" s="5">
+        <v>0.106</v>
       </c>
       <c r="J35" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K35" s="6">
-        <v>0.94140000000000001</v>
+        <v>0.86609999999999998</v>
       </c>
       <c r="L35" s="6">
-        <v>0.92920000000000003</v>
+        <v>0.79749999999999999</v>
       </c>
       <c r="M35" s="6">
-        <v>0.95040000000000002</v>
+        <v>0.93370000000000009</v>
       </c>
       <c r="N35" s="6">
-        <v>0.97010000000000007</v>
+        <v>0.94900000000000007</v>
       </c>
       <c r="O35" s="6">
-        <v>0.96840000000000004</v>
+        <v>0.90069999999999995</v>
       </c>
       <c r="P35" s="6">
-        <v>0.97239999999999993</v>
+        <v>0.98250000000000004</v>
       </c>
       <c r="Q35" s="5">
-        <v>0.68000000000000016</v>
+        <v>0.68899999999999995</v>
       </c>
       <c r="R35" s="10">
-        <f t="shared" si="4"/>
-        <v>0.64600000000000013</v>
+        <f t="shared" si="6"/>
+        <v>0.65454999999999997</v>
       </c>
       <c r="S35" s="10">
-        <f t="shared" si="5"/>
-        <v>0.67830000000000013</v>
+        <f t="shared" si="7"/>
+        <v>0.68727749999999999</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="B36" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
         <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>68</v>
-      </c>
-      <c r="F36" s="6">
-        <v>0.65300000000000002</v>
-      </c>
-      <c r="G36" s="6">
-        <v>0.02</v>
-      </c>
-      <c r="H36" s="7">
-        <f>1-SUM(F36:G36,I36)</f>
-        <v>0.2569999999999999</v>
+        <v>69</v>
+      </c>
+      <c r="F36" s="5">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5">
+        <v>1</v>
+      </c>
+      <c r="H36" s="5">
+        <v>0</v>
       </c>
       <c r="I36" s="5">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="J36" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K36" s="6">
-        <v>0.89379999999999993</v>
-      </c>
-      <c r="L36" s="6">
-        <v>0.8881</v>
-      </c>
-      <c r="M36" s="6">
-        <v>0.89969999999999994</v>
+      <c r="K36" s="5">
+        <v>0</v>
+      </c>
+      <c r="L36" s="5">
+        <f>K36*0.95</f>
+        <v>0</v>
+      </c>
+      <c r="M36" s="5">
+        <f>L36*1.05</f>
+        <v>0</v>
       </c>
       <c r="N36" s="6">
-        <v>0.95799999999999996</v>
+        <v>0.94900000000000007</v>
       </c>
       <c r="O36" s="6">
-        <v>0.9323999999999999</v>
+        <v>0.90069999999999995</v>
       </c>
       <c r="P36" s="6">
-        <v>0.97730000000000006</v>
+        <v>0.98250000000000004</v>
       </c>
       <c r="Q36" s="5">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="R36" s="10">
-        <f t="shared" si="4"/>
-        <v>0.77899999999999991</v>
+        <f t="shared" si="6"/>
+        <v>0</v>
       </c>
       <c r="S36" s="10">
-        <f t="shared" si="5"/>
-        <v>0.81794999999999995</v>
+        <f t="shared" si="7"/>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C37" t="s">
         <v>68</v>
       </c>
       <c r="D37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E37" t="s">
-        <v>69</v>
-      </c>
-      <c r="F37" s="5">
-        <v>0</v>
-      </c>
-      <c r="G37" s="5">
-        <v>1</v>
-      </c>
-      <c r="H37" s="5">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F37" s="6">
+        <f>81.85/100</f>
+        <v>0.81849999999999989</v>
+      </c>
+      <c r="G37" s="6">
+        <f>0.1448625</f>
+        <v>0.14486250000000001</v>
+      </c>
+      <c r="H37" s="7">
+        <f>1-SUM(F37:G37,I37)</f>
+        <v>6.6375000000000739E-3</v>
       </c>
       <c r="I37" s="5">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="J37" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K37" s="5">
-        <v>0</v>
-      </c>
-      <c r="L37" s="5">
-        <v>0</v>
-      </c>
-      <c r="M37" s="5">
-        <v>0</v>
-      </c>
-      <c r="N37" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O37" s="5">
-        <f t="shared" ref="O37:O45" si="7">N37*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P37" s="5">
-        <f>N37*1.05</f>
-        <v>0.99934990680000002</v>
+      <c r="K37" s="6">
+        <v>0.88379999999999992</v>
+      </c>
+      <c r="L37" s="6">
+        <v>0.87650000000000006</v>
+      </c>
+      <c r="M37" s="6">
+        <v>0.88790000000000002</v>
+      </c>
+      <c r="N37" s="6">
+        <v>0.96579999999999999</v>
+      </c>
+      <c r="O37" s="6">
+        <v>0.94930000000000003</v>
+      </c>
+      <c r="P37" s="6">
+        <v>0.98499999999999999</v>
       </c>
       <c r="Q37" s="5">
-        <v>0</v>
-      </c>
-      <c r="R37" s="7">
-        <v>0</v>
-      </c>
-      <c r="S37" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.88000000000000012</v>
+      </c>
+      <c r="R37" s="10">
+        <f t="shared" si="6"/>
+        <v>0.83600000000000008</v>
+      </c>
+      <c r="S37" s="10">
+        <f t="shared" si="7"/>
+        <v>0.87780000000000014</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D38" t="s">
         <v>68</v>
@@ -3764,131 +3776,124 @@
         <v>68</v>
       </c>
       <c r="F38" s="6">
-        <v>0.66174999999999995</v>
+        <v>0.75900000000000001</v>
       </c>
       <c r="G38" s="6">
-        <f>1.126924/100</f>
-        <v>1.126924E-2</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="H38" s="7">
         <f>1-SUM(F38:G38,I38)</f>
-        <v>0.25398076000000014</v>
-      </c>
-      <c r="I38" s="5">
-        <v>7.2999999999999995E-2</v>
+        <v>0</v>
+      </c>
+      <c r="I38" s="8">
+        <v>0.14000000000000001</v>
       </c>
       <c r="J38" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K38" s="6">
-        <v>0.87599999999999989</v>
+        <v>0.94140000000000001</v>
       </c>
       <c r="L38" s="6">
-        <v>0.8206</v>
+        <v>0.92920000000000003</v>
       </c>
       <c r="M38" s="6">
-        <v>0.92709999999999992</v>
-      </c>
-      <c r="N38" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O38" s="5">
+        <v>0.95040000000000002</v>
+      </c>
+      <c r="N38" s="6">
+        <v>0.97010000000000007</v>
+      </c>
+      <c r="O38" s="6">
+        <v>0.96840000000000004</v>
+      </c>
+      <c r="P38" s="6">
+        <v>0.97239999999999993</v>
+      </c>
+      <c r="Q38" s="5">
+        <v>0.68000000000000016</v>
+      </c>
+      <c r="R38" s="10">
+        <f t="shared" si="6"/>
+        <v>0.64600000000000013</v>
+      </c>
+      <c r="S38" s="10">
         <f t="shared" si="7"/>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P38" s="5">
-        <f>N38*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q38" s="5">
-        <v>0.875</v>
-      </c>
-      <c r="R38" s="10">
-        <f t="shared" ref="R38:R46" si="8">Q38*0.95</f>
-        <v>0.83124999999999993</v>
-      </c>
-      <c r="S38" s="10">
-        <f t="shared" si="5"/>
-        <v>0.87281249999999999</v>
+        <v>0.67830000000000013</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C39" t="s">
         <v>69</v>
       </c>
       <c r="D39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E39" t="s">
-        <v>69</v>
-      </c>
-      <c r="F39">
-        <v>0.63800000000000001</v>
-      </c>
-      <c r="G39">
-        <v>6.0999999999999999E-2</v>
+        <v>68</v>
+      </c>
+      <c r="F39" s="6">
+        <v>0.65300000000000002</v>
+      </c>
+      <c r="G39" s="6">
+        <v>0.02</v>
       </c>
       <c r="H39" s="7">
         <f>1-SUM(F39:G39,I39)</f>
-        <v>0.21199999999999997</v>
-      </c>
-      <c r="I39">
-        <v>8.8999999999999996E-2</v>
+        <v>0.2569999999999999</v>
+      </c>
+      <c r="I39" s="5">
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="J39" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K39">
-        <v>0.81</v>
-      </c>
-      <c r="L39" s="4">
-        <f>K39*0.95</f>
-        <v>0.76949999999999996</v>
-      </c>
-      <c r="M39" s="4">
-        <f>L39*1.05</f>
-        <v>0.807975</v>
-      </c>
-      <c r="N39">
-        <v>0.93</v>
-      </c>
-      <c r="O39">
+      <c r="K39" s="6">
+        <v>0.89379999999999993</v>
+      </c>
+      <c r="L39" s="6">
+        <v>0.8881</v>
+      </c>
+      <c r="M39" s="6">
+        <v>0.89969999999999994</v>
+      </c>
+      <c r="N39" s="6">
+        <v>0.95799999999999996</v>
+      </c>
+      <c r="O39" s="6">
+        <v>0.9323999999999999</v>
+      </c>
+      <c r="P39" s="6">
+        <v>0.97730000000000006</v>
+      </c>
+      <c r="Q39" s="5">
+        <v>0.82</v>
+      </c>
+      <c r="R39" s="10">
+        <f t="shared" si="6"/>
+        <v>0.77899999999999991</v>
+      </c>
+      <c r="S39" s="10">
         <f t="shared" si="7"/>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P39">
-        <f>MIN(N39*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q39">
-        <v>0.72</v>
-      </c>
-      <c r="R39" s="4">
-        <f t="shared" si="8"/>
-        <v>0.68399999999999994</v>
-      </c>
-      <c r="S39" s="4">
-        <f t="shared" si="5"/>
-        <v>0.71819999999999995</v>
+        <v>0.81794999999999995</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B40" t="s">
         <v>73</v>
       </c>
       <c r="C40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D40" t="s">
         <v>69</v>
@@ -3896,128 +3901,125 @@
       <c r="E40" t="s">
         <v>69</v>
       </c>
-      <c r="F40">
-        <v>0.32400000000000001</v>
-      </c>
-      <c r="G40">
-        <v>2.1999999999999999E-2</v>
-      </c>
-      <c r="H40">
-        <v>0.58299999999999996</v>
-      </c>
-      <c r="I40">
-        <v>7.0999999999999994E-2</v>
+      <c r="F40" s="5">
+        <v>0</v>
+      </c>
+      <c r="G40" s="5">
+        <v>1</v>
+      </c>
+      <c r="H40" s="5">
+        <v>0</v>
+      </c>
+      <c r="I40" s="5">
+        <v>0</v>
       </c>
       <c r="J40" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K40">
-        <v>0.87</v>
-      </c>
-      <c r="L40" s="4">
-        <f>K40*0.95</f>
-        <v>0.82650000000000001</v>
-      </c>
-      <c r="M40" s="4">
-        <f>L40*1.05</f>
-        <v>0.86782500000000007</v>
-      </c>
-      <c r="N40">
-        <v>0.93</v>
-      </c>
-      <c r="O40">
+      <c r="K40" s="5">
+        <v>0</v>
+      </c>
+      <c r="L40" s="5">
+        <v>0</v>
+      </c>
+      <c r="M40" s="5">
+        <v>0</v>
+      </c>
+      <c r="N40" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O40" s="5">
+        <f t="shared" ref="O40:O45" si="8">N40*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P40" s="5">
+        <f>N40*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q40" s="5">
+        <v>0</v>
+      </c>
+      <c r="R40" s="7">
+        <v>0</v>
+      </c>
+      <c r="S40" s="7">
         <f t="shared" si="7"/>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P40">
-        <f>MIN(N40*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q40">
-        <v>0.61</v>
-      </c>
-      <c r="R40" s="4">
-        <f t="shared" si="8"/>
-        <v>0.57950000000000002</v>
-      </c>
-      <c r="S40" s="4">
-        <f t="shared" si="5"/>
-        <v>0.60847499999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B41" t="s">
         <v>73</v>
       </c>
       <c r="C41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E41" t="s">
-        <v>69</v>
-      </c>
-      <c r="F41">
-        <v>0.377</v>
-      </c>
-      <c r="G41">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="H41">
-        <v>0.52800000000000002</v>
-      </c>
-      <c r="I41">
-        <v>7.6999999999999999E-2</v>
+        <v>68</v>
+      </c>
+      <c r="F41" s="6">
+        <v>0.66174999999999995</v>
+      </c>
+      <c r="G41" s="6">
+        <f>1.126924/100</f>
+        <v>1.126924E-2</v>
+      </c>
+      <c r="H41" s="7">
+        <f>1-SUM(F41:G41,I41)</f>
+        <v>0.25398076000000014</v>
+      </c>
+      <c r="I41" s="5">
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="J41" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K41">
-        <v>0.87</v>
-      </c>
-      <c r="L41" s="4">
-        <f>K41*0.95</f>
-        <v>0.82650000000000001</v>
-      </c>
-      <c r="M41" s="4">
-        <f>L41*1.05</f>
-        <v>0.86782500000000007</v>
-      </c>
-      <c r="N41">
-        <v>0.93</v>
-      </c>
-      <c r="O41">
+      <c r="K41" s="6">
+        <v>0.87599999999999989</v>
+      </c>
+      <c r="L41" s="6">
+        <v>0.8206</v>
+      </c>
+      <c r="M41" s="6">
+        <v>0.92709999999999992</v>
+      </c>
+      <c r="N41" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O41" s="5">
+        <f t="shared" si="8"/>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P41" s="5">
+        <f>N41*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q41" s="5">
+        <v>0.875</v>
+      </c>
+      <c r="R41" s="10">
+        <f>Q41*0.95</f>
+        <v>0.83124999999999993</v>
+      </c>
+      <c r="S41" s="10">
         <f t="shared" si="7"/>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P41">
-        <f>MIN(N41*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q41">
-        <v>0.61</v>
-      </c>
-      <c r="R41" s="4">
-        <f t="shared" si="8"/>
-        <v>0.57950000000000002</v>
-      </c>
-      <c r="S41" s="4">
-        <f t="shared" si="5"/>
-        <v>0.60847499999999999</v>
+        <v>0.87281249999999999</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C42" t="s">
         <v>69</v>
@@ -4029,37 +4031,38 @@
         <v>69</v>
       </c>
       <c r="F42">
-        <v>2.9000000000000001E-2</v>
+        <v>0.63800000000000001</v>
       </c>
       <c r="G42">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="H42">
-        <v>0.92500000000000004</v>
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="H42" s="7">
+        <f>1-SUM(F42:G42,I42)</f>
+        <v>0.21199999999999997</v>
       </c>
       <c r="I42">
-        <v>3.9E-2</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="J42" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K42">
-        <v>0.84000000000000008</v>
+        <v>0.81</v>
       </c>
       <c r="L42" s="4">
         <f>K42*0.95</f>
-        <v>0.79800000000000004</v>
+        <v>0.76949999999999996</v>
       </c>
       <c r="M42" s="4">
         <f>L42*1.05</f>
-        <v>0.83790000000000009</v>
+        <v>0.807975</v>
       </c>
       <c r="N42">
         <v>0.93</v>
       </c>
       <c r="O42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P42">
@@ -4067,160 +4070,155 @@
         <v>0.97650000000000015</v>
       </c>
       <c r="Q42">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="R42" s="4">
-        <f t="shared" si="8"/>
-        <v>0.66499999999999992</v>
+        <f>Q42*0.95</f>
+        <v>0.68399999999999994</v>
       </c>
       <c r="S42" s="4">
-        <f t="shared" si="5"/>
-        <v>0.69824999999999993</v>
+        <f t="shared" si="7"/>
+        <v>0.71819999999999995</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B43" t="s">
         <v>73</v>
       </c>
       <c r="C43" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D43" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E43" t="s">
         <v>69</v>
       </c>
-      <c r="F43" s="5">
-        <v>0.13</v>
-      </c>
-      <c r="G43" s="5">
-        <v>0.02</v>
-      </c>
-      <c r="H43" s="7">
-        <f>1-SUM(F43:G43,I43)</f>
-        <v>0.83000000000000007</v>
-      </c>
-      <c r="I43" s="5">
-        <v>0.02</v>
+      <c r="F43">
+        <v>0.32400000000000001</v>
+      </c>
+      <c r="G43">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="H43">
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="I43">
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="J43" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K43" s="5">
-        <v>0.9</v>
-      </c>
-      <c r="L43" s="10">
-        <f>K43*0.94</f>
-        <v>0.84599999999999997</v>
-      </c>
-      <c r="M43" s="10">
-        <f>L43*1.06</f>
-        <v>0.89676</v>
-      </c>
-      <c r="N43" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O43" s="5">
+      <c r="K43">
+        <v>0.87</v>
+      </c>
+      <c r="L43" s="4">
+        <f>K43*0.95</f>
+        <v>0.82650000000000001</v>
+      </c>
+      <c r="M43" s="4">
+        <f>L43*1.05</f>
+        <v>0.86782500000000007</v>
+      </c>
+      <c r="N43">
+        <v>0.93</v>
+      </c>
+      <c r="O43">
+        <f t="shared" si="8"/>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P43">
+        <f>MIN(N43*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q43">
+        <v>0.61</v>
+      </c>
+      <c r="R43" s="4">
+        <f>Q43*0.95</f>
+        <v>0.57950000000000002</v>
+      </c>
+      <c r="S43" s="4">
         <f t="shared" si="7"/>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P43" s="5">
-        <f>N43*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q43" s="5">
-        <v>0.8</v>
-      </c>
-      <c r="R43" s="10">
-        <f t="shared" si="8"/>
-        <v>0.76</v>
-      </c>
-      <c r="S43" s="10">
-        <f t="shared" si="5"/>
-        <v>0.79800000000000004</v>
+        <v>0.60847499999999999</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B44" t="s">
         <v>73</v>
       </c>
       <c r="C44" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D44" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E44" t="s">
         <v>69</v>
       </c>
-      <c r="F44" s="5">
-        <f>766/1000</f>
-        <v>0.76600000000000001</v>
-      </c>
-      <c r="G44" s="5">
-        <f>74/1000</f>
-        <v>7.3999999999999996E-2</v>
-      </c>
-      <c r="H44" s="7">
-        <f>1-SUM(F44:G44,I44)</f>
-        <v>0.15300000000000002</v>
-      </c>
-      <c r="I44" s="5">
-        <f>7/1000</f>
-        <v>7.0000000000000001E-3</v>
+      <c r="F44">
+        <v>0.377</v>
+      </c>
+      <c r="G44">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="H44">
+        <v>0.52800000000000002</v>
+      </c>
+      <c r="I44">
+        <v>7.6999999999999999E-2</v>
       </c>
       <c r="J44" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K44" s="5">
-        <v>0.89</v>
-      </c>
-      <c r="L44" s="10">
-        <f>K44*0.94</f>
-        <v>0.83660000000000001</v>
-      </c>
-      <c r="M44" s="10">
-        <f>L44*1.06</f>
-        <v>0.88679600000000003</v>
-      </c>
-      <c r="N44" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O44" s="5">
+      <c r="K44">
+        <v>0.87</v>
+      </c>
+      <c r="L44" s="4">
+        <f>K44*0.95</f>
+        <v>0.82650000000000001</v>
+      </c>
+      <c r="M44" s="4">
+        <f>L44*1.05</f>
+        <v>0.86782500000000007</v>
+      </c>
+      <c r="N44">
+        <v>0.93</v>
+      </c>
+      <c r="O44">
+        <f t="shared" si="8"/>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P44">
+        <f>MIN(N44*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q44">
+        <v>0.61</v>
+      </c>
+      <c r="R44" s="4">
+        <f>Q44*0.95</f>
+        <v>0.57950000000000002</v>
+      </c>
+      <c r="S44" s="4">
         <f t="shared" si="7"/>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P44" s="5">
-        <f>N44*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q44" s="5">
-        <v>0.75</v>
-      </c>
-      <c r="R44" s="10">
-        <f t="shared" si="8"/>
-        <v>0.71249999999999991</v>
-      </c>
-      <c r="S44" s="10">
-        <f t="shared" si="5"/>
-        <v>0.74812499999999993</v>
+        <v>0.60847499999999999</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B45" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C45" t="s">
         <v>69</v>
@@ -4232,37 +4230,37 @@
         <v>69</v>
       </c>
       <c r="F45">
-        <v>0.48</v>
+        <v>2.9000000000000001E-2</v>
       </c>
       <c r="G45">
-        <v>0.04</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="H45">
-        <v>0.41</v>
+        <v>0.92500000000000004</v>
       </c>
       <c r="I45">
-        <v>7.0000000000000007E-2</v>
+        <v>3.9E-2</v>
       </c>
       <c r="J45" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K45">
-        <v>0.82000000000000006</v>
+        <v>0.84000000000000008</v>
       </c>
       <c r="L45" s="4">
         <f>K45*0.95</f>
-        <v>0.77900000000000003</v>
+        <v>0.79800000000000004</v>
       </c>
       <c r="M45" s="4">
         <f>L45*1.05</f>
-        <v>0.81795000000000007</v>
+        <v>0.83790000000000009</v>
       </c>
       <c r="N45">
         <v>0.93</v>
       </c>
       <c r="O45">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P45">
@@ -4273,20 +4271,20 @@
         <v>0.7</v>
       </c>
       <c r="R45" s="4">
-        <f t="shared" si="8"/>
+        <f>Q45*0.95</f>
         <v>0.66499999999999992</v>
       </c>
       <c r="S45" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.69824999999999993</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="B46" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C46" t="s">
         <v>68</v>
@@ -4297,140 +4295,272 @@
       <c r="E46" t="s">
         <v>69</v>
       </c>
-      <c r="F46" s="11">
-        <v>0.84</v>
-      </c>
-      <c r="G46" s="11">
-        <v>0.05</v>
-      </c>
-      <c r="H46" s="11">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="I46" s="11">
-        <v>0.04</v>
-      </c>
-      <c r="J46" s="12">
-        <f t="shared" ref="J46" si="9">SUM(F46:I46)</f>
+      <c r="F46" s="5">
+        <f>AVERAGE('trash fish table'!F2:F6)</f>
+        <v>0.56830740870546492</v>
+      </c>
+      <c r="G46" s="5">
+        <f>AVERAGE('trash fish table'!G2:G6)</f>
+        <v>0.2240987667741102</v>
+      </c>
+      <c r="H46" s="5">
+        <f>AVERAGE('trash fish table'!I2:I6)</f>
+        <v>9.0773327441505319E-2</v>
+      </c>
+      <c r="I46" s="5">
+        <f>AVERAGE('trash fish table'!H2:H6)</f>
+        <v>0.11682049707891951</v>
+      </c>
+      <c r="J46" s="9">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K46" s="11">
-        <v>0.88</v>
-      </c>
-      <c r="L46" s="11">
-        <f>K46*0.94</f>
-        <v>0.82719999999999994</v>
-      </c>
-      <c r="M46" s="11">
-        <f>L46*1.06</f>
-        <v>0.87683199999999994</v>
-      </c>
-      <c r="N46" s="11">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O46" s="11">
-        <f>N46*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P46" s="11">
-        <f>N46*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q46" s="11">
-        <v>0.77</v>
-      </c>
-      <c r="R46" s="11">
-        <f t="shared" si="8"/>
-        <v>0.73149999999999993</v>
-      </c>
-      <c r="S46" s="11">
-        <f t="shared" ref="S46" si="10">R46*1.05</f>
-        <v>0.76807499999999995</v>
+      <c r="K46" s="10">
+        <v>0.87980000000000003</v>
+      </c>
+      <c r="L46" s="10">
+        <v>0.82969999999999999</v>
+      </c>
+      <c r="M46" s="10">
+        <v>0.92209999999999992</v>
+      </c>
+      <c r="N46" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O46" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P46" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q46" s="10">
+        <f>83.3/100</f>
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="R46" s="10">
+        <f>74.5/100</f>
+        <v>0.745</v>
+      </c>
+      <c r="S46" s="10">
+        <f>92.6/100</f>
+        <v>0.92599999999999993</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>113</v>
+        <v>31</v>
       </c>
       <c r="B47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C47" t="s">
         <v>68</v>
       </c>
       <c r="D47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E47" t="s">
         <v>69</v>
       </c>
       <c r="F47" s="5">
-        <f>AVERAGE('trash fish table'!F2:F6)</f>
-        <v>0.56830740870546492</v>
+        <v>0.13</v>
       </c>
       <c r="G47" s="5">
-        <f>AVERAGE('trash fish table'!G2:G6)</f>
-        <v>0.2240987667741102</v>
-      </c>
-      <c r="H47" s="5">
-        <f>AVERAGE('trash fish table'!I2:I6)</f>
-        <v>9.0773327441505319E-2</v>
+        <v>0.02</v>
+      </c>
+      <c r="H47" s="7">
+        <f>1-SUM(F47:G47,I47)</f>
+        <v>0.83000000000000007</v>
       </c>
       <c r="I47" s="5">
-        <f>AVERAGE('trash fish table'!H2:H6)</f>
-        <v>0.11682049707891951</v>
+        <v>0.02</v>
       </c>
       <c r="J47" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K47" s="10">
-        <v>0.87980000000000003</v>
+      <c r="K47" s="5">
+        <v>0.9</v>
       </c>
       <c r="L47" s="10">
-        <v>0.82969999999999999</v>
+        <f>K47*0.94</f>
+        <v>0.84599999999999997</v>
       </c>
       <c r="M47" s="10">
-        <v>0.92209999999999992</v>
-      </c>
-      <c r="N47" s="10">
-        <v>0.95669999999999999</v>
-      </c>
-      <c r="O47" s="10">
-        <v>0.8993000000000001</v>
-      </c>
-      <c r="P47" s="10">
-        <v>0.99199999999999999</v>
-      </c>
-      <c r="Q47" s="10">
-        <f>83.3/100</f>
-        <v>0.83299999999999996</v>
+        <f>L47*1.06</f>
+        <v>0.89676</v>
+      </c>
+      <c r="N47" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O47" s="5">
+        <f>N47*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P47" s="5">
+        <f>N47*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q47" s="5">
+        <v>0.8</v>
       </c>
       <c r="R47" s="10">
-        <f>74.5/100</f>
-        <v>0.745</v>
+        <f>Q47*0.95</f>
+        <v>0.76</v>
       </c>
       <c r="S47" s="10">
-        <f>92.6/100</f>
-        <v>0.92599999999999993</v>
+        <f>R47*1.05</f>
+        <v>0.79800000000000004</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48" t="s">
+        <v>68</v>
+      </c>
+      <c r="D48" t="s">
+        <v>68</v>
+      </c>
+      <c r="E48" t="s">
+        <v>69</v>
+      </c>
+      <c r="F48" s="5">
+        <f>766/1000</f>
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="G48" s="5">
+        <f>74/1000</f>
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="H48" s="7">
+        <f>1-SUM(F48:G48,I48)</f>
+        <v>0.15300000000000002</v>
+      </c>
+      <c r="I48" s="5">
+        <f>7/1000</f>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="J48" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K48" s="5">
+        <v>0.89</v>
+      </c>
+      <c r="L48" s="10">
+        <f>K48*0.94</f>
+        <v>0.83660000000000001</v>
+      </c>
+      <c r="M48" s="10">
+        <f>L48*1.06</f>
+        <v>0.88679600000000003</v>
+      </c>
+      <c r="N48" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O48" s="5">
+        <f>N48*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P48" s="5">
+        <f>N48*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q48" s="5">
+        <v>0.75</v>
+      </c>
+      <c r="R48" s="10">
+        <f>Q48*0.95</f>
+        <v>0.71249999999999991</v>
+      </c>
+      <c r="S48" s="10">
+        <f>R48*1.05</f>
+        <v>0.74812499999999993</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B49" t="s">
+        <v>72</v>
+      </c>
+      <c r="C49" t="s">
+        <v>69</v>
+      </c>
+      <c r="D49" t="s">
+        <v>69</v>
+      </c>
+      <c r="E49" t="s">
+        <v>69</v>
+      </c>
+      <c r="F49">
+        <v>0.48</v>
+      </c>
+      <c r="G49">
+        <v>0.04</v>
+      </c>
+      <c r="H49">
+        <v>0.41</v>
+      </c>
+      <c r="I49">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="J49" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K49">
+        <v>0.82000000000000006</v>
+      </c>
+      <c r="L49" s="4">
+        <f>K49*0.95</f>
+        <v>0.77900000000000003</v>
+      </c>
+      <c r="M49" s="4">
+        <f>L49*1.05</f>
+        <v>0.81795000000000007</v>
+      </c>
+      <c r="N49">
+        <v>0.93</v>
+      </c>
+      <c r="O49">
+        <f>N49*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P49">
+        <f>MIN(N49*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q49">
+        <v>0.7</v>
+      </c>
+      <c r="R49" s="4">
+        <f>Q49*0.95</f>
+        <v>0.66499999999999992</v>
+      </c>
+      <c r="S49" s="4">
+        <f>R49*1.05</f>
+        <v>0.69824999999999993</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S45" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S45">
-      <sortCondition ref="A1:A45"/>
+  <autoFilter ref="A1:S47" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S49">
+      <sortCondition ref="A1:A47"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="K2:S36">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+  <conditionalFormatting sqref="K2:S38">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K46:S46">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K47:S47">
+  <conditionalFormatting sqref="K48:S49">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>1</formula>
     </cfRule>

</xml_diff>

<commit_message>
Updated parameters, individual farm check plots
</commit_message>
<xml_diff>
--- a/data/raw_data/all_ingredients.xlsx
+++ b/data/raw_data/all_ingredients.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC45CDDA-4947-4CF3-ACD1-5B3569575FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0160536-06D3-4C16-AF8C-A63E1AB01DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
+    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="all_ingredients" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="trash fish table" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sources!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="127">
   <si>
     <t>ingredient</t>
   </si>
@@ -386,7 +386,40 @@
     <t>lupin-seed</t>
   </si>
   <si>
-    <t>blood-meal</t>
+    <t>poultry-blood-meal</t>
+  </si>
+  <si>
+    <t>peanut-meal</t>
+  </si>
+  <si>
+    <t>Composition and protein digestibility from feedipedia (https://www.feedipedia.org/node/699). Carb digestibility from https://onlinelibrary.wiley.com/doi/epdf/10.1111/j.1749-7345.2004.tb01069.x</t>
+  </si>
+  <si>
+    <t>squid-meal</t>
+  </si>
+  <si>
+    <t>cod-liver-oil</t>
+  </si>
+  <si>
+    <t>rice-bran</t>
+  </si>
+  <si>
+    <t>wheat-bran</t>
+  </si>
+  <si>
+    <t>copra-meal</t>
+  </si>
+  <si>
+    <t>Digestibility values taken from fishmeal-trimmings, except for protein which came from https://web.archive.org/web/20250422235548/https://www.fao.org/fileadmin/user_upload/affris/docs/Gilthead_Seabream/English/table_10.htm</t>
+  </si>
+  <si>
+    <t>Copra meal and coconut by-products | Feedipedia</t>
+  </si>
+  <si>
+    <t>Rice bran and other rice by-products | Feedipedia</t>
+  </si>
+  <si>
+    <t>Wheat bran | Feedipedia</t>
   </si>
 </sst>
 </file>
@@ -544,6 +577,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -922,7 +956,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -941,6 +975,9 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="44"/>
     <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="44" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="44" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="45">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -989,7 +1026,77 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1340,14 +1447,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-  <dimension ref="A1:S49"/>
+  <dimension ref="A1:S55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.6640625" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" hidden="1" customWidth="1"/>
     <col min="6" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
     <col min="11" max="19" width="12.88671875" customWidth="1"/>
@@ -1441,7 +1548,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="9">
-        <f t="shared" ref="J2:J49" si="0">SUM(F2:I2)</f>
+        <f t="shared" ref="J2:J55" si="0">SUM(F2:I2)</f>
         <v>1</v>
       </c>
       <c r="K2" s="5">
@@ -4549,19 +4656,323 @@
         <v>0.69824999999999993</v>
       </c>
     </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>116</v>
+      </c>
+      <c r="B50" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" t="s">
+        <v>69</v>
+      </c>
+      <c r="F50" s="5">
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="G50" s="5">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="H50" s="9">
+        <f>1-F50-G50-I50</f>
+        <v>0.37699999999999995</v>
+      </c>
+      <c r="I50" s="5">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="J50" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K50" s="16">
+        <v>0.81</v>
+      </c>
+      <c r="L50" s="4">
+        <f>K50*0.95</f>
+        <v>0.76949999999999996</v>
+      </c>
+      <c r="M50" s="4">
+        <f>L50*1.05</f>
+        <v>0.807975</v>
+      </c>
+      <c r="N50">
+        <v>0.96</v>
+      </c>
+      <c r="O50" s="4">
+        <f>N50*0.95</f>
+        <v>0.91199999999999992</v>
+      </c>
+      <c r="P50" s="4">
+        <f>O50*1.05</f>
+        <v>0.95760000000000001</v>
+      </c>
+      <c r="Q50">
+        <v>0.71</v>
+      </c>
+      <c r="R50" s="4">
+        <f>Q50*0.95</f>
+        <v>0.67449999999999999</v>
+      </c>
+      <c r="S50" s="4">
+        <f>R50*1.05</f>
+        <v>0.70822499999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>118</v>
+      </c>
+      <c r="B51" t="s">
+        <v>74</v>
+      </c>
+      <c r="E51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F51" s="16">
+        <v>0.69</v>
+      </c>
+      <c r="G51" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="H51" s="9">
+        <f>1-F51-G51-I51</f>
+        <v>0.21000000000000008</v>
+      </c>
+      <c r="I51" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="J51" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K51" s="10">
+        <v>0.83</v>
+      </c>
+      <c r="L51" s="10">
+        <f>K51*0.95</f>
+        <v>0.78849999999999998</v>
+      </c>
+      <c r="M51" s="10">
+        <f>K51*1.05</f>
+        <v>0.87149999999999994</v>
+      </c>
+      <c r="N51" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O51" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P51" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q51" s="10">
+        <f>81.7/100</f>
+        <v>0.81700000000000006</v>
+      </c>
+      <c r="R51" s="10">
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="S51" s="10">
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A52" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="B52" t="s">
+        <v>74</v>
+      </c>
+      <c r="E52" t="s">
+        <v>69</v>
+      </c>
+      <c r="F52" s="5">
+        <v>0</v>
+      </c>
+      <c r="G52" s="5">
+        <v>1</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52" s="5">
+        <v>0</v>
+      </c>
+      <c r="J52" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K52" s="9">
+        <v>0</v>
+      </c>
+      <c r="L52" s="9">
+        <v>0</v>
+      </c>
+      <c r="M52" s="9">
+        <v>0</v>
+      </c>
+      <c r="N52" s="9">
+        <v>0.96</v>
+      </c>
+      <c r="O52">
+        <f>N52*0.95</f>
+        <v>0.91199999999999992</v>
+      </c>
+      <c r="P52">
+        <f>N52*1.05</f>
+        <v>1.008</v>
+      </c>
+      <c r="Q52" s="9">
+        <v>0</v>
+      </c>
+      <c r="R52" s="9">
+        <v>0</v>
+      </c>
+      <c r="S52" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A53" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B53" t="s">
+        <v>73</v>
+      </c>
+      <c r="E53" t="s">
+        <v>69</v>
+      </c>
+      <c r="F53" s="18">
+        <v>0.224</v>
+      </c>
+      <c r="G53" s="5">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="H53" s="18">
+        <f>1-I53-F53-G53</f>
+        <v>0.61</v>
+      </c>
+      <c r="I53" s="5">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="J53" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K53" s="18">
+        <v>0.70899999999999996</v>
+      </c>
+      <c r="N53">
+        <v>0.96</v>
+      </c>
+      <c r="Q53" s="18">
+        <v>0.55500000000000005</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>120</v>
+      </c>
+      <c r="B54" t="s">
+        <v>73</v>
+      </c>
+      <c r="E54" t="s">
+        <v>69</v>
+      </c>
+      <c r="F54">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="G54" s="5">
+        <v>0.13200000000000001</v>
+      </c>
+      <c r="H54" s="9">
+        <f>1-F54-G54-I54</f>
+        <v>0.65700000000000003</v>
+      </c>
+      <c r="I54" s="5">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="J54" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K54" s="9">
+        <v>0.79500000000000004</v>
+      </c>
+      <c r="N54">
+        <v>0.96</v>
+      </c>
+      <c r="Q54" s="18">
+        <v>0.83699999999999997</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>121</v>
+      </c>
+      <c r="B55" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" t="s">
+        <v>69</v>
+      </c>
+      <c r="F55">
+        <v>0.17299999999999999</v>
+      </c>
+      <c r="G55" s="5">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="H55" s="9">
+        <f>1-F55-G55-I55</f>
+        <v>0.73299999999999987</v>
+      </c>
+      <c r="I55" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="J55" s="9">
+        <f t="shared" si="0"/>
+        <v>0.99999999999999989</v>
+      </c>
+      <c r="K55" s="9">
+        <v>0.64900000000000002</v>
+      </c>
+      <c r="N55">
+        <v>0.96</v>
+      </c>
+      <c r="Q55">
+        <v>0.57099999999999995</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S47" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S49">
-      <sortCondition ref="A1:A47"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:S55" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}"/>
   <conditionalFormatting sqref="K2:S38">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K48:S49">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K51:S51">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L50:M50">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O50:P50">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R50:S50">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4572,7 +4983,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA17DA89-E85F-4597-B94B-473613FC79D7}">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
@@ -4999,6 +5410,46 @@
       </c>
       <c r="B43" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>122</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>121</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -5016,6 +5467,9 @@
     <hyperlink ref="C19" r:id="rId6" display="https://www.feedipedia.org/node/11574" xr:uid="{9C3D8932-B7C3-4F23-B5AF-0CCF9B1CF004}"/>
     <hyperlink ref="C13" r:id="rId7" xr:uid="{731F2494-EBD0-4189-90DD-144FE15605E0}"/>
     <hyperlink ref="C14" r:id="rId8" display="https://www.feedipedia.org/node/11687" xr:uid="{0ABC761E-265E-4D42-A75F-0D6FCBFE9A86}"/>
+    <hyperlink ref="C46" r:id="rId9" display="https://www.feedipedia.org/node/46" xr:uid="{5AEB9992-3974-4C33-AF56-94BD939A9DFA}"/>
+    <hyperlink ref="C47" r:id="rId10" display="https://www.feedipedia.org/node/750" xr:uid="{FBED61B3-6D1C-4C1F-9A17-05EB5A4A4C2D}"/>
+    <hyperlink ref="C48" r:id="rId11" display="https://www.feedipedia.org/node/726" xr:uid="{1002B60E-2DED-4A45-AD21-8B1B21F8BC84}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Feed and ingredient updates
</commit_message>
<xml_diff>
--- a/data/raw_data/all_ingredients.xlsx
+++ b/data/raw_data/all_ingredients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0160536-06D3-4C16-AF8C-A63E1AB01DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C327E6-543D-4280-AD9C-F2194997EFE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
+    <workbookView xWindow="828" yWindow="840" windowWidth="21900" windowHeight="13908" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="all_ingredients" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="trash fish table" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sources!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="128">
   <si>
     <t>ingredient</t>
   </si>
@@ -420,6 +420,9 @@
   </si>
   <si>
     <t>Wheat bran | Feedipedia</t>
+  </si>
+  <si>
+    <t>cellulose</t>
   </si>
 </sst>
 </file>
@@ -956,7 +959,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -978,6 +981,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="45">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1026,37 +1030,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1447,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-  <dimension ref="A1:S55"/>
+  <dimension ref="A1:S56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.21875" bestFit="1" customWidth="1"/>
@@ -1548,7 +1522,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="9">
-        <f t="shared" ref="J2:J55" si="0">SUM(F2:I2)</f>
+        <f t="shared" ref="J2:J56" si="0">SUM(F2:I2)</f>
         <v>1</v>
       </c>
       <c r="K2" s="5">
@@ -1577,11 +1551,11 @@
         <v>0</v>
       </c>
       <c r="R2" s="7">
-        <f t="shared" ref="R2:R12" si="1">Q2*0.95</f>
+        <f t="shared" ref="R2:R13" si="1">Q2*0.95</f>
         <v>0</v>
       </c>
       <c r="S2" s="7">
-        <f t="shared" ref="S2:S12" si="2">R2*1.05</f>
+        <f t="shared" ref="S2:S13" si="2">R2*1.05</f>
         <v>0</v>
       </c>
     </row>
@@ -1819,7 +1793,7 @@
         <v>0.95176181599999998</v>
       </c>
       <c r="O6" s="5">
-        <f t="shared" ref="O6:O11" si="3">N6*0.95</f>
+        <f t="shared" ref="O6:O12" si="3">N6*0.95</f>
         <v>0.90417372519999994</v>
       </c>
       <c r="P6" s="5">
@@ -1904,76 +1878,60 @@
         <v>0.70970343749999976</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="8" spans="1:19" s="19" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="C8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="5">
-        <v>0.68</v>
-      </c>
-      <c r="G8" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H8" s="7">
-        <f>1-SUM(F8:G8,I8)</f>
-        <v>0.22999999999999998</v>
-      </c>
-      <c r="I8" s="5">
-        <v>0.02</v>
-      </c>
-      <c r="J8" s="5">
+      <c r="F8" s="8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8">
+        <v>1</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K8" s="5">
-        <v>0.94</v>
-      </c>
-      <c r="L8" s="10">
-        <f>K8*0.95</f>
-        <v>0.8929999999999999</v>
-      </c>
-      <c r="M8" s="10">
-        <f>L8*1.05</f>
-        <v>0.93764999999999998</v>
-      </c>
-      <c r="N8" s="5">
-        <v>0.93</v>
-      </c>
-      <c r="O8" s="5">
-        <f t="shared" si="3"/>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P8" s="5">
-        <f>MIN(N8*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q8" s="5">
-        <v>0.83</v>
-      </c>
-      <c r="R8" s="7">
-        <f t="shared" si="1"/>
-        <v>0.78849999999999998</v>
-      </c>
-      <c r="S8" s="7">
-        <f t="shared" si="2"/>
-        <v>0.82792500000000002</v>
+      <c r="K8" s="8">
+        <v>0</v>
+      </c>
+      <c r="L8" s="8">
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <v>0</v>
+      </c>
+      <c r="N8" s="8">
+        <v>0</v>
+      </c>
+      <c r="O8" s="8">
+        <v>0</v>
+      </c>
+      <c r="P8" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>0</v>
+      </c>
+      <c r="R8" s="8">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
         <v>73</v>
@@ -2040,7 +1998,7 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B10" t="s">
         <v>73</v>
@@ -2049,199 +2007,201 @@
         <v>68</v>
       </c>
       <c r="D10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="11">
-        <v>0.84</v>
-      </c>
-      <c r="G10" s="11">
-        <v>0.05</v>
-      </c>
-      <c r="H10" s="11">
+      <c r="F10" s="5">
+        <v>0.68</v>
+      </c>
+      <c r="G10" s="5">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I10" s="11">
-        <v>0.04</v>
-      </c>
-      <c r="J10" s="12">
+      <c r="H10" s="7">
+        <f>1-SUM(F10:G10,I10)</f>
+        <v>0.22999999999999998</v>
+      </c>
+      <c r="I10" s="5">
+        <v>0.02</v>
+      </c>
+      <c r="J10" s="5">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K10" s="11">
+      <c r="K10" s="5">
+        <v>0.94</v>
+      </c>
+      <c r="L10" s="10">
+        <f>K10*0.95</f>
+        <v>0.8929999999999999</v>
+      </c>
+      <c r="M10" s="10">
+        <f>L10*1.05</f>
+        <v>0.93764999999999998</v>
+      </c>
+      <c r="N10" s="5">
+        <v>0.93</v>
+      </c>
+      <c r="O10" s="5">
+        <f t="shared" si="3"/>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P10" s="5">
+        <f>MIN(N10*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>0.83</v>
+      </c>
+      <c r="R10" s="7">
+        <f t="shared" si="1"/>
+        <v>0.78849999999999998</v>
+      </c>
+      <c r="S10" s="7">
+        <f t="shared" si="2"/>
+        <v>0.82792500000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="11">
+        <v>0.84</v>
+      </c>
+      <c r="G11" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="H11" s="11">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I11" s="11">
+        <v>0.04</v>
+      </c>
+      <c r="J11" s="12">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K11" s="11">
         <v>0.88</v>
       </c>
-      <c r="L10" s="11">
-        <f>K10*0.94</f>
+      <c r="L11" s="11">
+        <f>K11*0.94</f>
         <v>0.82719999999999994</v>
       </c>
-      <c r="M10" s="11">
-        <f>L10*1.06</f>
+      <c r="M11" s="11">
+        <f>L11*1.06</f>
         <v>0.87683199999999994</v>
       </c>
-      <c r="N10" s="11">
+      <c r="N11" s="11">
         <v>0.95176181599999998</v>
       </c>
-      <c r="O10" s="11">
+      <c r="O11" s="11">
         <f t="shared" si="3"/>
         <v>0.90417372519999994</v>
       </c>
-      <c r="P10" s="11">
-        <f>N10*1.05</f>
+      <c r="P11" s="11">
+        <f>N11*1.05</f>
         <v>0.99934990680000002</v>
       </c>
-      <c r="Q10" s="11">
+      <c r="Q11" s="11">
         <v>0.77</v>
       </c>
-      <c r="R10" s="11">
+      <c r="R11" s="11">
         <f t="shared" si="1"/>
         <v>0.73149999999999993</v>
       </c>
-      <c r="S10" s="11">
+      <c r="S11" s="11">
         <f t="shared" si="2"/>
         <v>0.76807499999999995</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C11" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" t="s">
-        <v>69</v>
-      </c>
-      <c r="E11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F11">
-        <v>0.3</v>
-      </c>
-      <c r="G11">
-        <v>0.02</v>
-      </c>
-      <c r="H11" s="7">
-        <f>1-SUM(F11:G11,I11)</f>
-        <v>0.64</v>
-      </c>
-      <c r="I11">
-        <v>0.04</v>
-      </c>
-      <c r="J11" s="9">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="K11">
-        <v>0.86</v>
-      </c>
-      <c r="L11" s="4">
-        <f>K11*0.95</f>
-        <v>0.81699999999999995</v>
-      </c>
-      <c r="M11" s="4">
-        <f>L11*1.05</f>
-        <v>0.85785</v>
-      </c>
-      <c r="N11">
-        <v>0.93</v>
-      </c>
-      <c r="O11">
-        <f t="shared" si="3"/>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P11">
-        <f>MIN(N11*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q11">
-        <v>0.6</v>
-      </c>
-      <c r="R11" s="4">
-        <f t="shared" si="1"/>
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="S11" s="4">
-        <f t="shared" si="2"/>
-        <v>0.59849999999999992</v>
-      </c>
-    </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0.86849038461538397</v>
-      </c>
-      <c r="G12" s="6">
-        <f>6.7799419/100</f>
-        <v>6.7799419E-2</v>
+        <v>69</v>
+      </c>
+      <c r="F12">
+        <v>0.3</v>
+      </c>
+      <c r="G12">
+        <v>0.02</v>
       </c>
       <c r="H12" s="7">
         <f>1-SUM(F12:G12,I12)</f>
-        <v>1.3710196384616014E-2</v>
-      </c>
-      <c r="I12" s="5">
-        <f>5/100</f>
-        <v>0.05</v>
+        <v>0.64</v>
+      </c>
+      <c r="I12">
+        <v>0.04</v>
       </c>
       <c r="J12" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K12" s="6">
-        <v>0.86599999999999999</v>
-      </c>
-      <c r="L12" s="6">
-        <v>0.75829999999999997</v>
-      </c>
-      <c r="M12" s="6">
-        <v>0.94739999999999991</v>
-      </c>
-      <c r="N12" s="6">
-        <v>0.93709999999999993</v>
-      </c>
-      <c r="O12" s="6">
-        <v>0.87280000000000002</v>
-      </c>
-      <c r="P12" s="6">
-        <v>0.97950000000000004</v>
-      </c>
-      <c r="Q12" s="5">
-        <v>0.78</v>
-      </c>
-      <c r="R12" s="7">
+      <c r="K12">
+        <v>0.86</v>
+      </c>
+      <c r="L12" s="4">
+        <f>K12*0.95</f>
+        <v>0.81699999999999995</v>
+      </c>
+      <c r="M12" s="4">
+        <f>L12*1.05</f>
+        <v>0.85785</v>
+      </c>
+      <c r="N12">
+        <v>0.93</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="3"/>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P12">
+        <f>MIN(N12*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q12">
+        <v>0.6</v>
+      </c>
+      <c r="R12" s="4">
         <f t="shared" si="1"/>
-        <v>0.74099999999999999</v>
-      </c>
-      <c r="S12" s="7">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="S12" s="4">
         <f t="shared" si="2"/>
-        <v>0.77805000000000002</v>
+        <v>0.59849999999999992</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
         <v>68</v>
@@ -2253,57 +2213,57 @@
         <v>68</v>
       </c>
       <c r="F13" s="6">
-        <v>0.73424999999999996</v>
+        <v>0.86849038461538397</v>
       </c>
       <c r="G13" s="6">
-        <v>8.3000000000000004E-2</v>
+        <f>6.7799419/100</f>
+        <v>6.7799419E-2</v>
       </c>
       <c r="H13" s="7">
         <f>1-SUM(F13:G13,I13)</f>
-        <v>4.3750000000000067E-2</v>
+        <v>1.3710196384616014E-2</v>
       </c>
       <c r="I13" s="5">
-        <f>13.9/100</f>
-        <v>0.13900000000000001</v>
+        <f>5/100</f>
+        <v>0.05</v>
       </c>
       <c r="J13" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K13" s="6">
-        <v>0.87980000000000003</v>
+        <v>0.86599999999999999</v>
       </c>
       <c r="L13" s="6">
-        <v>0.82969999999999999</v>
+        <v>0.75829999999999997</v>
       </c>
       <c r="M13" s="6">
-        <v>0.92209999999999992</v>
+        <v>0.94739999999999991</v>
       </c>
       <c r="N13" s="6">
-        <v>0.95669999999999999</v>
+        <v>0.93709999999999993</v>
       </c>
       <c r="O13" s="6">
-        <v>0.8993000000000001</v>
+        <v>0.87280000000000002</v>
       </c>
       <c r="P13" s="6">
-        <v>0.99199999999999999</v>
+        <v>0.97950000000000004</v>
       </c>
       <c r="Q13" s="5">
-        <f>83.3/100</f>
-        <v>0.83299999999999996</v>
-      </c>
-      <c r="R13" s="5">
-        <f>74.5/100</f>
-        <v>0.745</v>
-      </c>
-      <c r="S13" s="5">
-        <f>92.6/100</f>
-        <v>0.92599999999999993</v>
+        <v>0.78</v>
+      </c>
+      <c r="R13" s="7">
+        <f t="shared" si="1"/>
+        <v>0.74099999999999999</v>
+      </c>
+      <c r="S13" s="7">
+        <f t="shared" si="2"/>
+        <v>0.77805000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
         <v>74</v>
@@ -2354,21 +2314,21 @@
         <v>0.99199999999999999</v>
       </c>
       <c r="Q14" s="5">
-        <f>81.7/100</f>
-        <v>0.81700000000000006</v>
+        <f>83.3/100</f>
+        <v>0.83299999999999996</v>
       </c>
       <c r="R14" s="5">
-        <f>71.8/100</f>
-        <v>0.71799999999999997</v>
+        <f>74.5/100</f>
+        <v>0.745</v>
       </c>
       <c r="S14" s="5">
-        <f>91.6/100</f>
-        <v>0.91599999999999993</v>
+        <f>92.6/100</f>
+        <v>0.92599999999999993</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
@@ -2380,34 +2340,34 @@
         <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" s="5">
-        <v>0</v>
-      </c>
-      <c r="G15" s="5">
-        <v>1</v>
-      </c>
-      <c r="H15" s="5">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0.73424999999999996</v>
+      </c>
+      <c r="G15" s="6">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="H15" s="7">
+        <f>1-SUM(F15:G15,I15)</f>
+        <v>4.3750000000000067E-2</v>
       </c>
       <c r="I15" s="5">
-        <v>0</v>
+        <f>13.9/100</f>
+        <v>0.13900000000000001</v>
       </c>
       <c r="J15" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K15" s="5">
-        <v>0</v>
-      </c>
-      <c r="L15" s="5">
-        <f>K15*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="5">
-        <f>L15*1.05</f>
-        <v>0</v>
+      <c r="K15" s="6">
+        <v>0.87980000000000003</v>
+      </c>
+      <c r="L15" s="6">
+        <v>0.82969999999999999</v>
+      </c>
+      <c r="M15" s="6">
+        <v>0.92209999999999992</v>
       </c>
       <c r="N15" s="6">
         <v>0.95669999999999999</v>
@@ -2419,20 +2379,21 @@
         <v>0.99199999999999999</v>
       </c>
       <c r="Q15" s="5">
-        <v>0</v>
-      </c>
-      <c r="R15" s="7">
-        <f>Q15*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="7">
-        <f>R15*1.05</f>
-        <v>0</v>
+        <f>81.7/100</f>
+        <v>0.81700000000000006</v>
+      </c>
+      <c r="R15" s="5">
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="S15" s="5">
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
         <v>74</v>
@@ -2496,16 +2457,16 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C17" t="s">
         <v>68</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
         <v>69</v>
@@ -2514,13 +2475,13 @@
         <v>0</v>
       </c>
       <c r="G17" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="5">
         <v>0</v>
       </c>
       <c r="I17" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" s="9">
         <f t="shared" si="0"/>
@@ -2530,33 +2491,37 @@
         <v>0</v>
       </c>
       <c r="L17" s="5">
+        <f>K17*0.95</f>
         <v>0</v>
       </c>
       <c r="M17" s="5">
-        <v>0</v>
-      </c>
-      <c r="N17" s="5">
-        <v>0</v>
-      </c>
-      <c r="O17" s="5">
-        <v>0</v>
-      </c>
-      <c r="P17" s="5">
-        <v>0</v>
+        <f>L17*1.05</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="6">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O17" s="6">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0.99199999999999999</v>
       </c>
       <c r="Q17" s="5">
         <v>0</v>
       </c>
-      <c r="R17" s="5">
-        <v>0</v>
-      </c>
-      <c r="S17" s="5">
+      <c r="R17" s="7">
+        <f>Q17*0.95</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="7">
+        <f>R17*1.05</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
         <v>73</v>
@@ -2565,197 +2530,190 @@
         <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
         <v>69</v>
       </c>
       <c r="F18" s="5">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="G18" s="5">
-        <v>5.2999999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="H18" s="5">
-        <v>0.46899999999999997</v>
+        <v>0</v>
       </c>
       <c r="I18" s="5">
-        <v>5.8000000000000003E-2</v>
+        <v>1</v>
       </c>
       <c r="J18" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K18" s="5">
-        <v>0.63000000000000012</v>
-      </c>
-      <c r="L18" s="10">
-        <f>K18*0.95</f>
-        <v>0.59850000000000003</v>
-      </c>
-      <c r="M18" s="10">
-        <f>L18*1.05</f>
-        <v>0.62842500000000001</v>
+        <v>0</v>
+      </c>
+      <c r="L18" s="5">
+        <v>0</v>
+      </c>
+      <c r="M18" s="5">
+        <v>0</v>
       </c>
       <c r="N18" s="5">
-        <v>0.95176181599999998</v>
+        <v>0</v>
       </c>
       <c r="O18" s="5">
-        <f>N18*0.95</f>
-        <v>0.90417372519999994</v>
+        <v>0</v>
       </c>
       <c r="P18" s="5">
-        <f>N18*1.05</f>
-        <v>0.99934990680000002</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="5">
-        <v>0.71</v>
-      </c>
-      <c r="R18" s="7">
-        <f>Q18*0.95</f>
-        <v>0.67449999999999999</v>
-      </c>
-      <c r="S18" s="7">
-        <f>R18*1.05</f>
-        <v>0.70822499999999999</v>
+        <v>0</v>
+      </c>
+      <c r="R18" s="5">
+        <v>0</v>
+      </c>
+      <c r="S18" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
         <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E19" t="s">
         <v>69</v>
       </c>
-      <c r="F19">
-        <v>0.55800000000000005</v>
-      </c>
-      <c r="G19">
-        <v>4.7E-2</v>
-      </c>
-      <c r="H19">
-        <v>0.34100000000000003</v>
-      </c>
-      <c r="I19">
-        <v>5.3999999999999999E-2</v>
+      <c r="F19" s="5">
+        <v>0.42</v>
+      </c>
+      <c r="G19" s="5">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="H19" s="5">
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="I19" s="5">
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" si="0"/>
-        <v>1.0000000000000002</v>
-      </c>
-      <c r="K19">
+        <v>1</v>
+      </c>
+      <c r="K19" s="5">
         <v>0.63000000000000012</v>
       </c>
-      <c r="L19" s="4">
+      <c r="L19" s="10">
         <f>K19*0.95</f>
         <v>0.59850000000000003</v>
       </c>
-      <c r="M19" s="4">
+      <c r="M19" s="10">
         <f>L19*1.05</f>
         <v>0.62842500000000001</v>
       </c>
-      <c r="N19">
-        <v>0.93</v>
-      </c>
-      <c r="O19">
+      <c r="N19" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O19" s="5">
         <f>N19*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P19">
-        <f>MIN(N19*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q19">
-        <v>0.65000000000000013</v>
-      </c>
-      <c r="R19" s="4">
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P19" s="5">
+        <f>N19*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q19" s="5">
+        <v>0.71</v>
+      </c>
+      <c r="R19" s="7">
         <f>Q19*0.95</f>
-        <v>0.61750000000000005</v>
-      </c>
-      <c r="S19" s="4">
+        <v>0.67449999999999999</v>
+      </c>
+      <c r="S19" s="7">
         <f>R19*1.05</f>
-        <v>0.64837500000000003</v>
+        <v>0.70822499999999999</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E20" t="s">
         <v>69</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="G20">
+        <v>4.7E-2</v>
+      </c>
+      <c r="H20">
+        <v>0.34100000000000003</v>
+      </c>
+      <c r="I20">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="J20" s="9">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="K20">
+        <v>0.63000000000000012</v>
+      </c>
+      <c r="L20" s="4">
+        <f>K20*0.95</f>
+        <v>0.59850000000000003</v>
+      </c>
+      <c r="M20" s="4">
+        <f>L20*1.05</f>
+        <v>0.62842500000000001</v>
+      </c>
+      <c r="N20">
         <v>0.93</v>
       </c>
-      <c r="G20" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="H20" s="7">
-        <f>1-SUM(F20:G20,I20)</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="5">
-        <v>0</v>
-      </c>
-      <c r="J20" s="9">
-        <f t="shared" ref="J20" si="4">SUM(F20:I20)</f>
-        <v>1</v>
-      </c>
-      <c r="K20" s="5">
-        <v>0.622</v>
-      </c>
-      <c r="L20" s="10">
-        <f>K20*0.94</f>
-        <v>0.58467999999999998</v>
-      </c>
-      <c r="M20" s="10">
-        <f>L20*1.06</f>
-        <v>0.6197608</v>
-      </c>
-      <c r="N20" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O20" s="5">
+      <c r="O20">
         <f>N20*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P20" s="5">
-        <f>N20*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q20" s="5">
-        <v>0.60399999999999998</v>
-      </c>
-      <c r="R20" s="7">
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P20">
+        <f>MIN(N20*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q20">
+        <v>0.65000000000000013</v>
+      </c>
+      <c r="R20" s="4">
         <f>Q20*0.95</f>
-        <v>0.57379999999999998</v>
-      </c>
-      <c r="S20" s="7">
+        <v>0.61750000000000005</v>
+      </c>
+      <c r="S20" s="4">
         <f>R20*1.05</f>
-        <v>0.60248999999999997</v>
+        <v>0.64837500000000003</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>49</v>
+        <v>115</v>
       </c>
       <c r="B21" t="s">
         <v>75</v>
@@ -2783,7 +2741,7 @@
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J21" si="4">SUM(F21:I21)</f>
         <v>1</v>
       </c>
       <c r="K21" s="5">
@@ -2822,273 +2780,268 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" t="s">
         <v>69</v>
       </c>
-      <c r="D22" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" t="s">
-        <v>68</v>
-      </c>
-      <c r="F22" s="6">
-        <v>0.58399999999999996</v>
-      </c>
-      <c r="G22" s="6">
-        <v>0.17899999999999999</v>
+      <c r="F22" s="5">
+        <v>0.93</v>
+      </c>
+      <c r="G22" s="5">
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H22" s="7">
         <f>1-SUM(F22:G22,I22)</f>
-        <v>0.1070000000000001</v>
+        <v>0</v>
       </c>
       <c r="I22" s="5">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="J22" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K22" s="6">
-        <v>0.88470000000000004</v>
-      </c>
-      <c r="L22" s="6">
-        <v>0.84920000000000007</v>
-      </c>
-      <c r="M22" s="6">
-        <v>0.93629999999999991</v>
-      </c>
-      <c r="N22" s="6">
-        <v>0.9466</v>
-      </c>
-      <c r="O22" s="6">
-        <v>0.91510000000000002</v>
-      </c>
-      <c r="P22" s="6">
-        <v>0.97360000000000002</v>
+      <c r="K22" s="5">
+        <v>0.622</v>
+      </c>
+      <c r="L22" s="10">
+        <f>K22*0.94</f>
+        <v>0.58467999999999998</v>
+      </c>
+      <c r="M22" s="10">
+        <f>L22*1.06</f>
+        <v>0.6197608</v>
+      </c>
+      <c r="N22" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O22" s="5">
+        <f>N22*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P22" s="5">
+        <f>N22*1.05</f>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q22" s="5">
-        <v>0.41000000000000003</v>
+        <v>0.60399999999999998</v>
       </c>
       <c r="R22" s="7">
         <f>Q22*0.95</f>
-        <v>0.38950000000000001</v>
+        <v>0.57379999999999998</v>
       </c>
       <c r="S22" s="7">
         <f>R22*1.05</f>
-        <v>0.40897500000000003</v>
+        <v>0.60248999999999997</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D23" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E23" t="s">
         <v>68</v>
       </c>
       <c r="F23" s="6">
-        <v>0.55099999999999993</v>
+        <v>0.58399999999999996</v>
       </c>
       <c r="G23" s="6">
-        <f>26.92252/100</f>
-        <v>0.2692252</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="H23" s="7">
         <f>1-SUM(F23:G23,I23)</f>
-        <v>4.08748000000001E-2</v>
+        <v>0.1070000000000001</v>
       </c>
       <c r="I23" s="5">
-        <f>13.89/100</f>
-        <v>0.1389</v>
+        <v>0.13</v>
       </c>
       <c r="J23" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K23" s="6">
-        <v>0.87769999999999992</v>
+        <v>0.88470000000000004</v>
       </c>
       <c r="L23" s="6">
-        <v>0.86930000000000007</v>
+        <v>0.84920000000000007</v>
       </c>
       <c r="M23" s="6">
-        <v>0.88549999999999995</v>
+        <v>0.93629999999999991</v>
       </c>
       <c r="N23" s="6">
-        <v>0.95109999999999995</v>
+        <v>0.9466</v>
       </c>
       <c r="O23" s="6">
-        <v>0.93889999999999996</v>
+        <v>0.91510000000000002</v>
       </c>
       <c r="P23" s="6">
-        <v>0.95739999999999992</v>
+        <v>0.97360000000000002</v>
       </c>
       <c r="Q23" s="5">
-        <v>0.59399999999999997</v>
-      </c>
-      <c r="R23" s="5">
-        <f>Q23-3*(2.16/100)</f>
-        <v>0.5292</v>
-      </c>
-      <c r="S23" s="5">
-        <f>Q23+3*(2.16/100)</f>
-        <v>0.65879999999999994</v>
+        <v>0.41000000000000003</v>
+      </c>
+      <c r="R23" s="7">
+        <f>Q23*0.95</f>
+        <v>0.38950000000000001</v>
+      </c>
+      <c r="S23" s="7">
+        <f>R23*1.05</f>
+        <v>0.40897500000000003</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E24" t="s">
-        <v>69</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24">
-        <v>1</v>
-      </c>
-      <c r="H24">
-        <v>0</v>
-      </c>
-      <c r="I24">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F24" s="6">
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="G24" s="6">
+        <f>26.92252/100</f>
+        <v>0.2692252</v>
+      </c>
+      <c r="H24" s="7">
+        <f>1-SUM(F24:G24,I24)</f>
+        <v>4.08748000000001E-2</v>
+      </c>
+      <c r="I24" s="5">
+        <f>13.89/100</f>
+        <v>0.1389</v>
       </c>
       <c r="J24" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K24" s="4">
-        <v>0.84588505065844988</v>
-      </c>
-      <c r="L24" s="4">
-        <f>K24*0.95</f>
-        <v>0.80359079812552736</v>
-      </c>
-      <c r="M24" s="4">
-        <f>L24*1.05</f>
-        <v>0.84377033803180379</v>
-      </c>
-      <c r="N24">
-        <v>0.93</v>
-      </c>
-      <c r="O24">
-        <f>N24*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P24">
-        <f>MIN(N24*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q24" s="4">
-        <v>0.71148214285714262</v>
-      </c>
-      <c r="R24" s="4">
-        <f>Q24*0.95</f>
-        <v>0.67590803571428548</v>
-      </c>
-      <c r="S24" s="4">
-        <f>R24*1.05</f>
-        <v>0.70970343749999976</v>
+      <c r="K24" s="6">
+        <v>0.87769999999999992</v>
+      </c>
+      <c r="L24" s="6">
+        <v>0.86930000000000007</v>
+      </c>
+      <c r="M24" s="6">
+        <v>0.88549999999999995</v>
+      </c>
+      <c r="N24" s="6">
+        <v>0.95109999999999995</v>
+      </c>
+      <c r="O24" s="6">
+        <v>0.93889999999999996</v>
+      </c>
+      <c r="P24" s="6">
+        <v>0.95739999999999992</v>
+      </c>
+      <c r="Q24" s="5">
+        <v>0.59399999999999997</v>
+      </c>
+      <c r="R24" s="5">
+        <f>Q24-3*(2.16/100)</f>
+        <v>0.5292</v>
+      </c>
+      <c r="S24" s="5">
+        <f>Q24+3*(2.16/100)</f>
+        <v>0.65879999999999994</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
         <v>73</v>
       </c>
       <c r="C25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E25" t="s">
         <v>69</v>
       </c>
-      <c r="F25" s="5">
-        <f>AVERAGE(420.2,405.3,420.2,403.8,390.7,468.4)/1000</f>
-        <v>0.41809999999999997</v>
-      </c>
-      <c r="G25" s="5">
-        <f>AVERAGE(175.4,153.9,171.8,132.3,106.7,100.1)/1000</f>
-        <v>0.14003333333333337</v>
-      </c>
-      <c r="H25" s="7">
-        <f>1-SUM(F25:G25,I25)</f>
-        <v>0.41068333333333329</v>
-      </c>
-      <c r="I25" s="5">
-        <f>AVERAGE(28.6,37.6,28,37.3,25.9,29.7)/1000</f>
-        <v>3.1183333333333334E-2</v>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
       </c>
       <c r="J25" s="9">
-        <f t="shared" ref="J25" si="5">SUM(F25:I25)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K25" s="5">
-        <f>AVERAGE(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
-        <v>0.89050000000000007</v>
-      </c>
-      <c r="L25" s="5">
-        <f>MIN(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
-        <v>0.879</v>
-      </c>
-      <c r="M25" s="5">
-        <f>MAX(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
-        <v>0.90099999999999991</v>
-      </c>
-      <c r="N25" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O25" s="5">
+      <c r="K25" s="4">
+        <v>0.84588505065844988</v>
+      </c>
+      <c r="L25" s="4">
+        <f>K25*0.95</f>
+        <v>0.80359079812552736</v>
+      </c>
+      <c r="M25" s="4">
+        <f>L25*1.05</f>
+        <v>0.84377033803180379</v>
+      </c>
+      <c r="N25">
+        <v>0.93</v>
+      </c>
+      <c r="O25">
         <f>N25*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P25" s="5">
-        <f>N25*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q25" s="5">
-        <f>AVERAGE(79.7,80.2,80,80,81.2,77.4)/100</f>
-        <v>0.79749999999999999</v>
-      </c>
-      <c r="R25" s="5">
-        <f>MIN(79.7,80.2,80,80,81.2,77.4)/100</f>
-        <v>0.77400000000000002</v>
-      </c>
-      <c r="S25" s="5">
-        <f>MAX(79.7,80.2,80,80,81.2,77.4)/100</f>
-        <v>0.81200000000000006</v>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P25">
+        <f>MIN(N25*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q25" s="4">
+        <v>0.71148214285714262</v>
+      </c>
+      <c r="R25" s="4">
+        <f>Q25*0.95</f>
+        <v>0.67590803571428548</v>
+      </c>
+      <c r="S25" s="4">
+        <f>R25*1.05</f>
+        <v>0.70970343749999976</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="B26" t="s">
         <v>73</v>
@@ -3119,7 +3072,7 @@
         <v>3.1183333333333334E-2</v>
       </c>
       <c r="J26" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J26" si="5">SUM(F26:I26)</f>
         <v>1</v>
       </c>
       <c r="K26" s="5">
@@ -3160,10 +3113,10 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>88</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C27" t="s">
         <v>68</v>
@@ -3172,65 +3125,73 @@
         <v>68</v>
       </c>
       <c r="E27" t="s">
-        <v>68</v>
-      </c>
-      <c r="F27" s="6">
-        <v>0.53783333333333327</v>
-      </c>
-      <c r="G27" s="6">
-        <f>13.249433/100</f>
-        <v>0.13249432999999999</v>
+        <v>69</v>
+      </c>
+      <c r="F27" s="5">
+        <f>AVERAGE(420.2,405.3,420.2,403.8,390.7,468.4)/1000</f>
+        <v>0.41809999999999997</v>
+      </c>
+      <c r="G27" s="5">
+        <f>AVERAGE(175.4,153.9,171.8,132.3,106.7,100.1)/1000</f>
+        <v>0.14003333333333337</v>
       </c>
       <c r="H27" s="7">
         <f>1-SUM(F27:G27,I27)</f>
-        <v>2.4672336666666794E-2</v>
+        <v>0.41068333333333329</v>
       </c>
       <c r="I27" s="5">
-        <v>0.30499999999999999</v>
+        <f>AVERAGE(28.6,37.6,28,37.3,25.9,29.7)/1000</f>
+        <v>3.1183333333333334E-2</v>
       </c>
       <c r="J27" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K27" s="6">
-        <v>0.83030000000000004</v>
-      </c>
-      <c r="L27" s="6">
-        <v>0.72499999999999998</v>
-      </c>
-      <c r="M27" s="6">
-        <v>0.9194</v>
-      </c>
-      <c r="N27" s="6">
-        <v>0.93189999999999995</v>
-      </c>
-      <c r="O27" s="6">
-        <v>0.86629999999999996</v>
-      </c>
-      <c r="P27" s="6">
-        <v>0.96779999999999999</v>
+      <c r="K27" s="5">
+        <f>AVERAGE(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.89050000000000007</v>
+      </c>
+      <c r="L27" s="5">
+        <f>MIN(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.879</v>
+      </c>
+      <c r="M27" s="5">
+        <f>MAX(89.5,89.3,87.9,88.2,89.3,90.1)/100</f>
+        <v>0.90099999999999991</v>
+      </c>
+      <c r="N27" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O27" s="5">
+        <f>N27*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P27" s="5">
+        <f>N27*1.05</f>
+        <v>0.99934990680000002</v>
       </c>
       <c r="Q27" s="5">
-        <v>0.68700000000000006</v>
-      </c>
-      <c r="R27" s="10">
-        <f t="shared" ref="R27:R39" si="6">Q27*0.95</f>
-        <v>0.65265000000000006</v>
-      </c>
-      <c r="S27" s="10">
-        <f t="shared" ref="S27:S45" si="7">R27*1.05</f>
-        <v>0.68528250000000013</v>
+        <f>AVERAGE(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.79749999999999999</v>
+      </c>
+      <c r="R27" s="5">
+        <f>MIN(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="S27" s="5">
+        <f>MAX(79.7,80.2,80,80,81.2,77.4)/100</f>
+        <v>0.81200000000000006</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
         <v>75</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
         <v>68</v>
@@ -3239,377 +3200,375 @@
         <v>68</v>
       </c>
       <c r="F28" s="6">
-        <v>0.56188888888888899</v>
+        <v>0.53783333333333327</v>
       </c>
       <c r="G28" s="6">
-        <v>8.6999999999999994E-2</v>
+        <f>13.249433/100</f>
+        <v>0.13249432999999999</v>
       </c>
       <c r="H28" s="7">
         <f>1-SUM(F28:G28,I28)</f>
-        <v>0.23711111111111105</v>
-      </c>
-      <c r="I28" s="8">
-        <v>0.114</v>
+        <v>2.4672336666666794E-2</v>
+      </c>
+      <c r="I28" s="5">
+        <v>0.30499999999999999</v>
       </c>
       <c r="J28" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K28" s="6">
-        <v>0.81159999999999999</v>
+        <v>0.83030000000000004</v>
       </c>
       <c r="L28" s="6">
-        <v>0.70010000000000006</v>
+        <v>0.72499999999999998</v>
       </c>
       <c r="M28" s="6">
-        <v>0.93319999999999992</v>
+        <v>0.9194</v>
       </c>
       <c r="N28" s="6">
-        <v>0.95489999999999997</v>
+        <v>0.93189999999999995</v>
       </c>
       <c r="O28" s="6">
-        <v>0.90229999999999999</v>
+        <v>0.86629999999999996</v>
       </c>
       <c r="P28" s="6">
-        <v>0.98790000000000011</v>
+        <v>0.96779999999999999</v>
       </c>
       <c r="Q28" s="5">
         <v>0.68700000000000006</v>
       </c>
       <c r="R28" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="R28:R40" si="6">Q28*0.95</f>
         <v>0.65265000000000006</v>
       </c>
       <c r="S28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="S28:S46" si="7">R28*1.05</f>
         <v>0.68528250000000013</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>66</v>
+      </c>
+      <c r="B29" t="s">
+        <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D29" t="s">
         <v>68</v>
       </c>
       <c r="E29" t="s">
-        <v>69</v>
-      </c>
-      <c r="F29" s="5">
-        <v>0</v>
-      </c>
-      <c r="G29" s="5">
-        <v>0</v>
-      </c>
-      <c r="H29" s="5">
-        <v>0</v>
-      </c>
-      <c r="I29" s="5">
-        <v>1</v>
+        <v>68</v>
+      </c>
+      <c r="F29" s="6">
+        <v>0.56188888888888899</v>
+      </c>
+      <c r="G29" s="6">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="H29" s="7">
+        <f>1-SUM(F29:G29,I29)</f>
+        <v>0.23711111111111105</v>
+      </c>
+      <c r="I29" s="8">
+        <v>0.114</v>
       </c>
       <c r="J29" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K29" s="5">
-        <v>0</v>
-      </c>
-      <c r="L29" s="5">
-        <v>0</v>
-      </c>
-      <c r="M29" s="5">
-        <v>0</v>
-      </c>
-      <c r="N29" s="5">
-        <v>0</v>
-      </c>
-      <c r="O29" s="5">
-        <f>N29*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="P29" s="5">
-        <f>N29*1.05</f>
-        <v>0</v>
+      <c r="K29" s="6">
+        <v>0.81159999999999999</v>
+      </c>
+      <c r="L29" s="6">
+        <v>0.70010000000000006</v>
+      </c>
+      <c r="M29" s="6">
+        <v>0.93319999999999992</v>
+      </c>
+      <c r="N29" s="6">
+        <v>0.95489999999999997</v>
+      </c>
+      <c r="O29" s="6">
+        <v>0.90229999999999999</v>
+      </c>
+      <c r="P29" s="6">
+        <v>0.98790000000000011</v>
       </c>
       <c r="Q29" s="5">
-        <v>0</v>
+        <v>0.68700000000000006</v>
       </c>
       <c r="R29" s="10">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.65265000000000006</v>
       </c>
       <c r="S29" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.68528250000000013</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>18</v>
-      </c>
-      <c r="B30" t="s">
-        <v>75</v>
+        <v>17</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
         <v>68</v>
       </c>
       <c r="E30" t="s">
-        <v>68</v>
-      </c>
-      <c r="F30" s="6">
-        <v>0.62166666666666659</v>
-      </c>
-      <c r="G30" s="6">
-        <v>0.122</v>
-      </c>
-      <c r="H30" s="7">
-        <f>1-SUM(F30:G30,I30)</f>
-        <v>0.14233333333333342</v>
-      </c>
-      <c r="I30" s="8">
-        <v>0.114</v>
+        <v>69</v>
+      </c>
+      <c r="F30" s="5">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5">
+        <v>0</v>
+      </c>
+      <c r="H30" s="5">
+        <v>0</v>
+      </c>
+      <c r="I30" s="5">
+        <v>1</v>
       </c>
       <c r="J30" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K30" s="6">
-        <v>0.78639999999999999</v>
-      </c>
-      <c r="L30" s="6">
-        <v>0.71209999999999996</v>
-      </c>
-      <c r="M30" s="6">
-        <v>0.84200000000000008</v>
-      </c>
-      <c r="N30" s="6">
-        <v>0.9325</v>
-      </c>
-      <c r="O30" s="6">
-        <v>0.91139999999999999</v>
-      </c>
-      <c r="P30" s="6">
-        <v>0.94950000000000001</v>
+      <c r="K30" s="5">
+        <v>0</v>
+      </c>
+      <c r="L30" s="5">
+        <v>0</v>
+      </c>
+      <c r="M30" s="5">
+        <v>0</v>
+      </c>
+      <c r="N30" s="5">
+        <v>0</v>
+      </c>
+      <c r="O30" s="5">
+        <f>N30*0.95</f>
+        <v>0</v>
+      </c>
+      <c r="P30" s="5">
+        <f>N30*1.05</f>
+        <v>0</v>
       </c>
       <c r="Q30" s="5">
-        <v>0.68900000000000006</v>
+        <v>0</v>
       </c>
       <c r="R30" s="10">
         <f t="shared" si="6"/>
-        <v>0.65455000000000008</v>
+        <v>0</v>
       </c>
       <c r="S30" s="10">
         <f t="shared" si="7"/>
-        <v>0.6872775000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C31" t="s">
         <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E31" t="s">
-        <v>69</v>
-      </c>
-      <c r="F31">
-        <v>0.23</v>
-      </c>
-      <c r="G31">
-        <v>0.01</v>
-      </c>
-      <c r="H31">
-        <v>0.45</v>
-      </c>
-      <c r="I31">
-        <v>0.31</v>
+        <v>68</v>
+      </c>
+      <c r="F31" s="6">
+        <v>0.62166666666666659</v>
+      </c>
+      <c r="G31" s="6">
+        <v>0.122</v>
+      </c>
+      <c r="H31" s="7">
+        <f>1-SUM(F31:G31,I31)</f>
+        <v>0.14233333333333342</v>
+      </c>
+      <c r="I31" s="8">
+        <v>0.114</v>
       </c>
       <c r="J31" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K31">
-        <v>0.8</v>
-      </c>
-      <c r="L31" s="4">
-        <f>K31*0.95</f>
-        <v>0.76</v>
-      </c>
-      <c r="M31" s="4">
-        <f>L31*1.05</f>
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="N31">
-        <v>0.93</v>
-      </c>
-      <c r="O31">
-        <f>N31*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P31">
-        <f>MIN(N31*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q31">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="R31" s="4">
+      <c r="K31" s="6">
+        <v>0.78639999999999999</v>
+      </c>
+      <c r="L31" s="6">
+        <v>0.71209999999999996</v>
+      </c>
+      <c r="M31" s="6">
+        <v>0.84200000000000008</v>
+      </c>
+      <c r="N31" s="6">
+        <v>0.9325</v>
+      </c>
+      <c r="O31" s="6">
+        <v>0.91139999999999999</v>
+      </c>
+      <c r="P31" s="6">
+        <v>0.94950000000000001</v>
+      </c>
+      <c r="Q31" s="5">
+        <v>0.68900000000000006</v>
+      </c>
+      <c r="R31" s="10">
         <f t="shared" si="6"/>
-        <v>0.55099999999999993</v>
-      </c>
-      <c r="S31" s="4">
+        <v>0.65455000000000008</v>
+      </c>
+      <c r="S31" s="10">
         <f t="shared" si="7"/>
-        <v>0.57855000000000001</v>
+        <v>0.6872775000000001</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B32" t="s">
         <v>73</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E32" t="s">
         <v>69</v>
       </c>
-      <c r="F32" s="5">
-        <v>0.84</v>
-      </c>
-      <c r="G32" s="5">
-        <v>0.05</v>
-      </c>
-      <c r="H32" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="I32" s="5">
-        <v>0.04</v>
+      <c r="F32">
+        <v>0.23</v>
+      </c>
+      <c r="G32">
+        <v>0.01</v>
+      </c>
+      <c r="H32">
+        <v>0.45</v>
+      </c>
+      <c r="I32">
+        <v>0.31</v>
       </c>
       <c r="J32" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K32" s="5">
-        <v>0.88</v>
-      </c>
-      <c r="L32" s="10">
-        <f>K32*0.94</f>
-        <v>0.82719999999999994</v>
-      </c>
-      <c r="M32" s="10">
-        <f>L32*1.06</f>
-        <v>0.87683199999999994</v>
-      </c>
-      <c r="N32" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O32" s="5">
+      <c r="K32">
+        <v>0.8</v>
+      </c>
+      <c r="L32" s="4">
+        <f>K32*0.95</f>
+        <v>0.76</v>
+      </c>
+      <c r="M32" s="4">
+        <f>L32*1.05</f>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="N32">
+        <v>0.93</v>
+      </c>
+      <c r="O32">
         <f>N32*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P32" s="5">
-        <f>N32*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q32" s="5">
-        <v>0.77</v>
-      </c>
-      <c r="R32" s="10">
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P32">
+        <f>MIN(N32*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q32">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="R32" s="4">
         <f t="shared" si="6"/>
-        <v>0.73149999999999993</v>
-      </c>
-      <c r="S32" s="10">
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="S32" s="4">
         <f t="shared" si="7"/>
-        <v>0.76807499999999995</v>
+        <v>0.57855000000000001</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
         <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E33" t="s">
         <v>69</v>
       </c>
-      <c r="F33">
-        <v>0.23</v>
-      </c>
-      <c r="G33">
-        <v>0.01</v>
-      </c>
-      <c r="H33">
-        <v>0.45</v>
-      </c>
-      <c r="I33">
-        <v>0.31</v>
+      <c r="F33" s="5">
+        <v>0.84</v>
+      </c>
+      <c r="G33" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="H33" s="5">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I33" s="5">
+        <v>0.04</v>
       </c>
       <c r="J33" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K33">
-        <v>0.8</v>
-      </c>
-      <c r="L33" s="4">
-        <f>K33*0.95</f>
-        <v>0.76</v>
-      </c>
-      <c r="M33" s="4">
-        <f>L33*1.05</f>
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="N33">
-        <v>0.93</v>
-      </c>
-      <c r="O33">
+      <c r="K33" s="5">
+        <v>0.88</v>
+      </c>
+      <c r="L33" s="10">
+        <f>K33*0.94</f>
+        <v>0.82719999999999994</v>
+      </c>
+      <c r="M33" s="10">
+        <f>L33*1.06</f>
+        <v>0.87683199999999994</v>
+      </c>
+      <c r="N33" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O33" s="5">
         <f>N33*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P33">
-        <f>MIN(N33*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q33">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="R33" s="4">
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P33" s="5">
+        <f>N33*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q33" s="5">
+        <v>0.77</v>
+      </c>
+      <c r="R33" s="10">
         <f t="shared" si="6"/>
-        <v>0.55099999999999993</v>
-      </c>
-      <c r="S33" s="4">
+        <v>0.73149999999999993</v>
+      </c>
+      <c r="S33" s="10">
         <f t="shared" si="7"/>
-        <v>0.57855000000000001</v>
+        <v>0.76807499999999995</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B34" t="s">
         <v>73</v>
@@ -3675,71 +3634,73 @@
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>95</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E35" t="s">
-        <v>68</v>
-      </c>
-      <c r="F35" s="6">
-        <v>0.72292857142857125</v>
-      </c>
-      <c r="G35" s="6">
-        <f>11.68969/100</f>
-        <v>0.11689690000000001</v>
-      </c>
-      <c r="H35" s="7">
-        <f>1-SUM(F35:G35,I35)</f>
-        <v>5.4174528571428793E-2</v>
-      </c>
-      <c r="I35" s="5">
-        <v>0.106</v>
+        <v>69</v>
+      </c>
+      <c r="F35">
+        <v>0.23</v>
+      </c>
+      <c r="G35">
+        <v>0.01</v>
+      </c>
+      <c r="H35">
+        <v>0.45</v>
+      </c>
+      <c r="I35">
+        <v>0.31</v>
       </c>
       <c r="J35" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K35" s="6">
-        <v>0.86609999999999998</v>
-      </c>
-      <c r="L35" s="6">
-        <v>0.79749999999999999</v>
-      </c>
-      <c r="M35" s="6">
-        <v>0.93370000000000009</v>
-      </c>
-      <c r="N35" s="6">
-        <v>0.94900000000000007</v>
-      </c>
-      <c r="O35" s="6">
-        <v>0.90069999999999995</v>
-      </c>
-      <c r="P35" s="6">
-        <v>0.98250000000000004</v>
-      </c>
-      <c r="Q35" s="5">
-        <v>0.68899999999999995</v>
-      </c>
-      <c r="R35" s="10">
+      <c r="K35">
+        <v>0.8</v>
+      </c>
+      <c r="L35" s="4">
+        <f>K35*0.95</f>
+        <v>0.76</v>
+      </c>
+      <c r="M35" s="4">
+        <f>L35*1.05</f>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="N35">
+        <v>0.93</v>
+      </c>
+      <c r="O35">
+        <f>N35*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P35">
+        <f>MIN(N35*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q35">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="R35" s="4">
         <f t="shared" si="6"/>
-        <v>0.65454999999999997</v>
-      </c>
-      <c r="S35" s="10">
+        <v>0.55099999999999993</v>
+      </c>
+      <c r="S35" s="4">
         <f t="shared" si="7"/>
-        <v>0.68727749999999999</v>
+        <v>0.57855000000000001</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="B36" t="s">
         <v>75</v>
@@ -3751,34 +3712,34 @@
         <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>69</v>
-      </c>
-      <c r="F36" s="5">
-        <v>0</v>
-      </c>
-      <c r="G36" s="5">
-        <v>1</v>
-      </c>
-      <c r="H36" s="5">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F36" s="6">
+        <v>0.72292857142857125</v>
+      </c>
+      <c r="G36" s="6">
+        <f>11.68969/100</f>
+        <v>0.11689690000000001</v>
+      </c>
+      <c r="H36" s="7">
+        <f>1-SUM(F36:G36,I36)</f>
+        <v>5.4174528571428793E-2</v>
       </c>
       <c r="I36" s="5">
-        <v>0</v>
+        <v>0.106</v>
       </c>
       <c r="J36" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K36" s="5">
-        <v>0</v>
-      </c>
-      <c r="L36" s="5">
-        <f>K36*0.95</f>
-        <v>0</v>
-      </c>
-      <c r="M36" s="5">
-        <f>L36*1.05</f>
-        <v>0</v>
+      <c r="K36" s="6">
+        <v>0.86609999999999998</v>
+      </c>
+      <c r="L36" s="6">
+        <v>0.79749999999999999</v>
+      </c>
+      <c r="M36" s="6">
+        <v>0.93370000000000009</v>
       </c>
       <c r="N36" s="6">
         <v>0.94900000000000007</v>
@@ -3790,20 +3751,20 @@
         <v>0.98250000000000004</v>
       </c>
       <c r="Q36" s="5">
-        <v>0</v>
+        <v>0.68899999999999995</v>
       </c>
       <c r="R36" s="10">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.65454999999999997</v>
       </c>
       <c r="S36" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.68727749999999999</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B37" t="s">
         <v>75</v>
@@ -3815,66 +3776,65 @@
         <v>68</v>
       </c>
       <c r="E37" t="s">
-        <v>68</v>
-      </c>
-      <c r="F37" s="6">
-        <f>81.85/100</f>
-        <v>0.81849999999999989</v>
-      </c>
-      <c r="G37" s="6">
-        <f>0.1448625</f>
-        <v>0.14486250000000001</v>
-      </c>
-      <c r="H37" s="7">
-        <f>1-SUM(F37:G37,I37)</f>
-        <v>6.6375000000000739E-3</v>
+        <v>69</v>
+      </c>
+      <c r="F37" s="5">
+        <v>0</v>
+      </c>
+      <c r="G37" s="5">
+        <v>1</v>
+      </c>
+      <c r="H37" s="5">
+        <v>0</v>
       </c>
       <c r="I37" s="5">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="J37" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K37" s="6">
-        <v>0.88379999999999992</v>
-      </c>
-      <c r="L37" s="6">
-        <v>0.87650000000000006</v>
-      </c>
-      <c r="M37" s="6">
-        <v>0.88790000000000002</v>
+      <c r="K37" s="5">
+        <v>0</v>
+      </c>
+      <c r="L37" s="5">
+        <f>K37*0.95</f>
+        <v>0</v>
+      </c>
+      <c r="M37" s="5">
+        <f>L37*1.05</f>
+        <v>0</v>
       </c>
       <c r="N37" s="6">
-        <v>0.96579999999999999</v>
+        <v>0.94900000000000007</v>
       </c>
       <c r="O37" s="6">
-        <v>0.94930000000000003</v>
+        <v>0.90069999999999995</v>
       </c>
       <c r="P37" s="6">
-        <v>0.98499999999999999</v>
+        <v>0.98250000000000004</v>
       </c>
       <c r="Q37" s="5">
-        <v>0.88000000000000012</v>
+        <v>0</v>
       </c>
       <c r="R37" s="10">
         <f t="shared" si="6"/>
-        <v>0.83600000000000008</v>
+        <v>0</v>
       </c>
       <c r="S37" s="10">
         <f t="shared" si="7"/>
-        <v>0.87780000000000014</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D38" t="s">
         <v>68</v>
@@ -3883,58 +3843,60 @@
         <v>68</v>
       </c>
       <c r="F38" s="6">
-        <v>0.75900000000000001</v>
+        <f>81.85/100</f>
+        <v>0.81849999999999989</v>
       </c>
       <c r="G38" s="6">
-        <v>0.10100000000000001</v>
+        <f>0.1448625</f>
+        <v>0.14486250000000001</v>
       </c>
       <c r="H38" s="7">
         <f>1-SUM(F38:G38,I38)</f>
-        <v>0</v>
-      </c>
-      <c r="I38" s="8">
-        <v>0.14000000000000001</v>
+        <v>6.6375000000000739E-3</v>
+      </c>
+      <c r="I38" s="5">
+        <v>0.03</v>
       </c>
       <c r="J38" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K38" s="6">
-        <v>0.94140000000000001</v>
+        <v>0.88379999999999992</v>
       </c>
       <c r="L38" s="6">
-        <v>0.92920000000000003</v>
+        <v>0.87650000000000006</v>
       </c>
       <c r="M38" s="6">
-        <v>0.95040000000000002</v>
+        <v>0.88790000000000002</v>
       </c>
       <c r="N38" s="6">
-        <v>0.97010000000000007</v>
+        <v>0.96579999999999999</v>
       </c>
       <c r="O38" s="6">
-        <v>0.96840000000000004</v>
+        <v>0.94930000000000003</v>
       </c>
       <c r="P38" s="6">
-        <v>0.97239999999999993</v>
+        <v>0.98499999999999999</v>
       </c>
       <c r="Q38" s="5">
-        <v>0.68000000000000016</v>
+        <v>0.88000000000000012</v>
       </c>
       <c r="R38" s="10">
         <f t="shared" si="6"/>
-        <v>0.64600000000000013</v>
+        <v>0.83600000000000008</v>
       </c>
       <c r="S38" s="10">
         <f t="shared" si="7"/>
-        <v>0.67830000000000013</v>
+        <v>0.87780000000000014</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C39" t="s">
         <v>69</v>
@@ -3946,118 +3908,118 @@
         <v>68</v>
       </c>
       <c r="F39" s="6">
-        <v>0.65300000000000002</v>
+        <v>0.75900000000000001</v>
       </c>
       <c r="G39" s="6">
-        <v>0.02</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="H39" s="7">
         <f>1-SUM(F39:G39,I39)</f>
-        <v>0.2569999999999999</v>
-      </c>
-      <c r="I39" s="5">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
+      </c>
+      <c r="I39" s="8">
+        <v>0.14000000000000001</v>
       </c>
       <c r="J39" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K39" s="6">
-        <v>0.89379999999999993</v>
+        <v>0.94140000000000001</v>
       </c>
       <c r="L39" s="6">
-        <v>0.8881</v>
+        <v>0.92920000000000003</v>
       </c>
       <c r="M39" s="6">
-        <v>0.89969999999999994</v>
+        <v>0.95040000000000002</v>
       </c>
       <c r="N39" s="6">
-        <v>0.95799999999999996</v>
+        <v>0.97010000000000007</v>
       </c>
       <c r="O39" s="6">
-        <v>0.9323999999999999</v>
+        <v>0.96840000000000004</v>
       </c>
       <c r="P39" s="6">
-        <v>0.97730000000000006</v>
+        <v>0.97239999999999993</v>
       </c>
       <c r="Q39" s="5">
-        <v>0.82</v>
+        <v>0.68000000000000016</v>
       </c>
       <c r="R39" s="10">
         <f t="shared" si="6"/>
-        <v>0.77899999999999991</v>
+        <v>0.64600000000000013</v>
       </c>
       <c r="S39" s="10">
         <f t="shared" si="7"/>
-        <v>0.81794999999999995</v>
+        <v>0.67830000000000013</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B40" t="s">
         <v>73</v>
       </c>
       <c r="C40" t="s">
+        <v>69</v>
+      </c>
+      <c r="D40" t="s">
         <v>68</v>
       </c>
-      <c r="D40" t="s">
-        <v>69</v>
-      </c>
       <c r="E40" t="s">
-        <v>69</v>
-      </c>
-      <c r="F40" s="5">
-        <v>0</v>
-      </c>
-      <c r="G40" s="5">
-        <v>1</v>
-      </c>
-      <c r="H40" s="5">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F40" s="6">
+        <v>0.65300000000000002</v>
+      </c>
+      <c r="G40" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="H40" s="7">
+        <f>1-SUM(F40:G40,I40)</f>
+        <v>0.2569999999999999</v>
       </c>
       <c r="I40" s="5">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="J40" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K40" s="5">
-        <v>0</v>
-      </c>
-      <c r="L40" s="5">
-        <v>0</v>
-      </c>
-      <c r="M40" s="5">
-        <v>0</v>
-      </c>
-      <c r="N40" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O40" s="5">
-        <f t="shared" ref="O40:O45" si="8">N40*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P40" s="5">
-        <f>N40*1.05</f>
-        <v>0.99934990680000002</v>
+      <c r="K40" s="6">
+        <v>0.89379999999999993</v>
+      </c>
+      <c r="L40" s="6">
+        <v>0.8881</v>
+      </c>
+      <c r="M40" s="6">
+        <v>0.89969999999999994</v>
+      </c>
+      <c r="N40" s="6">
+        <v>0.95799999999999996</v>
+      </c>
+      <c r="O40" s="6">
+        <v>0.9323999999999999</v>
+      </c>
+      <c r="P40" s="6">
+        <v>0.97730000000000006</v>
       </c>
       <c r="Q40" s="5">
-        <v>0</v>
-      </c>
-      <c r="R40" s="7">
-        <v>0</v>
-      </c>
-      <c r="S40" s="7">
+        <v>0.82</v>
+      </c>
+      <c r="R40" s="10">
+        <f t="shared" si="6"/>
+        <v>0.77899999999999991</v>
+      </c>
+      <c r="S40" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.81794999999999995</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B41" t="s">
         <v>73</v>
@@ -4066,43 +4028,41 @@
         <v>68</v>
       </c>
       <c r="D41" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E41" t="s">
-        <v>68</v>
-      </c>
-      <c r="F41" s="6">
-        <v>0.66174999999999995</v>
-      </c>
-      <c r="G41" s="6">
-        <f>1.126924/100</f>
-        <v>1.126924E-2</v>
-      </c>
-      <c r="H41" s="7">
-        <f>1-SUM(F41:G41,I41)</f>
-        <v>0.25398076000000014</v>
+        <v>69</v>
+      </c>
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
+      <c r="G41" s="5">
+        <v>1</v>
+      </c>
+      <c r="H41" s="5">
+        <v>0</v>
       </c>
       <c r="I41" s="5">
-        <v>7.2999999999999995E-2</v>
+        <v>0</v>
       </c>
       <c r="J41" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K41" s="6">
-        <v>0.87599999999999989</v>
-      </c>
-      <c r="L41" s="6">
-        <v>0.8206</v>
-      </c>
-      <c r="M41" s="6">
-        <v>0.92709999999999992</v>
+      <c r="K41" s="5">
+        <v>0</v>
+      </c>
+      <c r="L41" s="5">
+        <v>0</v>
+      </c>
+      <c r="M41" s="5">
+        <v>0</v>
       </c>
       <c r="N41" s="5">
         <v>0.95176181599999998</v>
       </c>
       <c r="O41" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="O41:O46" si="8">N41*0.95</f>
         <v>0.90417372519999994</v>
       </c>
       <c r="P41" s="5">
@@ -4110,90 +4070,88 @@
         <v>0.99934990680000002</v>
       </c>
       <c r="Q41" s="5">
-        <v>0.875</v>
-      </c>
-      <c r="R41" s="10">
-        <f>Q41*0.95</f>
-        <v>0.83124999999999993</v>
-      </c>
-      <c r="S41" s="10">
+        <v>0</v>
+      </c>
+      <c r="R41" s="7">
+        <v>0</v>
+      </c>
+      <c r="S41" s="7">
         <f t="shared" si="7"/>
-        <v>0.87281249999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E42" t="s">
-        <v>69</v>
-      </c>
-      <c r="F42">
-        <v>0.63800000000000001</v>
-      </c>
-      <c r="G42">
-        <v>6.0999999999999999E-2</v>
+        <v>68</v>
+      </c>
+      <c r="F42" s="6">
+        <v>0.66174999999999995</v>
+      </c>
+      <c r="G42" s="6">
+        <f>1.126924/100</f>
+        <v>1.126924E-2</v>
       </c>
       <c r="H42" s="7">
         <f>1-SUM(F42:G42,I42)</f>
-        <v>0.21199999999999997</v>
-      </c>
-      <c r="I42">
-        <v>8.8999999999999996E-2</v>
+        <v>0.25398076000000014</v>
+      </c>
+      <c r="I42" s="5">
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="J42" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K42">
-        <v>0.81</v>
-      </c>
-      <c r="L42" s="4">
-        <f>K42*0.95</f>
-        <v>0.76949999999999996</v>
-      </c>
-      <c r="M42" s="4">
-        <f>L42*1.05</f>
-        <v>0.807975</v>
-      </c>
-      <c r="N42">
-        <v>0.93</v>
-      </c>
-      <c r="O42">
+      <c r="K42" s="6">
+        <v>0.87599999999999989</v>
+      </c>
+      <c r="L42" s="6">
+        <v>0.8206</v>
+      </c>
+      <c r="M42" s="6">
+        <v>0.92709999999999992</v>
+      </c>
+      <c r="N42" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O42" s="5">
         <f t="shared" si="8"/>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P42">
-        <f>MIN(N42*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q42">
-        <v>0.72</v>
-      </c>
-      <c r="R42" s="4">
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P42" s="5">
+        <f>N42*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q42" s="5">
+        <v>0.875</v>
+      </c>
+      <c r="R42" s="10">
         <f>Q42*0.95</f>
-        <v>0.68399999999999994</v>
-      </c>
-      <c r="S42" s="4">
+        <v>0.83124999999999993</v>
+      </c>
+      <c r="S42" s="10">
         <f t="shared" si="7"/>
-        <v>0.71819999999999995</v>
+        <v>0.87281249999999999</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C43" t="s">
         <v>69</v>
@@ -4205,31 +4163,32 @@
         <v>69</v>
       </c>
       <c r="F43">
-        <v>0.32400000000000001</v>
+        <v>0.63800000000000001</v>
       </c>
       <c r="G43">
-        <v>2.1999999999999999E-2</v>
-      </c>
-      <c r="H43">
-        <v>0.58299999999999996</v>
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="H43" s="7">
+        <f>1-SUM(F43:G43,I43)</f>
+        <v>0.21199999999999997</v>
       </c>
       <c r="I43">
-        <v>7.0999999999999994E-2</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="J43" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K43">
-        <v>0.87</v>
+        <v>0.81</v>
       </c>
       <c r="L43" s="4">
         <f>K43*0.95</f>
-        <v>0.82650000000000001</v>
+        <v>0.76949999999999996</v>
       </c>
       <c r="M43" s="4">
         <f>L43*1.05</f>
-        <v>0.86782500000000007</v>
+        <v>0.807975</v>
       </c>
       <c r="N43">
         <v>0.93</v>
@@ -4243,20 +4202,20 @@
         <v>0.97650000000000015</v>
       </c>
       <c r="Q43">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="R43" s="4">
         <f>Q43*0.95</f>
-        <v>0.57950000000000002</v>
+        <v>0.68399999999999994</v>
       </c>
       <c r="S43" s="4">
         <f t="shared" si="7"/>
-        <v>0.60847499999999999</v>
+        <v>0.71819999999999995</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B44" t="s">
         <v>73</v>
@@ -4271,16 +4230,16 @@
         <v>69</v>
       </c>
       <c r="F44">
-        <v>0.377</v>
+        <v>0.32400000000000001</v>
       </c>
       <c r="G44">
-        <v>1.7999999999999999E-2</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="H44">
-        <v>0.52800000000000002</v>
+        <v>0.58299999999999996</v>
       </c>
       <c r="I44">
-        <v>7.6999999999999999E-2</v>
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="J44" s="9">
         <f t="shared" si="0"/>
@@ -4322,7 +4281,7 @@
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B45" t="s">
         <v>73</v>
@@ -4337,31 +4296,31 @@
         <v>69</v>
       </c>
       <c r="F45">
-        <v>2.9000000000000001E-2</v>
+        <v>0.377</v>
       </c>
       <c r="G45">
-        <v>7.0000000000000001E-3</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="H45">
-        <v>0.92500000000000004</v>
+        <v>0.52800000000000002</v>
       </c>
       <c r="I45">
-        <v>3.9E-2</v>
+        <v>7.6999999999999999E-2</v>
       </c>
       <c r="J45" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K45">
-        <v>0.84000000000000008</v>
+        <v>0.87</v>
       </c>
       <c r="L45" s="4">
         <f>K45*0.95</f>
-        <v>0.79800000000000004</v>
+        <v>0.82650000000000001</v>
       </c>
       <c r="M45" s="4">
         <f>L45*1.05</f>
-        <v>0.83790000000000009</v>
+        <v>0.86782500000000007</v>
       </c>
       <c r="N45">
         <v>0.93</v>
@@ -4375,26 +4334,26 @@
         <v>0.97650000000000015</v>
       </c>
       <c r="Q45">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="R45" s="4">
         <f>Q45*0.95</f>
-        <v>0.66499999999999992</v>
+        <v>0.57950000000000002</v>
       </c>
       <c r="S45" s="4">
         <f t="shared" si="7"/>
-        <v>0.69824999999999993</v>
+        <v>0.60847499999999999</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>113</v>
+        <v>30</v>
       </c>
       <c r="B46" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C46" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D46" t="s">
         <v>69</v>
@@ -4402,127 +4361,126 @@
       <c r="E46" t="s">
         <v>69</v>
       </c>
-      <c r="F46" s="5">
-        <f>AVERAGE('trash fish table'!F2:F6)</f>
-        <v>0.56830740870546492</v>
-      </c>
-      <c r="G46" s="5">
-        <f>AVERAGE('trash fish table'!G2:G6)</f>
-        <v>0.2240987667741102</v>
-      </c>
-      <c r="H46" s="5">
-        <f>AVERAGE('trash fish table'!I2:I6)</f>
-        <v>9.0773327441505319E-2</v>
-      </c>
-      <c r="I46" s="5">
-        <f>AVERAGE('trash fish table'!H2:H6)</f>
-        <v>0.11682049707891951</v>
+      <c r="F46">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="G46">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="H46">
+        <v>0.92500000000000004</v>
+      </c>
+      <c r="I46">
+        <v>3.9E-2</v>
       </c>
       <c r="J46" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K46" s="10">
-        <v>0.87980000000000003</v>
-      </c>
-      <c r="L46" s="10">
-        <v>0.82969999999999999</v>
-      </c>
-      <c r="M46" s="10">
-        <v>0.92209999999999992</v>
-      </c>
-      <c r="N46" s="10">
-        <v>0.95669999999999999</v>
-      </c>
-      <c r="O46" s="10">
-        <v>0.8993000000000001</v>
-      </c>
-      <c r="P46" s="10">
-        <v>0.99199999999999999</v>
-      </c>
-      <c r="Q46" s="10">
-        <f>83.3/100</f>
-        <v>0.83299999999999996</v>
-      </c>
-      <c r="R46" s="10">
-        <f>74.5/100</f>
-        <v>0.745</v>
-      </c>
-      <c r="S46" s="10">
-        <f>92.6/100</f>
-        <v>0.92599999999999993</v>
+      <c r="K46">
+        <v>0.84000000000000008</v>
+      </c>
+      <c r="L46" s="4">
+        <f>K46*0.95</f>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="M46" s="4">
+        <f>L46*1.05</f>
+        <v>0.83790000000000009</v>
+      </c>
+      <c r="N46">
+        <v>0.93</v>
+      </c>
+      <c r="O46">
+        <f t="shared" si="8"/>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P46">
+        <f>MIN(N46*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q46">
+        <v>0.7</v>
+      </c>
+      <c r="R46" s="4">
+        <f>Q46*0.95</f>
+        <v>0.66499999999999992</v>
+      </c>
+      <c r="S46" s="4">
+        <f t="shared" si="7"/>
+        <v>0.69824999999999993</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>31</v>
+        <v>113</v>
       </c>
       <c r="B47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C47" t="s">
         <v>68</v>
       </c>
       <c r="D47" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E47" t="s">
         <v>69</v>
       </c>
       <c r="F47" s="5">
-        <v>0.13</v>
+        <f>AVERAGE('trash fish table'!F2:F6)</f>
+        <v>0.56830740870546492</v>
       </c>
       <c r="G47" s="5">
-        <v>0.02</v>
-      </c>
-      <c r="H47" s="7">
-        <f>1-SUM(F47:G47,I47)</f>
-        <v>0.83000000000000007</v>
+        <f>AVERAGE('trash fish table'!G2:G6)</f>
+        <v>0.2240987667741102</v>
+      </c>
+      <c r="H47" s="5">
+        <f>AVERAGE('trash fish table'!I2:I6)</f>
+        <v>9.0773327441505319E-2</v>
       </c>
       <c r="I47" s="5">
-        <v>0.02</v>
+        <f>AVERAGE('trash fish table'!H2:H6)</f>
+        <v>0.11682049707891951</v>
       </c>
       <c r="J47" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K47" s="5">
-        <v>0.9</v>
+      <c r="K47" s="10">
+        <v>0.87980000000000003</v>
       </c>
       <c r="L47" s="10">
-        <f>K47*0.94</f>
-        <v>0.84599999999999997</v>
+        <v>0.82969999999999999</v>
       </c>
       <c r="M47" s="10">
-        <f>L47*1.06</f>
-        <v>0.89676</v>
-      </c>
-      <c r="N47" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O47" s="5">
-        <f>N47*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P47" s="5">
-        <f>N47*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q47" s="5">
-        <v>0.8</v>
+        <v>0.92209999999999992</v>
+      </c>
+      <c r="N47" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O47" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P47" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q47" s="10">
+        <f>83.3/100</f>
+        <v>0.83299999999999996</v>
       </c>
       <c r="R47" s="10">
-        <f>Q47*0.95</f>
-        <v>0.76</v>
+        <f>74.5/100</f>
+        <v>0.745</v>
       </c>
       <c r="S47" s="10">
-        <f>R47*1.05</f>
-        <v>0.79800000000000004</v>
+        <f>92.6/100</f>
+        <v>0.92599999999999993</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B48" t="s">
         <v>73</v>
@@ -4537,35 +4495,32 @@
         <v>69</v>
       </c>
       <c r="F48" s="5">
-        <f>766/1000</f>
-        <v>0.76600000000000001</v>
+        <v>0.13</v>
       </c>
       <c r="G48" s="5">
-        <f>74/1000</f>
-        <v>7.3999999999999996E-2</v>
+        <v>0.02</v>
       </c>
       <c r="H48" s="7">
         <f>1-SUM(F48:G48,I48)</f>
-        <v>0.15300000000000002</v>
+        <v>0.83000000000000007</v>
       </c>
       <c r="I48" s="5">
-        <f>7/1000</f>
-        <v>7.0000000000000001E-3</v>
+        <v>0.02</v>
       </c>
       <c r="J48" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K48" s="5">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="L48" s="10">
         <f>K48*0.94</f>
-        <v>0.83660000000000001</v>
+        <v>0.84599999999999997</v>
       </c>
       <c r="M48" s="10">
         <f>L48*1.06</f>
-        <v>0.88679600000000003</v>
+        <v>0.89676</v>
       </c>
       <c r="N48" s="5">
         <v>0.95176181599999998</v>
@@ -4579,207 +4534,217 @@
         <v>0.99934990680000002</v>
       </c>
       <c r="Q48" s="5">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="R48" s="10">
         <f>Q48*0.95</f>
-        <v>0.71249999999999991</v>
+        <v>0.76</v>
       </c>
       <c r="S48" s="10">
         <f>R48*1.05</f>
-        <v>0.74812499999999993</v>
+        <v>0.79800000000000004</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B49" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E49" t="s">
         <v>69</v>
       </c>
-      <c r="F49">
-        <v>0.48</v>
-      </c>
-      <c r="G49">
-        <v>0.04</v>
-      </c>
-      <c r="H49">
-        <v>0.41</v>
-      </c>
-      <c r="I49">
-        <v>7.0000000000000007E-2</v>
+      <c r="F49" s="5">
+        <f>766/1000</f>
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="G49" s="5">
+        <f>74/1000</f>
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="H49" s="7">
+        <f>1-SUM(F49:G49,I49)</f>
+        <v>0.15300000000000002</v>
+      </c>
+      <c r="I49" s="5">
+        <f>7/1000</f>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="J49" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K49">
-        <v>0.82000000000000006</v>
-      </c>
-      <c r="L49" s="4">
-        <f>K49*0.95</f>
-        <v>0.77900000000000003</v>
-      </c>
-      <c r="M49" s="4">
-        <f>L49*1.05</f>
-        <v>0.81795000000000007</v>
-      </c>
-      <c r="N49">
-        <v>0.93</v>
-      </c>
-      <c r="O49">
+      <c r="K49" s="5">
+        <v>0.89</v>
+      </c>
+      <c r="L49" s="10">
+        <f>K49*0.94</f>
+        <v>0.83660000000000001</v>
+      </c>
+      <c r="M49" s="10">
+        <f>L49*1.06</f>
+        <v>0.88679600000000003</v>
+      </c>
+      <c r="N49" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O49" s="5">
         <f>N49*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P49">
-        <f>MIN(N49*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q49">
-        <v>0.7</v>
-      </c>
-      <c r="R49" s="4">
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P49" s="5">
+        <f>N49*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q49" s="5">
+        <v>0.75</v>
+      </c>
+      <c r="R49" s="10">
         <f>Q49*0.95</f>
-        <v>0.66499999999999992</v>
-      </c>
-      <c r="S49" s="4">
+        <v>0.71249999999999991</v>
+      </c>
+      <c r="S49" s="10">
         <f>R49*1.05</f>
-        <v>0.69824999999999993</v>
+        <v>0.74812499999999993</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>116</v>
+        <v>33</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="C50" t="s">
+        <v>69</v>
+      </c>
+      <c r="D50" t="s">
+        <v>69</v>
       </c>
       <c r="E50" t="s">
         <v>69</v>
       </c>
-      <c r="F50" s="5">
-        <v>0.53300000000000003</v>
-      </c>
-      <c r="G50" s="5">
-        <v>2.1000000000000001E-2</v>
-      </c>
-      <c r="H50" s="9">
-        <f>1-F50-G50-I50</f>
-        <v>0.37699999999999995</v>
-      </c>
-      <c r="I50" s="5">
-        <v>6.9000000000000006E-2</v>
+      <c r="F50">
+        <v>0.48</v>
+      </c>
+      <c r="G50">
+        <v>0.04</v>
+      </c>
+      <c r="H50">
+        <v>0.41</v>
+      </c>
+      <c r="I50">
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="J50" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K50" s="16">
-        <v>0.81</v>
+      <c r="K50">
+        <v>0.82000000000000006</v>
       </c>
       <c r="L50" s="4">
         <f>K50*0.95</f>
-        <v>0.76949999999999996</v>
+        <v>0.77900000000000003</v>
       </c>
       <c r="M50" s="4">
         <f>L50*1.05</f>
-        <v>0.807975</v>
+        <v>0.81795000000000007</v>
       </c>
       <c r="N50">
-        <v>0.96</v>
-      </c>
-      <c r="O50" s="4">
+        <v>0.93</v>
+      </c>
+      <c r="O50">
         <f>N50*0.95</f>
-        <v>0.91199999999999992</v>
-      </c>
-      <c r="P50" s="4">
-        <f>O50*1.05</f>
-        <v>0.95760000000000001</v>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P50">
+        <f>MIN(N50*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
       </c>
       <c r="Q50">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="R50" s="4">
         <f>Q50*0.95</f>
-        <v>0.67449999999999999</v>
+        <v>0.66499999999999992</v>
       </c>
       <c r="S50" s="4">
         <f>R50*1.05</f>
-        <v>0.70822499999999999</v>
+        <v>0.69824999999999993</v>
       </c>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B51" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E51" t="s">
         <v>69</v>
       </c>
-      <c r="F51" s="16">
-        <v>0.69</v>
-      </c>
-      <c r="G51" s="16">
-        <v>0.05</v>
+      <c r="F51" s="5">
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="G51" s="5">
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="H51" s="9">
         <f>1-F51-G51-I51</f>
-        <v>0.21000000000000008</v>
-      </c>
-      <c r="I51" s="16">
-        <v>0.05</v>
+        <v>0.37699999999999995</v>
+      </c>
+      <c r="I51" s="5">
+        <v>6.9000000000000006E-2</v>
       </c>
       <c r="J51" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K51" s="10">
-        <v>0.83</v>
-      </c>
-      <c r="L51" s="10">
+      <c r="K51" s="16">
+        <v>0.81</v>
+      </c>
+      <c r="L51" s="4">
         <f>K51*0.95</f>
-        <v>0.78849999999999998</v>
-      </c>
-      <c r="M51" s="10">
-        <f>K51*1.05</f>
-        <v>0.87149999999999994</v>
-      </c>
-      <c r="N51" s="10">
-        <v>0.95669999999999999</v>
-      </c>
-      <c r="O51" s="10">
-        <v>0.8993000000000001</v>
-      </c>
-      <c r="P51" s="10">
-        <v>0.99199999999999999</v>
-      </c>
-      <c r="Q51" s="10">
-        <f>81.7/100</f>
-        <v>0.81700000000000006</v>
-      </c>
-      <c r="R51" s="10">
-        <f>71.8/100</f>
-        <v>0.71799999999999997</v>
-      </c>
-      <c r="S51" s="10">
-        <f>91.6/100</f>
-        <v>0.91599999999999993</v>
+        <v>0.76949999999999996</v>
+      </c>
+      <c r="M51" s="4">
+        <f>L51*1.05</f>
+        <v>0.807975</v>
+      </c>
+      <c r="N51">
+        <v>0.96</v>
+      </c>
+      <c r="O51" s="4">
+        <f>N51*0.95</f>
+        <v>0.91199999999999992</v>
+      </c>
+      <c r="P51" s="4">
+        <f>O51*1.05</f>
+        <v>0.95760000000000001</v>
+      </c>
+      <c r="Q51">
+        <v>0.71</v>
+      </c>
+      <c r="R51" s="4">
+        <f>Q51*0.95</f>
+        <v>0.67449999999999999</v>
+      </c>
+      <c r="S51" s="4">
+        <f>R51*1.05</f>
+        <v>0.70822499999999999</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A52" s="17" t="s">
-        <v>119</v>
+      <c r="A52" t="s">
+        <v>118</v>
       </c>
       <c r="B52" t="s">
         <v>74</v>
@@ -4787,92 +4752,115 @@
       <c r="E52" t="s">
         <v>69</v>
       </c>
-      <c r="F52" s="5">
-        <v>0</v>
-      </c>
-      <c r="G52" s="5">
-        <v>1</v>
-      </c>
-      <c r="H52">
-        <v>0</v>
-      </c>
-      <c r="I52" s="5">
-        <v>0</v>
+      <c r="F52" s="16">
+        <v>0.69</v>
+      </c>
+      <c r="G52" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="H52" s="9">
+        <f>1-F52-G52-I52</f>
+        <v>0.21000000000000008</v>
+      </c>
+      <c r="I52" s="16">
+        <v>0.05</v>
       </c>
       <c r="J52" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K52" s="9">
-        <v>0</v>
-      </c>
-      <c r="L52" s="9">
-        <v>0</v>
-      </c>
-      <c r="M52" s="9">
-        <v>0</v>
-      </c>
-      <c r="N52" s="9">
-        <v>0.96</v>
-      </c>
-      <c r="O52">
-        <f>N52*0.95</f>
-        <v>0.91199999999999992</v>
-      </c>
-      <c r="P52">
-        <f>N52*1.05</f>
-        <v>1.008</v>
-      </c>
-      <c r="Q52" s="9">
-        <v>0</v>
-      </c>
-      <c r="R52" s="9">
-        <v>0</v>
-      </c>
-      <c r="S52" s="9">
-        <v>0</v>
+      <c r="K52" s="10">
+        <v>0.83</v>
+      </c>
+      <c r="L52" s="10">
+        <f>K52*0.95</f>
+        <v>0.78849999999999998</v>
+      </c>
+      <c r="M52" s="10">
+        <f>K52*1.05</f>
+        <v>0.87149999999999994</v>
+      </c>
+      <c r="N52" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O52" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P52" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q52" s="10">
+        <f>81.7/100</f>
+        <v>0.81700000000000006</v>
+      </c>
+      <c r="R52" s="10">
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="S52" s="10">
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B53" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E53" t="s">
         <v>69</v>
       </c>
-      <c r="F53" s="18">
-        <v>0.224</v>
+      <c r="F53" s="5">
+        <v>0</v>
       </c>
       <c r="G53" s="5">
-        <v>9.8000000000000004E-2</v>
-      </c>
-      <c r="H53" s="18">
-        <f>1-I53-F53-G53</f>
-        <v>0.61</v>
+        <v>1</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
       </c>
       <c r="I53" s="5">
-        <v>6.8000000000000005E-2</v>
+        <v>0</v>
       </c>
       <c r="J53" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K53" s="18">
-        <v>0.70899999999999996</v>
-      </c>
-      <c r="N53">
+      <c r="K53" s="9">
+        <v>0</v>
+      </c>
+      <c r="L53" s="9">
+        <v>0</v>
+      </c>
+      <c r="M53" s="9">
+        <v>0</v>
+      </c>
+      <c r="N53" s="9">
         <v>0.96</v>
       </c>
-      <c r="Q53" s="18">
-        <v>0.55500000000000005</v>
+      <c r="O53">
+        <f>N53*0.95</f>
+        <v>0.91199999999999992</v>
+      </c>
+      <c r="P53">
+        <f>N53*1.05</f>
+        <v>1.008</v>
+      </c>
+      <c r="Q53" s="9">
+        <v>0</v>
+      </c>
+      <c r="R53" s="9">
+        <v>0</v>
+      </c>
+      <c r="S53" s="9">
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>120</v>
+      <c r="A54" s="17" t="s">
+        <v>122</v>
       </c>
       <c r="B54" t="s">
         <v>73</v>
@@ -4880,36 +4868,36 @@
       <c r="E54" t="s">
         <v>69</v>
       </c>
-      <c r="F54">
-        <v>0.14199999999999999</v>
+      <c r="F54" s="18">
+        <v>0.224</v>
       </c>
       <c r="G54" s="5">
-        <v>0.13200000000000001</v>
-      </c>
-      <c r="H54" s="9">
-        <f>1-F54-G54-I54</f>
-        <v>0.65700000000000003</v>
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="H54" s="18">
+        <f>1-I54-F54-G54</f>
+        <v>0.61</v>
       </c>
       <c r="I54" s="5">
-        <v>6.9000000000000006E-2</v>
+        <v>6.8000000000000005E-2</v>
       </c>
       <c r="J54" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K54" s="9">
-        <v>0.79500000000000004</v>
+      <c r="K54" s="18">
+        <v>0.70899999999999996</v>
       </c>
       <c r="N54">
         <v>0.96</v>
       </c>
       <c r="Q54" s="18">
-        <v>0.83699999999999997</v>
+        <v>0.55500000000000005</v>
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B55" t="s">
         <v>73</v>
@@ -4918,61 +4906,98 @@
         <v>69</v>
       </c>
       <c r="F55">
-        <v>0.17299999999999999</v>
+        <v>0.14199999999999999</v>
       </c>
       <c r="G55" s="5">
-        <v>3.7999999999999999E-2</v>
+        <v>0.13200000000000001</v>
       </c>
       <c r="H55" s="9">
         <f>1-F55-G55-I55</f>
-        <v>0.73299999999999987</v>
+        <v>0.65700000000000003</v>
       </c>
       <c r="I55" s="5">
-        <v>5.6000000000000001E-2</v>
+        <v>6.9000000000000006E-2</v>
       </c>
       <c r="J55" s="9">
         <f t="shared" si="0"/>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
       <c r="K55" s="9">
-        <v>0.64900000000000002</v>
+        <v>0.79500000000000004</v>
       </c>
       <c r="N55">
         <v>0.96</v>
       </c>
-      <c r="Q55">
+      <c r="Q55" s="18">
+        <v>0.83699999999999997</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>121</v>
+      </c>
+      <c r="B56" t="s">
+        <v>73</v>
+      </c>
+      <c r="E56" t="s">
+        <v>69</v>
+      </c>
+      <c r="F56">
+        <v>0.17299999999999999</v>
+      </c>
+      <c r="G56" s="5">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="H56" s="9">
+        <f>1-F56-G56-I56</f>
+        <v>0.73299999999999987</v>
+      </c>
+      <c r="I56" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="J56" s="9">
+        <f t="shared" si="0"/>
+        <v>0.99999999999999989</v>
+      </c>
+      <c r="K56" s="9">
+        <v>0.64900000000000002</v>
+      </c>
+      <c r="N56">
+        <v>0.96</v>
+      </c>
+      <c r="Q56">
         <v>0.57099999999999995</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S55" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}"/>
-  <conditionalFormatting sqref="K2:S38">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
+  <autoFilter ref="A1:S56" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}"/>
+  <conditionalFormatting sqref="K2:S39">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K48:S49">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
+  <conditionalFormatting sqref="K49:S50">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K51:S51">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="K52:S52">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L50:M50">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="L51:M51">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O50:P50">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
+  <conditionalFormatting sqref="O51:P51">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R50:S50">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="R51:S51">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Fixed problematic whiteleg_shrimp population params
</commit_message>
<xml_diff>
--- a/data/raw_data/all_ingredients.xlsx
+++ b/data/raw_data/all_ingredients.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\treimer\Documents\R-temp-files\climate_risks_to_fed_mariculture\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091A0C66-A267-47A7-A43D-AFA43A7F5035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F2AD20-AC53-4A80-B6B7-ABF704C7ECF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2376" yWindow="1020" windowWidth="20136" windowHeight="13908" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
+    <workbookView xWindow="36" yWindow="0" windowWidth="23016" windowHeight="16656" xr2:uid="{EACE1C46-B374-4940-8FA1-58EDCA6D9B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="all_ingredients" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="trash fish table" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">all_ingredients!$A$1:$S$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sources!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="134">
   <si>
     <t>ingredient</t>
   </si>
@@ -429,6 +429,18 @@
   </si>
   <si>
     <t>palm-oil</t>
+  </si>
+  <si>
+    <t>squid-oil</t>
+  </si>
+  <si>
+    <t>shrimp-meal</t>
+  </si>
+  <si>
+    <t>shrimp-head-meal</t>
+  </si>
+  <si>
+    <t>Shrimp meal | Feedipedia</t>
   </si>
 </sst>
 </file>
@@ -965,7 +977,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -986,7 +998,6 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="45">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1035,7 +1046,17 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1426,7 +1447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-  <dimension ref="A1:S58"/>
+  <dimension ref="A1:S61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" customWidth="1"/>
@@ -1590,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="J3" s="9">
-        <f t="shared" ref="J3:J58" si="0">SUM(F3:I3)</f>
+        <f t="shared" ref="J3:J61" si="0">SUM(F3:I3)</f>
         <v>1</v>
       </c>
       <c r="K3" s="5">
@@ -1751,7 +1772,7 @@
         <v>0.68428500000000014</v>
       </c>
     </row>
-    <row r="6" spans="1:19" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1817,11 +1838,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:19" s="18" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>128</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" t="s">
         <v>73</v>
       </c>
       <c r="F7" s="8">
@@ -1857,16 +1878,13 @@
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
     </row>
-    <row r="8" spans="1:19" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>127</v>
       </c>
       <c r="B8" t="s">
         <v>73</v>
       </c>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
       <c r="F8" s="8">
         <v>0</v>
       </c>
@@ -3509,15 +3527,12 @@
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A34" s="18" t="s">
+      <c r="A34" t="s">
         <v>129</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
       <c r="F34" s="8">
         <v>0</v>
       </c>
@@ -3609,7 +3624,7 @@
         <v>0.93</v>
       </c>
       <c r="O35">
-        <f>N35*0.95</f>
+        <f t="shared" ref="O35:O40" si="1">N35*0.95</f>
         <v>0.88349999999999995</v>
       </c>
       <c r="P35">
@@ -3620,11 +3635,11 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="R35" s="4">
-        <f>Q35*0.95</f>
+        <f t="shared" ref="R35:R43" si="2">Q35*0.95</f>
         <v>0.55099999999999993</v>
       </c>
       <c r="S35" s="4">
-        <f>R35*1.05</f>
+        <f t="shared" ref="S35:S43" si="3">R35*1.05</f>
         <v>0.57855000000000001</v>
       </c>
     </row>
@@ -3670,7 +3685,7 @@
         <v>0.96</v>
       </c>
       <c r="O36" s="4">
-        <f>N36*0.95</f>
+        <f t="shared" si="1"/>
         <v>0.91199999999999992</v>
       </c>
       <c r="P36" s="4">
@@ -3681,11 +3696,11 @@
         <v>0.71</v>
       </c>
       <c r="R36" s="4">
-        <f>Q36*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.67449999999999999</v>
       </c>
       <c r="S36" s="4">
-        <f>R36*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.70822499999999999</v>
       </c>
     </row>
@@ -3736,7 +3751,7 @@
         <v>0.95176181599999998</v>
       </c>
       <c r="O37" s="5">
-        <f>N37*0.95</f>
+        <f t="shared" si="1"/>
         <v>0.90417372519999994</v>
       </c>
       <c r="P37" s="5">
@@ -3747,11 +3762,11 @@
         <v>0.77</v>
       </c>
       <c r="R37" s="10">
-        <f>Q37*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.73149999999999993</v>
       </c>
       <c r="S37" s="10">
-        <f>R37*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.76807499999999995</v>
       </c>
     </row>
@@ -3802,7 +3817,7 @@
         <v>0.93</v>
       </c>
       <c r="O38">
-        <f>N38*0.95</f>
+        <f t="shared" si="1"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P38">
@@ -3813,11 +3828,11 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="R38" s="4">
-        <f>Q38*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.55099999999999993</v>
       </c>
       <c r="S38" s="4">
-        <f>R38*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.57855000000000001</v>
       </c>
     </row>
@@ -3868,7 +3883,7 @@
         <v>0.93</v>
       </c>
       <c r="O39">
-        <f>N39*0.95</f>
+        <f t="shared" si="1"/>
         <v>0.88349999999999995</v>
       </c>
       <c r="P39">
@@ -3879,11 +3894,11 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="R39" s="4">
-        <f>Q39*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.55099999999999993</v>
       </c>
       <c r="S39" s="4">
-        <f>R39*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.57855000000000001</v>
       </c>
     </row>
@@ -3935,7 +3950,7 @@
         <v>0.95176181599999998</v>
       </c>
       <c r="O40" s="5">
-        <f>N40*0.95</f>
+        <f t="shared" si="1"/>
         <v>0.90417372519999994</v>
       </c>
       <c r="P40" s="5">
@@ -3946,11 +3961,11 @@
         <v>0.60399999999999998</v>
       </c>
       <c r="R40" s="7">
-        <f>Q40*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.57379999999999998</v>
       </c>
       <c r="S40" s="7">
-        <f>R40*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.60248999999999997</v>
       </c>
     </row>
@@ -4010,11 +4025,11 @@
         <v>0.68899999999999995</v>
       </c>
       <c r="R41" s="10">
-        <f>Q41*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.65454999999999997</v>
       </c>
       <c r="S41" s="10">
-        <f>R41*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.68727749999999999</v>
       </c>
     </row>
@@ -4074,11 +4089,11 @@
         <v>0</v>
       </c>
       <c r="R42" s="10">
-        <f>Q42*0.95</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S42" s="10">
-        <f>R42*1.05</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4139,11 +4154,11 @@
         <v>0.88000000000000012</v>
       </c>
       <c r="R43" s="10">
-        <f>Q43*0.95</f>
+        <f t="shared" si="2"/>
         <v>0.83600000000000008</v>
       </c>
       <c r="S43" s="10">
-        <f>R43*1.05</f>
+        <f t="shared" si="3"/>
         <v>0.87780000000000014</v>
       </c>
     </row>
@@ -4186,202 +4201,194 @@
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>23</v>
+        <v>132</v>
       </c>
       <c r="B45" t="s">
-        <v>72</v>
-      </c>
-      <c r="C45" t="s">
+        <v>74</v>
+      </c>
+      <c r="E45" t="s">
         <v>69</v>
       </c>
-      <c r="D45" t="s">
-        <v>68</v>
-      </c>
-      <c r="E45" t="s">
-        <v>68</v>
-      </c>
-      <c r="F45" s="6">
-        <v>0.75900000000000001</v>
-      </c>
-      <c r="G45" s="6">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="H45" s="7">
-        <f>1-SUM(F45:G45,I45)</f>
-        <v>0</v>
-      </c>
-      <c r="I45" s="8">
-        <v>0.14000000000000001</v>
+      <c r="F45" s="15">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="G45" s="15">
+        <v>3.9E-2</v>
+      </c>
+      <c r="H45" s="9">
+        <f>1-I45-F45-G45</f>
+        <v>7.5999999999999984E-2</v>
+      </c>
+      <c r="I45" s="15">
+        <v>0.40600000000000003</v>
       </c>
       <c r="J45" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K45" s="6">
-        <v>0.94140000000000001</v>
-      </c>
-      <c r="L45" s="6">
-        <v>0.92920000000000003</v>
-      </c>
-      <c r="M45" s="6">
-        <v>0.95040000000000002</v>
-      </c>
-      <c r="N45" s="6">
-        <v>0.97010000000000007</v>
-      </c>
-      <c r="O45" s="6">
-        <v>0.96840000000000004</v>
-      </c>
-      <c r="P45" s="6">
-        <v>0.97239999999999993</v>
-      </c>
-      <c r="Q45" s="5">
-        <v>0.68000000000000016</v>
+      <c r="K45" s="10">
+        <v>0.83</v>
+      </c>
+      <c r="L45" s="10">
+        <f>K45*0.95</f>
+        <v>0.78849999999999998</v>
+      </c>
+      <c r="M45" s="10">
+        <f>K45*1.05</f>
+        <v>0.87149999999999994</v>
+      </c>
+      <c r="N45" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O45" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P45" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q45" s="8">
+        <v>0.73499999999999999</v>
       </c>
       <c r="R45" s="10">
-        <f>Q45*0.95</f>
-        <v>0.64600000000000013</v>
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
       </c>
       <c r="S45" s="10">
-        <f>R45*1.05</f>
-        <v>0.67830000000000013</v>
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>24</v>
+        <v>131</v>
       </c>
       <c r="B46" t="s">
-        <v>73</v>
-      </c>
-      <c r="C46" t="s">
+        <v>74</v>
+      </c>
+      <c r="E46" t="s">
         <v>69</v>
       </c>
-      <c r="D46" t="s">
-        <v>68</v>
-      </c>
-      <c r="E46" t="s">
-        <v>68</v>
-      </c>
-      <c r="F46" s="6">
-        <v>0.65300000000000002</v>
-      </c>
-      <c r="G46" s="6">
-        <v>0.02</v>
-      </c>
-      <c r="H46" s="7">
-        <f>1-SUM(F46:G46,I46)</f>
-        <v>0.2569999999999999</v>
-      </c>
-      <c r="I46" s="5">
-        <v>7.0000000000000007E-2</v>
+      <c r="F46" s="9">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="G46" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="H46" s="9">
+        <f>1-I46-F46-G46</f>
+        <v>0.13799999999999996</v>
+      </c>
+      <c r="I46" s="15">
+        <v>0.17699999999999999</v>
       </c>
       <c r="J46" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J46" si="4">SUM(F46:I46)</f>
         <v>1</v>
       </c>
-      <c r="K46" s="6">
-        <v>0.89379999999999993</v>
-      </c>
-      <c r="L46" s="6">
-        <v>0.8881</v>
-      </c>
-      <c r="M46" s="6">
-        <v>0.89969999999999994</v>
-      </c>
-      <c r="N46" s="6">
-        <v>0.95799999999999996</v>
-      </c>
-      <c r="O46" s="6">
-        <v>0.9323999999999999</v>
-      </c>
-      <c r="P46" s="6">
-        <v>0.97730000000000006</v>
-      </c>
-      <c r="Q46" s="5">
-        <v>0.82</v>
+      <c r="K46" s="10">
+        <v>0.83</v>
+      </c>
+      <c r="L46" s="10">
+        <f>K46*0.95</f>
+        <v>0.78849999999999998</v>
+      </c>
+      <c r="M46" s="10">
+        <f>K46*1.05</f>
+        <v>0.87149999999999994</v>
+      </c>
+      <c r="N46" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O46" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P46" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q46" s="8">
+        <v>0.88200000000000001</v>
       </c>
       <c r="R46" s="10">
-        <f>Q46*0.95</f>
-        <v>0.77899999999999991</v>
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
       </c>
       <c r="S46" s="10">
-        <f>R46*1.05</f>
-        <v>0.81794999999999995</v>
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C47" t="s">
+        <v>69</v>
+      </c>
+      <c r="D47" t="s">
         <v>68</v>
       </c>
-      <c r="D47" t="s">
-        <v>69</v>
-      </c>
       <c r="E47" t="s">
-        <v>69</v>
-      </c>
-      <c r="F47" s="5">
-        <v>0</v>
-      </c>
-      <c r="G47" s="5">
-        <v>1</v>
-      </c>
-      <c r="H47" s="5">
-        <v>0</v>
-      </c>
-      <c r="I47" s="5">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="F47" s="6">
+        <v>0.75900000000000001</v>
+      </c>
+      <c r="G47" s="6">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="H47" s="7">
+        <f>1-SUM(F47:G47,I47)</f>
+        <v>0</v>
+      </c>
+      <c r="I47" s="8">
+        <v>0.14000000000000001</v>
       </c>
       <c r="J47" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K47" s="5">
-        <v>0</v>
-      </c>
-      <c r="L47" s="5">
-        <v>0</v>
-      </c>
-      <c r="M47" s="5">
-        <v>0</v>
-      </c>
-      <c r="N47" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O47" s="5">
-        <f>N47*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P47" s="5">
-        <f>N47*1.05</f>
-        <v>0.99934990680000002</v>
+      <c r="K47" s="6">
+        <v>0.94140000000000001</v>
+      </c>
+      <c r="L47" s="6">
+        <v>0.92920000000000003</v>
+      </c>
+      <c r="M47" s="6">
+        <v>0.95040000000000002</v>
+      </c>
+      <c r="N47" s="6">
+        <v>0.97010000000000007</v>
+      </c>
+      <c r="O47" s="6">
+        <v>0.96840000000000004</v>
+      </c>
+      <c r="P47" s="6">
+        <v>0.97239999999999993</v>
       </c>
       <c r="Q47" s="5">
-        <v>0</v>
-      </c>
-      <c r="R47" s="7">
-        <v>0</v>
-      </c>
-      <c r="S47" s="7">
+        <v>0.68000000000000016</v>
+      </c>
+      <c r="R47" s="10">
+        <f>Q47*0.95</f>
+        <v>0.64600000000000013</v>
+      </c>
+      <c r="S47" s="10">
         <f>R47*1.05</f>
-        <v>0</v>
+        <v>0.67830000000000013</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B48" t="s">
         <v>73</v>
       </c>
       <c r="C48" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D48" t="s">
         <v>68</v>
@@ -4390,64 +4397,61 @@
         <v>68</v>
       </c>
       <c r="F48" s="6">
-        <v>0.66174999999999995</v>
+        <v>0.65300000000000002</v>
       </c>
       <c r="G48" s="6">
-        <f>1.126924/100</f>
-        <v>1.126924E-2</v>
+        <v>0.02</v>
       </c>
       <c r="H48" s="7">
         <f>1-SUM(F48:G48,I48)</f>
-        <v>0.25398076000000014</v>
+        <v>0.2569999999999999</v>
       </c>
       <c r="I48" s="5">
-        <v>7.2999999999999995E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="J48" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K48" s="6">
-        <v>0.87599999999999989</v>
+        <v>0.89379999999999993</v>
       </c>
       <c r="L48" s="6">
-        <v>0.8206</v>
+        <v>0.8881</v>
       </c>
       <c r="M48" s="6">
-        <v>0.92709999999999992</v>
-      </c>
-      <c r="N48" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O48" s="5">
-        <f>N48*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P48" s="5">
-        <f>N48*1.05</f>
-        <v>0.99934990680000002</v>
+        <v>0.89969999999999994</v>
+      </c>
+      <c r="N48" s="6">
+        <v>0.95799999999999996</v>
+      </c>
+      <c r="O48" s="6">
+        <v>0.9323999999999999</v>
+      </c>
+      <c r="P48" s="6">
+        <v>0.97730000000000006</v>
       </c>
       <c r="Q48" s="5">
-        <v>0.875</v>
+        <v>0.82</v>
       </c>
       <c r="R48" s="10">
         <f>Q48*0.95</f>
-        <v>0.83124999999999993</v>
+        <v>0.77899999999999991</v>
       </c>
       <c r="S48" s="10">
         <f>R48*1.05</f>
-        <v>0.87281249999999999</v>
+        <v>0.81794999999999995</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B49" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D49" t="s">
         <v>69</v>
@@ -4455,123 +4459,125 @@
       <c r="E49" t="s">
         <v>69</v>
       </c>
-      <c r="F49">
-        <v>0.63800000000000001</v>
-      </c>
-      <c r="G49">
-        <v>6.0999999999999999E-2</v>
-      </c>
-      <c r="H49" s="7">
-        <f>1-SUM(F49:G49,I49)</f>
-        <v>0.21199999999999997</v>
-      </c>
-      <c r="I49">
-        <v>8.8999999999999996E-2</v>
+      <c r="F49" s="5">
+        <v>0</v>
+      </c>
+      <c r="G49" s="5">
+        <v>1</v>
+      </c>
+      <c r="H49" s="5">
+        <v>0</v>
+      </c>
+      <c r="I49" s="5">
+        <v>0</v>
       </c>
       <c r="J49" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K49">
-        <v>0.81</v>
-      </c>
-      <c r="L49" s="4">
-        <f>K49*0.95</f>
-        <v>0.76949999999999996</v>
-      </c>
-      <c r="M49" s="4">
-        <f>L49*1.05</f>
-        <v>0.807975</v>
-      </c>
-      <c r="N49">
-        <v>0.93</v>
-      </c>
-      <c r="O49">
+      <c r="K49" s="5">
+        <v>0</v>
+      </c>
+      <c r="L49" s="5">
+        <v>0</v>
+      </c>
+      <c r="M49" s="5">
+        <v>0</v>
+      </c>
+      <c r="N49" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O49" s="5">
         <f>N49*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P49">
-        <f>MIN(N49*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q49">
-        <v>0.72</v>
-      </c>
-      <c r="R49" s="4">
-        <f>Q49*0.95</f>
-        <v>0.68399999999999994</v>
-      </c>
-      <c r="S49" s="4">
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P49" s="5">
+        <f>N49*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q49" s="5">
+        <v>0</v>
+      </c>
+      <c r="R49" s="7">
+        <v>0</v>
+      </c>
+      <c r="S49" s="7">
         <f>R49*1.05</f>
-        <v>0.71819999999999995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>118</v>
+        <v>26</v>
       </c>
       <c r="B50" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50" t="s">
+        <v>68</v>
       </c>
       <c r="E50" t="s">
-        <v>69</v>
-      </c>
-      <c r="F50" s="15">
-        <v>0.69</v>
-      </c>
-      <c r="G50" s="15">
-        <v>0.05</v>
-      </c>
-      <c r="H50" s="9">
-        <f>1-F50-G50-I50</f>
-        <v>0.21000000000000008</v>
-      </c>
-      <c r="I50" s="15">
-        <v>0.05</v>
+        <v>68</v>
+      </c>
+      <c r="F50" s="6">
+        <v>0.66174999999999995</v>
+      </c>
+      <c r="G50" s="6">
+        <f>1.126924/100</f>
+        <v>1.126924E-2</v>
+      </c>
+      <c r="H50" s="7">
+        <f>1-SUM(F50:G50,I50)</f>
+        <v>0.25398076000000014</v>
+      </c>
+      <c r="I50" s="5">
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="J50" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K50" s="10">
-        <v>0.83</v>
-      </c>
-      <c r="L50" s="10">
-        <f>K50*0.95</f>
-        <v>0.78849999999999998</v>
-      </c>
-      <c r="M50" s="10">
-        <f>K50*1.05</f>
-        <v>0.87149999999999994</v>
-      </c>
-      <c r="N50" s="10">
-        <v>0.95669999999999999</v>
-      </c>
-      <c r="O50" s="10">
-        <v>0.8993000000000001</v>
-      </c>
-      <c r="P50" s="10">
-        <v>0.99199999999999999</v>
-      </c>
-      <c r="Q50" s="10">
-        <f>81.7/100</f>
-        <v>0.81700000000000006</v>
+      <c r="K50" s="6">
+        <v>0.87599999999999989</v>
+      </c>
+      <c r="L50" s="6">
+        <v>0.8206</v>
+      </c>
+      <c r="M50" s="6">
+        <v>0.92709999999999992</v>
+      </c>
+      <c r="N50" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O50" s="5">
+        <f>N50*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P50" s="5">
+        <f>N50*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q50" s="5">
+        <v>0.875</v>
       </c>
       <c r="R50" s="10">
-        <f>71.8/100</f>
-        <v>0.71799999999999997</v>
+        <f>Q50*0.95</f>
+        <v>0.83124999999999993</v>
       </c>
       <c r="S50" s="10">
-        <f>91.6/100</f>
-        <v>0.91599999999999993</v>
+        <f>R50*1.05</f>
+        <v>0.87281249999999999</v>
       </c>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B51" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C51" t="s">
         <v>69</v>
@@ -4583,31 +4589,32 @@
         <v>69</v>
       </c>
       <c r="F51">
-        <v>0.32400000000000001</v>
+        <v>0.63800000000000001</v>
       </c>
       <c r="G51">
-        <v>2.1999999999999999E-2</v>
-      </c>
-      <c r="H51">
-        <v>0.58299999999999996</v>
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="H51" s="7">
+        <f>1-SUM(F51:G51,I51)</f>
+        <v>0.21199999999999997</v>
       </c>
       <c r="I51">
-        <v>7.0999999999999994E-2</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="J51" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K51">
-        <v>0.87</v>
+        <v>0.81</v>
       </c>
       <c r="L51" s="4">
         <f>K51*0.95</f>
-        <v>0.82650000000000001</v>
+        <v>0.76949999999999996</v>
       </c>
       <c r="M51" s="4">
         <f>L51*1.05</f>
-        <v>0.86782500000000007</v>
+        <v>0.807975</v>
       </c>
       <c r="N51">
         <v>0.93</v>
@@ -4621,158 +4628,144 @@
         <v>0.97650000000000015</v>
       </c>
       <c r="Q51">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="R51" s="4">
         <f>Q51*0.95</f>
-        <v>0.57950000000000002</v>
+        <v>0.68399999999999994</v>
       </c>
       <c r="S51" s="4">
         <f>R51*1.05</f>
-        <v>0.60847499999999999</v>
+        <v>0.71819999999999995</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>29</v>
+        <v>130</v>
       </c>
       <c r="B52" t="s">
-        <v>73</v>
-      </c>
-      <c r="C52" t="s">
-        <v>69</v>
-      </c>
-      <c r="D52" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E52" t="s">
         <v>69</v>
       </c>
-      <c r="F52">
-        <v>0.377</v>
-      </c>
-      <c r="G52">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="H52">
-        <v>0.52800000000000002</v>
-      </c>
-      <c r="I52">
-        <v>7.6999999999999999E-2</v>
+      <c r="F52" s="5">
+        <v>0</v>
+      </c>
+      <c r="G52" s="5">
+        <v>1</v>
+      </c>
+      <c r="H52" s="5">
+        <v>0</v>
+      </c>
+      <c r="I52" s="5">
+        <v>0</v>
       </c>
       <c r="J52" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="J52" si="5">SUM(F52:I52)</f>
         <v>1</v>
       </c>
-      <c r="K52">
-        <v>0.87</v>
-      </c>
-      <c r="L52" s="4">
+      <c r="K52" s="5">
+        <v>0</v>
+      </c>
+      <c r="L52" s="5">
         <f>K52*0.95</f>
-        <v>0.82650000000000001</v>
-      </c>
-      <c r="M52" s="4">
+        <v>0</v>
+      </c>
+      <c r="M52" s="5">
         <f>L52*1.05</f>
-        <v>0.86782500000000007</v>
-      </c>
-      <c r="N52">
-        <v>0.93</v>
-      </c>
-      <c r="O52">
-        <f>N52*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P52">
-        <f>MIN(N52*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q52">
-        <v>0.61</v>
-      </c>
-      <c r="R52" s="4">
+        <v>0</v>
+      </c>
+      <c r="N52" s="6">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O52" s="6">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P52" s="6">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q52" s="5">
+        <v>0</v>
+      </c>
+      <c r="R52" s="7">
         <f>Q52*0.95</f>
-        <v>0.57950000000000002</v>
-      </c>
-      <c r="S52" s="4">
+        <v>0</v>
+      </c>
+      <c r="S52" s="7">
         <f>R52*1.05</f>
-        <v>0.60847499999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="B53" t="s">
-        <v>73</v>
-      </c>
-      <c r="C53" t="s">
-        <v>69</v>
-      </c>
-      <c r="D53" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E53" t="s">
         <v>69</v>
       </c>
-      <c r="F53">
-        <v>2.9000000000000001E-2</v>
-      </c>
-      <c r="G53">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="H53">
-        <v>0.92500000000000004</v>
-      </c>
-      <c r="I53">
-        <v>3.9E-2</v>
+      <c r="F53" s="15">
+        <v>0.69</v>
+      </c>
+      <c r="G53" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="H53" s="9">
+        <f>1-F53-G53-I53</f>
+        <v>0.21000000000000008</v>
+      </c>
+      <c r="I53" s="15">
+        <v>0.05</v>
       </c>
       <c r="J53" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K53">
-        <v>0.84000000000000008</v>
-      </c>
-      <c r="L53" s="4">
+      <c r="K53" s="10">
+        <v>0.83</v>
+      </c>
+      <c r="L53" s="10">
         <f>K53*0.95</f>
-        <v>0.79800000000000004</v>
-      </c>
-      <c r="M53" s="4">
-        <f>L53*1.05</f>
-        <v>0.83790000000000009</v>
-      </c>
-      <c r="N53">
-        <v>0.93</v>
-      </c>
-      <c r="O53">
-        <f>N53*0.95</f>
-        <v>0.88349999999999995</v>
-      </c>
-      <c r="P53">
-        <f>MIN(N53*1.05, 0.995)</f>
-        <v>0.97650000000000015</v>
-      </c>
-      <c r="Q53">
-        <v>0.7</v>
-      </c>
-      <c r="R53" s="4">
-        <f>Q53*0.95</f>
-        <v>0.66499999999999992</v>
-      </c>
-      <c r="S53" s="4">
-        <f>R53*1.05</f>
-        <v>0.69824999999999993</v>
+        <v>0.78849999999999998</v>
+      </c>
+      <c r="M53" s="10">
+        <f>K53*1.05</f>
+        <v>0.87149999999999994</v>
+      </c>
+      <c r="N53" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O53" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P53" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q53" s="10">
+        <f>81.7/100</f>
+        <v>0.81700000000000006</v>
+      </c>
+      <c r="R53" s="10">
+        <f>71.8/100</f>
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="S53" s="10">
+        <f>91.6/100</f>
+        <v>0.91599999999999993</v>
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>113</v>
+        <v>28</v>
       </c>
       <c r="B54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C54" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D54" t="s">
         <v>69</v>
@@ -4780,330 +4773,533 @@
       <c r="E54" t="s">
         <v>69</v>
       </c>
-      <c r="F54" s="5">
-        <f>AVERAGE('trash fish table'!F2:F6)</f>
-        <v>0.56830740870546492</v>
-      </c>
-      <c r="G54" s="5">
-        <f>AVERAGE('trash fish table'!G2:G6)</f>
-        <v>0.2240987667741102</v>
-      </c>
-      <c r="H54" s="5">
-        <f>AVERAGE('trash fish table'!I2:I6)</f>
-        <v>9.0773327441505319E-2</v>
-      </c>
-      <c r="I54" s="5">
-        <f>AVERAGE('trash fish table'!H2:H6)</f>
-        <v>0.11682049707891951</v>
+      <c r="F54">
+        <v>0.32400000000000001</v>
+      </c>
+      <c r="G54">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="H54">
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="I54">
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="J54" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K54" s="10">
-        <v>0.87980000000000003</v>
-      </c>
-      <c r="L54" s="10">
-        <v>0.82969999999999999</v>
-      </c>
-      <c r="M54" s="10">
-        <v>0.92209999999999992</v>
-      </c>
-      <c r="N54" s="10">
-        <v>0.95669999999999999</v>
-      </c>
-      <c r="O54" s="10">
-        <v>0.8993000000000001</v>
-      </c>
-      <c r="P54" s="10">
-        <v>0.99199999999999999</v>
-      </c>
-      <c r="Q54" s="10">
-        <f>83.3/100</f>
-        <v>0.83299999999999996</v>
-      </c>
-      <c r="R54" s="10">
-        <f>74.5/100</f>
-        <v>0.745</v>
-      </c>
-      <c r="S54" s="10">
-        <f>92.6/100</f>
-        <v>0.92599999999999993</v>
+      <c r="K54">
+        <v>0.87</v>
+      </c>
+      <c r="L54" s="4">
+        <f>K54*0.95</f>
+        <v>0.82650000000000001</v>
+      </c>
+      <c r="M54" s="4">
+        <f>L54*1.05</f>
+        <v>0.86782500000000007</v>
+      </c>
+      <c r="N54">
+        <v>0.93</v>
+      </c>
+      <c r="O54">
+        <f>N54*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P54">
+        <f>MIN(N54*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q54">
+        <v>0.61</v>
+      </c>
+      <c r="R54" s="4">
+        <f>Q54*0.95</f>
+        <v>0.57950000000000002</v>
+      </c>
+      <c r="S54" s="4">
+        <f>R54*1.05</f>
+        <v>0.60847499999999999</v>
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B55" t="s">
         <v>73</v>
       </c>
       <c r="C55" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D55" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E55" t="s">
         <v>69</v>
       </c>
-      <c r="F55" s="5">
-        <v>0.13</v>
-      </c>
-      <c r="G55" s="5">
-        <v>0.02</v>
-      </c>
-      <c r="H55" s="7">
-        <f>1-SUM(F55:G55,I55)</f>
-        <v>0.83000000000000007</v>
-      </c>
-      <c r="I55" s="5">
-        <v>0.02</v>
+      <c r="F55">
+        <v>0.377</v>
+      </c>
+      <c r="G55">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="H55">
+        <v>0.52800000000000002</v>
+      </c>
+      <c r="I55">
+        <v>7.6999999999999999E-2</v>
       </c>
       <c r="J55" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K55" s="5">
-        <v>0.9</v>
-      </c>
-      <c r="L55" s="10">
-        <f>K55*0.94</f>
-        <v>0.84599999999999997</v>
-      </c>
-      <c r="M55" s="10">
-        <f>L55*1.06</f>
-        <v>0.89676</v>
-      </c>
-      <c r="N55" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O55" s="5">
+      <c r="K55">
+        <v>0.87</v>
+      </c>
+      <c r="L55" s="4">
+        <f>K55*0.95</f>
+        <v>0.82650000000000001</v>
+      </c>
+      <c r="M55" s="4">
+        <f>L55*1.05</f>
+        <v>0.86782500000000007</v>
+      </c>
+      <c r="N55">
+        <v>0.93</v>
+      </c>
+      <c r="O55">
         <f>N55*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P55" s="5">
-        <f>N55*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q55" s="5">
-        <v>0.8</v>
-      </c>
-      <c r="R55" s="10">
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P55">
+        <f>MIN(N55*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
+      </c>
+      <c r="Q55">
+        <v>0.61</v>
+      </c>
+      <c r="R55" s="4">
         <f>Q55*0.95</f>
-        <v>0.76</v>
-      </c>
-      <c r="S55" s="10">
+        <v>0.57950000000000002</v>
+      </c>
+      <c r="S55" s="4">
         <f>R55*1.05</f>
-        <v>0.79800000000000004</v>
+        <v>0.60847499999999999</v>
       </c>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>121</v>
+        <v>30</v>
       </c>
       <c r="B56" t="s">
         <v>73</v>
       </c>
+      <c r="C56" t="s">
+        <v>69</v>
+      </c>
+      <c r="D56" t="s">
+        <v>69</v>
+      </c>
       <c r="E56" t="s">
         <v>69</v>
       </c>
       <c r="F56">
-        <v>0.17299999999999999</v>
-      </c>
-      <c r="G56" s="5">
-        <v>3.7999999999999999E-2</v>
-      </c>
-      <c r="H56" s="9">
-        <f>1-F56-G56-I56</f>
-        <v>0.73299999999999987</v>
-      </c>
-      <c r="I56" s="5">
-        <v>5.6000000000000001E-2</v>
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="G56">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="H56">
+        <v>0.92500000000000004</v>
+      </c>
+      <c r="I56">
+        <v>3.9E-2</v>
       </c>
       <c r="J56" s="9">
         <f t="shared" si="0"/>
-        <v>0.99999999999999989</v>
-      </c>
-      <c r="K56" s="9">
-        <v>0.64900000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="K56">
+        <v>0.84000000000000008</v>
+      </c>
+      <c r="L56" s="4">
+        <f>K56*0.95</f>
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="M56" s="4">
+        <f>L56*1.05</f>
+        <v>0.83790000000000009</v>
       </c>
       <c r="N56">
-        <v>0.96</v>
+        <v>0.93</v>
+      </c>
+      <c r="O56">
+        <f>N56*0.95</f>
+        <v>0.88349999999999995</v>
+      </c>
+      <c r="P56">
+        <f>MIN(N56*1.05, 0.995)</f>
+        <v>0.97650000000000015</v>
       </c>
       <c r="Q56">
-        <v>0.57099999999999995</v>
+        <v>0.7</v>
+      </c>
+      <c r="R56" s="4">
+        <f>Q56*0.95</f>
+        <v>0.66499999999999992</v>
+      </c>
+      <c r="S56" s="4">
+        <f>R56*1.05</f>
+        <v>0.69824999999999993</v>
       </c>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>32</v>
+        <v>113</v>
       </c>
       <c r="B57" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C57" t="s">
         <v>68</v>
       </c>
       <c r="D57" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E57" t="s">
         <v>69</v>
       </c>
       <c r="F57" s="5">
-        <f>766/1000</f>
-        <v>0.76600000000000001</v>
+        <f>AVERAGE('trash fish table'!F2:F6)</f>
+        <v>0.56830740870546492</v>
       </c>
       <c r="G57" s="5">
-        <f>74/1000</f>
-        <v>7.3999999999999996E-2</v>
-      </c>
-      <c r="H57" s="7">
-        <f>1-SUM(F57:G57,I57)</f>
-        <v>0.15300000000000002</v>
+        <f>AVERAGE('trash fish table'!G2:G6)</f>
+        <v>0.2240987667741102</v>
+      </c>
+      <c r="H57" s="5">
+        <f>AVERAGE('trash fish table'!I2:I6)</f>
+        <v>9.0773327441505319E-2</v>
       </c>
       <c r="I57" s="5">
-        <f>7/1000</f>
-        <v>7.0000000000000001E-3</v>
+        <f>AVERAGE('trash fish table'!H2:H6)</f>
+        <v>0.11682049707891951</v>
       </c>
       <c r="J57" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K57" s="5">
-        <v>0.89</v>
+      <c r="K57" s="10">
+        <v>0.87980000000000003</v>
       </c>
       <c r="L57" s="10">
-        <f>K57*0.94</f>
-        <v>0.83660000000000001</v>
+        <v>0.82969999999999999</v>
       </c>
       <c r="M57" s="10">
-        <f>L57*1.06</f>
-        <v>0.88679600000000003</v>
-      </c>
-      <c r="N57" s="5">
-        <v>0.95176181599999998</v>
-      </c>
-      <c r="O57" s="5">
-        <f>N57*0.95</f>
-        <v>0.90417372519999994</v>
-      </c>
-      <c r="P57" s="5">
-        <f>N57*1.05</f>
-        <v>0.99934990680000002</v>
-      </c>
-      <c r="Q57" s="5">
-        <v>0.75</v>
+        <v>0.92209999999999992</v>
+      </c>
+      <c r="N57" s="10">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="O57" s="10">
+        <v>0.8993000000000001</v>
+      </c>
+      <c r="P57" s="10">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="Q57" s="10">
+        <f>83.3/100</f>
+        <v>0.83299999999999996</v>
       </c>
       <c r="R57" s="10">
-        <f>Q57*0.95</f>
-        <v>0.71249999999999991</v>
+        <f>74.5/100</f>
+        <v>0.745</v>
       </c>
       <c r="S57" s="10">
-        <f>R57*1.05</f>
-        <v>0.74812499999999993</v>
+        <f>92.6/100</f>
+        <v>0.92599999999999993</v>
       </c>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B58" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C58" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D58" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E58" t="s">
         <v>69</v>
       </c>
-      <c r="F58">
-        <v>0.48</v>
-      </c>
-      <c r="G58">
-        <v>0.04</v>
-      </c>
-      <c r="H58">
-        <v>0.41</v>
-      </c>
-      <c r="I58">
-        <v>7.0000000000000007E-2</v>
+      <c r="F58" s="5">
+        <v>0.13</v>
+      </c>
+      <c r="G58" s="5">
+        <v>0.02</v>
+      </c>
+      <c r="H58" s="7">
+        <f>1-SUM(F58:G58,I58)</f>
+        <v>0.83000000000000007</v>
+      </c>
+      <c r="I58" s="5">
+        <v>0.02</v>
       </c>
       <c r="J58" s="9">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K58">
+      <c r="K58" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="L58" s="10">
+        <f>K58*0.94</f>
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="M58" s="10">
+        <f>L58*1.06</f>
+        <v>0.89676</v>
+      </c>
+      <c r="N58" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O58" s="5">
+        <f>N58*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P58" s="5">
+        <f>N58*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q58" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="R58" s="10">
+        <f>Q58*0.95</f>
+        <v>0.76</v>
+      </c>
+      <c r="S58" s="10">
+        <f>R58*1.05</f>
+        <v>0.79800000000000004</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>121</v>
+      </c>
+      <c r="B59" t="s">
+        <v>73</v>
+      </c>
+      <c r="E59" t="s">
+        <v>69</v>
+      </c>
+      <c r="F59">
+        <v>0.17299999999999999</v>
+      </c>
+      <c r="G59" s="5">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="H59" s="9">
+        <f>1-F59-G59-I59</f>
+        <v>0.73299999999999987</v>
+      </c>
+      <c r="I59" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="J59" s="9">
+        <f t="shared" si="0"/>
+        <v>0.99999999999999989</v>
+      </c>
+      <c r="K59" s="9">
+        <v>0.64900000000000002</v>
+      </c>
+      <c r="N59">
+        <v>0.96</v>
+      </c>
+      <c r="Q59">
+        <v>0.57099999999999995</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>32</v>
+      </c>
+      <c r="B60" t="s">
+        <v>73</v>
+      </c>
+      <c r="C60" t="s">
+        <v>68</v>
+      </c>
+      <c r="D60" t="s">
+        <v>68</v>
+      </c>
+      <c r="E60" t="s">
+        <v>69</v>
+      </c>
+      <c r="F60" s="5">
+        <f>766/1000</f>
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="G60" s="5">
+        <f>74/1000</f>
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="H60" s="7">
+        <f>1-SUM(F60:G60,I60)</f>
+        <v>0.15300000000000002</v>
+      </c>
+      <c r="I60" s="5">
+        <f>7/1000</f>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="J60" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K60" s="5">
+        <v>0.89</v>
+      </c>
+      <c r="L60" s="10">
+        <f>K60*0.94</f>
+        <v>0.83660000000000001</v>
+      </c>
+      <c r="M60" s="10">
+        <f>L60*1.06</f>
+        <v>0.88679600000000003</v>
+      </c>
+      <c r="N60" s="5">
+        <v>0.95176181599999998</v>
+      </c>
+      <c r="O60" s="5">
+        <f>N60*0.95</f>
+        <v>0.90417372519999994</v>
+      </c>
+      <c r="P60" s="5">
+        <f>N60*1.05</f>
+        <v>0.99934990680000002</v>
+      </c>
+      <c r="Q60" s="5">
+        <v>0.75</v>
+      </c>
+      <c r="R60" s="10">
+        <f>Q60*0.95</f>
+        <v>0.71249999999999991</v>
+      </c>
+      <c r="S60" s="10">
+        <f>R60*1.05</f>
+        <v>0.74812499999999993</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>33</v>
+      </c>
+      <c r="B61" t="s">
+        <v>72</v>
+      </c>
+      <c r="C61" t="s">
+        <v>69</v>
+      </c>
+      <c r="D61" t="s">
+        <v>69</v>
+      </c>
+      <c r="E61" t="s">
+        <v>69</v>
+      </c>
+      <c r="F61">
+        <v>0.48</v>
+      </c>
+      <c r="G61">
+        <v>0.04</v>
+      </c>
+      <c r="H61">
+        <v>0.41</v>
+      </c>
+      <c r="I61">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="J61" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K61">
         <v>0.82000000000000006</v>
       </c>
-      <c r="L58" s="4">
-        <f>K58*0.95</f>
+      <c r="L61" s="4">
+        <f>K61*0.95</f>
         <v>0.77900000000000003</v>
       </c>
-      <c r="M58" s="4">
-        <f>L58*1.05</f>
+      <c r="M61" s="4">
+        <f>L61*1.05</f>
         <v>0.81795000000000007</v>
       </c>
-      <c r="N58">
+      <c r="N61">
         <v>0.93</v>
       </c>
-      <c r="O58">
-        <f>N58*0.95</f>
+      <c r="O61">
+        <f>N61*0.95</f>
         <v>0.88349999999999995</v>
       </c>
-      <c r="P58">
-        <f>MIN(N58*1.05, 0.995)</f>
+      <c r="P61">
+        <f>MIN(N61*1.05, 0.995)</f>
         <v>0.97650000000000015</v>
       </c>
-      <c r="Q58">
+      <c r="Q61">
         <v>0.7</v>
       </c>
-      <c r="R58" s="4">
-        <f>Q58*0.95</f>
+      <c r="R61" s="4">
+        <f>Q61*0.95</f>
         <v>0.66499999999999992</v>
       </c>
-      <c r="S58" s="4">
-        <f>R58*1.05</f>
+      <c r="S61" s="4">
+        <f>R61*1.05</f>
         <v>0.69824999999999993</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S58" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S58">
-      <sortCondition ref="A1:A58"/>
+  <autoFilter ref="A1:S61" xr:uid="{FEB86C80-6855-4296-9746-1E92B0D65FFA}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S61">
+      <sortCondition ref="A1:A61"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="K2:S42">
-    <cfRule type="cellIs" dxfId="5" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K51:S52">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="greaterThan">
+  <conditionalFormatting sqref="K54:S55">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K54:S54">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="K57:S57">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L53:M53">
+  <conditionalFormatting sqref="L56:M56">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O56:P56">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O53:P53">
+  <conditionalFormatting sqref="R56:S56">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R53:S53">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="K52:S52">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5114,7 +5310,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA17DA89-E85F-4597-B94B-473613FC79D7}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
@@ -5581,6 +5777,22 @@
       </c>
       <c r="C48" s="1" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>132</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -5601,6 +5813,8 @@
     <hyperlink ref="C46" r:id="rId9" display="https://www.feedipedia.org/node/46" xr:uid="{5AEB9992-3974-4C33-AF56-94BD939A9DFA}"/>
     <hyperlink ref="C47" r:id="rId10" display="https://www.feedipedia.org/node/750" xr:uid="{FBED61B3-6D1C-4C1F-9A17-05EB5A4A4C2D}"/>
     <hyperlink ref="C48" r:id="rId11" display="https://www.feedipedia.org/node/726" xr:uid="{1002B60E-2DED-4A45-AD21-8B1B21F8BC84}"/>
+    <hyperlink ref="C49" r:id="rId12" display="https://www.feedipedia.org/node/202" xr:uid="{B6FDA1BD-485B-4D31-894B-38C079A0C135}"/>
+    <hyperlink ref="C50" r:id="rId13" display="https://www.feedipedia.org/node/202" xr:uid="{40B925EC-163E-405F-9EF2-19DDD0F8F80E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>